<commit_message>
Fix report-checklist: remove razionale from SI rows (C002), fill F/G/H/I for rows 191/376 (C010)
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#CENTROPOLISPECIALISTICOGIOVANNIPAOLOIXX/GPI_HEALTH_SYSTEM/FSE_SENDER/V.1.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#CENTROPOLISPECIALISTICOGIOVANNIPAOLOIXX/GPI_HEALTH_SYSTEM/FSE_SENDER/V.1.0/report-checklist.xlsx
@@ -2598,11 +2598,7 @@
           <t>APPLICABILITA'</t>
         </is>
       </c>
-      <c r="K9" s="17" t="inlineStr">
-        <is>
-          <t>RAZIONALE DI APPLICABILITA'</t>
-        </is>
-      </c>
+      <c r="K9" s="17" t="n"/>
       <c r="L9" s="17" t="inlineStr">
         <is>
           <t>RAZIONALE DI APPLICABILITA' - ALTRO</t>
@@ -2778,11 +2774,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K11" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K11" s="32" t="n"/>
       <c r="L11" s="32" t="n"/>
       <c r="M11" s="32" t="inlineStr">
         <is>
@@ -2869,11 +2861,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K12" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K12" s="32" t="n"/>
       <c r="L12" s="32" t="n"/>
       <c r="M12" s="32" t="n"/>
       <c r="N12" s="32" t="n"/>
@@ -2928,11 +2916,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K13" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K13" s="32" t="n"/>
       <c r="L13" s="32" t="n"/>
       <c r="M13" s="32" t="n"/>
       <c r="N13" s="32" t="n"/>
@@ -2991,11 +2975,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K14" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K14" s="32" t="n"/>
       <c r="L14" s="32" t="n"/>
       <c r="M14" s="32" t="inlineStr">
         <is>
@@ -3086,11 +3066,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K15" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K15" s="32" t="n"/>
       <c r="L15" s="32" t="n"/>
       <c r="M15" s="32" t="inlineStr">
         <is>
@@ -3177,11 +3153,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K16" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K16" s="32" t="n"/>
       <c r="L16" s="32" t="n"/>
       <c r="M16" s="32" t="n"/>
       <c r="N16" s="32" t="n"/>
@@ -3236,11 +3208,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K17" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K17" s="32" t="n"/>
       <c r="L17" s="32" t="n"/>
       <c r="M17" s="32" t="n"/>
       <c r="N17" s="32" t="n"/>
@@ -3295,11 +3263,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K18" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K18" s="32" t="n"/>
       <c r="L18" s="32" t="n"/>
       <c r="M18" s="32" t="n"/>
       <c r="N18" s="32" t="n"/>
@@ -3358,11 +3322,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K19" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K19" s="32" t="n"/>
       <c r="L19" s="32" t="n"/>
       <c r="M19" s="32" t="inlineStr">
         <is>
@@ -3449,11 +3409,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K20" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K20" s="32" t="n"/>
       <c r="L20" s="32" t="n"/>
       <c r="M20" s="32" t="n"/>
       <c r="N20" s="32" t="n"/>
@@ -3508,11 +3464,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K21" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K21" s="32" t="n"/>
       <c r="L21" s="32" t="n"/>
       <c r="M21" s="32" t="n"/>
       <c r="N21" s="32" t="n"/>
@@ -3571,11 +3523,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K22" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K22" s="32" t="n"/>
       <c r="L22" s="32" t="n"/>
       <c r="M22" s="32" t="inlineStr">
         <is>
@@ -3666,11 +3614,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K23" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K23" s="32" t="n"/>
       <c r="L23" s="32" t="n"/>
       <c r="M23" s="32" t="inlineStr">
         <is>
@@ -3757,11 +3701,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K24" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K24" s="32" t="n"/>
       <c r="L24" s="32" t="n"/>
       <c r="M24" s="32" t="n"/>
       <c r="N24" s="32" t="n"/>
@@ -3816,11 +3756,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K25" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K25" s="32" t="n"/>
       <c r="L25" s="32" t="n"/>
       <c r="M25" s="32" t="n"/>
       <c r="N25" s="32" t="n"/>
@@ -3875,11 +3811,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K26" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K26" s="32" t="n"/>
       <c r="L26" s="32" t="n"/>
       <c r="M26" s="32" t="n"/>
       <c r="N26" s="32" t="n"/>
@@ -3935,11 +3867,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K27" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K27" s="32" t="n"/>
       <c r="L27" s="32" t="n"/>
       <c r="M27" s="32" t="inlineStr">
         <is>
@@ -4027,11 +3955,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K28" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K28" s="32" t="n"/>
       <c r="L28" s="32" t="n"/>
       <c r="M28" s="32" t="n"/>
       <c r="N28" s="32" t="n"/>
@@ -4087,11 +4011,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K29" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K29" s="32" t="n"/>
       <c r="L29" s="32" t="n"/>
       <c r="M29" s="32" t="n"/>
       <c r="N29" s="32" t="n"/>
@@ -4151,11 +4071,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K30" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K30" s="32" t="n"/>
       <c r="L30" s="32" t="n"/>
       <c r="M30" s="32" t="inlineStr">
         <is>
@@ -4247,11 +4163,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K31" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K31" s="32" t="n"/>
       <c r="L31" s="32" t="n"/>
       <c r="M31" s="32" t="inlineStr">
         <is>
@@ -4339,11 +4251,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K32" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K32" s="32" t="n"/>
       <c r="L32" s="32" t="n"/>
       <c r="M32" s="32" t="n"/>
       <c r="N32" s="32" t="n"/>
@@ -4399,11 +4307,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K33" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K33" s="32" t="n"/>
       <c r="L33" s="32" t="n"/>
       <c r="M33" s="32" t="n"/>
       <c r="N33" s="32" t="n"/>
@@ -4459,11 +4363,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K34" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K34" s="32" t="n"/>
       <c r="L34" s="32" t="n"/>
       <c r="M34" s="32" t="n"/>
       <c r="N34" s="32" t="n"/>
@@ -4523,11 +4423,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K35" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K35" s="32" t="n"/>
       <c r="L35" s="32" t="n"/>
       <c r="M35" s="32" t="inlineStr">
         <is>
@@ -4615,11 +4511,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K36" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K36" s="32" t="n"/>
       <c r="L36" s="32" t="n"/>
       <c r="M36" s="32" t="inlineStr">
         <is>
@@ -4707,11 +4599,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K37" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K37" s="32" t="n"/>
       <c r="L37" s="32" t="n"/>
       <c r="M37" s="32" t="inlineStr">
         <is>
@@ -4799,11 +4687,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K38" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K38" s="32" t="n"/>
       <c r="L38" s="32" t="n"/>
       <c r="M38" s="32" t="inlineStr">
         <is>
@@ -4891,11 +4775,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K39" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K39" s="32" t="n"/>
       <c r="L39" s="32" t="n"/>
       <c r="M39" s="32" t="inlineStr">
         <is>
@@ -4983,11 +4863,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K40" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K40" s="32" t="n"/>
       <c r="L40" s="32" t="n"/>
       <c r="M40" s="32" t="inlineStr">
         <is>
@@ -5075,11 +4951,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K41" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K41" s="32" t="n"/>
       <c r="L41" s="32" t="n"/>
       <c r="M41" s="32" t="inlineStr">
         <is>
@@ -5167,11 +5039,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K42" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K42" s="32" t="n"/>
       <c r="L42" s="32" t="n"/>
       <c r="M42" s="32" t="inlineStr">
         <is>
@@ -5255,11 +5123,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K43" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K43" s="32" t="n"/>
       <c r="L43" s="32" t="n"/>
       <c r="M43" s="32" t="n"/>
       <c r="N43" s="32" t="n"/>
@@ -5311,11 +5175,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K44" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K44" s="32" t="n"/>
       <c r="L44" s="32" t="n"/>
       <c r="M44" s="32" t="n"/>
       <c r="N44" s="32" t="n"/>
@@ -5367,11 +5227,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K45" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K45" s="32" t="n"/>
       <c r="L45" s="32" t="n"/>
       <c r="M45" s="32" t="n"/>
       <c r="N45" s="32" t="n"/>
@@ -5423,11 +5279,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K46" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K46" s="32" t="n"/>
       <c r="L46" s="32" t="n"/>
       <c r="M46" s="32" t="n"/>
       <c r="N46" s="32" t="n"/>
@@ -5479,11 +5331,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K47" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K47" s="32" t="n"/>
       <c r="L47" s="32" t="n"/>
       <c r="M47" s="32" t="n"/>
       <c r="N47" s="32" t="n"/>
@@ -5535,11 +5383,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K48" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K48" s="32" t="n"/>
       <c r="L48" s="32" t="n"/>
       <c r="M48" s="32" t="n"/>
       <c r="N48" s="32" t="n"/>
@@ -5591,11 +5435,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K49" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K49" s="32" t="n"/>
       <c r="L49" s="32" t="n"/>
       <c r="M49" s="32" t="n"/>
       <c r="N49" s="32" t="n"/>
@@ -5647,11 +5487,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K50" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K50" s="32" t="n"/>
       <c r="L50" s="32" t="n"/>
       <c r="M50" s="32" t="n"/>
       <c r="N50" s="32" t="n"/>
@@ -5703,11 +5539,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K51" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K51" s="32" t="n"/>
       <c r="L51" s="32" t="n"/>
       <c r="M51" s="32" t="n"/>
       <c r="N51" s="32" t="n"/>
@@ -5759,11 +5591,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K52" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K52" s="32" t="n"/>
       <c r="L52" s="32" t="n"/>
       <c r="M52" s="32" t="n"/>
       <c r="N52" s="32" t="n"/>
@@ -5819,11 +5647,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K53" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K53" s="32" t="n"/>
       <c r="L53" s="32" t="n"/>
       <c r="M53" s="32" t="inlineStr">
         <is>
@@ -5911,11 +5735,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K54" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K54" s="32" t="n"/>
       <c r="L54" s="32" t="n"/>
       <c r="M54" s="32" t="inlineStr">
         <is>
@@ -6003,11 +5823,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K55" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K55" s="32" t="n"/>
       <c r="L55" s="32" t="n"/>
       <c r="M55" s="32" t="inlineStr">
         <is>
@@ -6095,11 +5911,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K56" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K56" s="32" t="n"/>
       <c r="L56" s="32" t="n"/>
       <c r="M56" s="32" t="inlineStr">
         <is>
@@ -6187,11 +5999,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K57" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K57" s="32" t="n"/>
       <c r="L57" s="32" t="n"/>
       <c r="M57" s="32" t="inlineStr">
         <is>
@@ -6279,11 +6087,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K58" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K58" s="32" t="n"/>
       <c r="L58" s="32" t="n"/>
       <c r="M58" s="32" t="inlineStr">
         <is>
@@ -6371,11 +6175,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K59" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K59" s="32" t="n"/>
       <c r="L59" s="32" t="n"/>
       <c r="M59" s="32" t="inlineStr">
         <is>
@@ -6463,11 +6263,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K60" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K60" s="32" t="n"/>
       <c r="L60" s="32" t="n"/>
       <c r="M60" s="32" t="inlineStr">
         <is>
@@ -6555,11 +6351,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K61" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K61" s="32" t="n"/>
       <c r="L61" s="32" t="n"/>
       <c r="M61" s="32" t="inlineStr">
         <is>
@@ -6647,11 +6439,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K62" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K62" s="32" t="n"/>
       <c r="L62" s="32" t="n"/>
       <c r="M62" s="32" t="inlineStr">
         <is>
@@ -6739,11 +6527,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K63" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K63" s="32" t="n"/>
       <c r="L63" s="32" t="n"/>
       <c r="M63" s="32" t="inlineStr">
         <is>
@@ -6831,11 +6615,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K64" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K64" s="32" t="n"/>
       <c r="L64" s="32" t="n"/>
       <c r="M64" s="32" t="inlineStr">
         <is>
@@ -6923,11 +6703,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K65" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K65" s="32" t="n"/>
       <c r="L65" s="32" t="n"/>
       <c r="M65" s="32" t="inlineStr">
         <is>
@@ -7015,11 +6791,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K66" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K66" s="32" t="n"/>
       <c r="L66" s="32" t="n"/>
       <c r="M66" s="32" t="inlineStr">
         <is>
@@ -7107,11 +6879,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K67" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K67" s="32" t="n"/>
       <c r="L67" s="32" t="n"/>
       <c r="M67" s="32" t="inlineStr">
         <is>
@@ -7199,11 +6967,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K68" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K68" s="32" t="n"/>
       <c r="L68" s="32" t="n"/>
       <c r="M68" s="32" t="inlineStr">
         <is>
@@ -7287,11 +7051,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K69" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K69" s="32" t="n"/>
       <c r="L69" s="32" t="n"/>
       <c r="M69" s="32" t="n"/>
       <c r="N69" s="32" t="n"/>
@@ -7343,11 +7103,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K70" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K70" s="32" t="n"/>
       <c r="L70" s="32" t="n"/>
       <c r="M70" s="32" t="n"/>
       <c r="N70" s="32" t="n"/>
@@ -7399,11 +7155,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K71" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K71" s="32" t="n"/>
       <c r="L71" s="32" t="n"/>
       <c r="M71" s="32" t="n"/>
       <c r="N71" s="32" t="n"/>
@@ -7455,11 +7207,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K72" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K72" s="32" t="n"/>
       <c r="L72" s="32" t="n"/>
       <c r="M72" s="32" t="n"/>
       <c r="N72" s="32" t="n"/>
@@ -7511,11 +7259,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K73" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K73" s="32" t="n"/>
       <c r="L73" s="32" t="n"/>
       <c r="M73" s="32" t="n"/>
       <c r="N73" s="32" t="n"/>
@@ -7567,11 +7311,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K74" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K74" s="32" t="n"/>
       <c r="L74" s="32" t="n"/>
       <c r="M74" s="32" t="n"/>
       <c r="N74" s="32" t="n"/>
@@ -7623,11 +7363,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K75" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K75" s="32" t="n"/>
       <c r="L75" s="32" t="n"/>
       <c r="M75" s="32" t="n"/>
       <c r="N75" s="32" t="n"/>
@@ -7679,11 +7415,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K76" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K76" s="32" t="n"/>
       <c r="L76" s="32" t="n"/>
       <c r="M76" s="32" t="n"/>
       <c r="N76" s="32" t="n"/>
@@ -7735,11 +7467,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K77" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K77" s="32" t="n"/>
       <c r="L77" s="32" t="n"/>
       <c r="M77" s="32" t="n"/>
       <c r="N77" s="32" t="n"/>
@@ -7791,11 +7519,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K78" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K78" s="32" t="n"/>
       <c r="L78" s="32" t="n"/>
       <c r="M78" s="32" t="n"/>
       <c r="N78" s="32" t="n"/>
@@ -7847,11 +7571,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K79" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K79" s="32" t="n"/>
       <c r="L79" s="32" t="n"/>
       <c r="M79" s="32" t="n"/>
       <c r="N79" s="32" t="n"/>
@@ -7903,11 +7623,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K80" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K80" s="32" t="n"/>
       <c r="L80" s="32" t="n"/>
       <c r="M80" s="32" t="n"/>
       <c r="N80" s="32" t="n"/>
@@ -7959,11 +7675,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K81" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K81" s="32" t="n"/>
       <c r="L81" s="32" t="n"/>
       <c r="M81" s="32" t="n"/>
       <c r="N81" s="32" t="n"/>
@@ -8015,11 +7727,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K82" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K82" s="32" t="n"/>
       <c r="L82" s="32" t="n"/>
       <c r="M82" s="32" t="n"/>
       <c r="N82" s="32" t="n"/>
@@ -8071,11 +7779,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K83" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K83" s="32" t="n"/>
       <c r="L83" s="32" t="n"/>
       <c r="M83" s="32" t="n"/>
       <c r="N83" s="32" t="n"/>
@@ -8127,11 +7831,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K84" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K84" s="32" t="n"/>
       <c r="L84" s="32" t="n"/>
       <c r="M84" s="32" t="n"/>
       <c r="N84" s="32" t="n"/>
@@ -8183,11 +7883,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K85" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K85" s="32" t="n"/>
       <c r="L85" s="32" t="n"/>
       <c r="M85" s="32" t="n"/>
       <c r="N85" s="32" t="n"/>
@@ -8239,11 +7935,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K86" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K86" s="32" t="n"/>
       <c r="L86" s="32" t="n"/>
       <c r="M86" s="32" t="n"/>
       <c r="N86" s="32" t="n"/>
@@ -8295,11 +7987,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K87" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K87" s="32" t="n"/>
       <c r="L87" s="32" t="n"/>
       <c r="M87" s="32" t="n"/>
       <c r="N87" s="32" t="n"/>
@@ -8351,11 +8039,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K88" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K88" s="32" t="n"/>
       <c r="L88" s="32" t="n"/>
       <c r="M88" s="32" t="n"/>
       <c r="N88" s="32" t="n"/>
@@ -8407,11 +8091,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K89" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K89" s="32" t="n"/>
       <c r="L89" s="32" t="n"/>
       <c r="M89" s="32" t="n"/>
       <c r="N89" s="32" t="n"/>
@@ -8463,11 +8143,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K90" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K90" s="32" t="n"/>
       <c r="L90" s="32" t="n"/>
       <c r="M90" s="32" t="n"/>
       <c r="N90" s="32" t="n"/>
@@ -8519,11 +8195,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K91" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K91" s="32" t="n"/>
       <c r="L91" s="32" t="n"/>
       <c r="M91" s="32" t="n"/>
       <c r="N91" s="32" t="n"/>
@@ -8575,11 +8247,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K92" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K92" s="32" t="n"/>
       <c r="L92" s="32" t="n"/>
       <c r="M92" s="32" t="n"/>
       <c r="N92" s="32" t="n"/>
@@ -8631,11 +8299,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K93" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K93" s="32" t="n"/>
       <c r="L93" s="32" t="n"/>
       <c r="M93" s="32" t="n"/>
       <c r="N93" s="32" t="n"/>
@@ -8687,11 +8351,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K94" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K94" s="32" t="n"/>
       <c r="L94" s="32" t="n"/>
       <c r="M94" s="32" t="n"/>
       <c r="N94" s="32" t="n"/>
@@ -8743,11 +8403,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K95" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K95" s="32" t="n"/>
       <c r="L95" s="32" t="n"/>
       <c r="M95" s="32" t="n"/>
       <c r="N95" s="32" t="n"/>
@@ -8799,11 +8455,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K96" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K96" s="32" t="n"/>
       <c r="L96" s="32" t="n"/>
       <c r="M96" s="32" t="n"/>
       <c r="N96" s="32" t="n"/>
@@ -8855,11 +8507,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K97" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K97" s="32" t="n"/>
       <c r="L97" s="32" t="n"/>
       <c r="M97" s="32" t="n"/>
       <c r="N97" s="32" t="n"/>
@@ -8911,11 +8559,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K98" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K98" s="32" t="n"/>
       <c r="L98" s="32" t="n"/>
       <c r="M98" s="32" t="n"/>
       <c r="N98" s="32" t="n"/>
@@ -8967,11 +8611,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K99" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K99" s="32" t="n"/>
       <c r="L99" s="32" t="n"/>
       <c r="M99" s="32" t="n"/>
       <c r="N99" s="32" t="n"/>
@@ -9023,11 +8663,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K100" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K100" s="32" t="n"/>
       <c r="L100" s="32" t="n"/>
       <c r="M100" s="32" t="n"/>
       <c r="N100" s="32" t="n"/>
@@ -9079,11 +8715,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K101" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K101" s="32" t="n"/>
       <c r="L101" s="32" t="n"/>
       <c r="M101" s="32" t="n"/>
       <c r="N101" s="32" t="n"/>
@@ -9135,11 +8767,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K102" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K102" s="32" t="n"/>
       <c r="L102" s="32" t="n"/>
       <c r="M102" s="32" t="n"/>
       <c r="N102" s="32" t="n"/>
@@ -9191,11 +8819,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K103" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K103" s="32" t="n"/>
       <c r="L103" s="32" t="n"/>
       <c r="M103" s="32" t="n"/>
       <c r="N103" s="32" t="n"/>
@@ -9247,11 +8871,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K104" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K104" s="32" t="n"/>
       <c r="L104" s="32" t="n"/>
       <c r="M104" s="32" t="n"/>
       <c r="N104" s="32" t="n"/>
@@ -9303,11 +8923,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K105" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K105" s="32" t="n"/>
       <c r="L105" s="32" t="n"/>
       <c r="M105" s="32" t="n"/>
       <c r="N105" s="32" t="n"/>
@@ -9359,11 +8975,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K106" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K106" s="32" t="n"/>
       <c r="L106" s="32" t="n"/>
       <c r="M106" s="32" t="n"/>
       <c r="N106" s="32" t="n"/>
@@ -9415,11 +9027,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K107" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K107" s="32" t="n"/>
       <c r="L107" s="32" t="n"/>
       <c r="M107" s="32" t="n"/>
       <c r="N107" s="32" t="n"/>
@@ -9471,11 +9079,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K108" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K108" s="32" t="n"/>
       <c r="L108" s="32" t="n"/>
       <c r="M108" s="32" t="n"/>
       <c r="N108" s="32" t="n"/>
@@ -9527,11 +9131,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K109" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K109" s="32" t="n"/>
       <c r="L109" s="32" t="n"/>
       <c r="M109" s="32" t="n"/>
       <c r="N109" s="32" t="n"/>
@@ -9583,11 +9183,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K110" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K110" s="32" t="n"/>
       <c r="L110" s="32" t="n"/>
       <c r="M110" s="32" t="n"/>
       <c r="N110" s="32" t="n"/>
@@ -9639,11 +9235,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K111" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K111" s="32" t="n"/>
       <c r="L111" s="32" t="n"/>
       <c r="M111" s="32" t="n"/>
       <c r="N111" s="32" t="n"/>
@@ -9695,11 +9287,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K112" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K112" s="32" t="n"/>
       <c r="L112" s="32" t="n"/>
       <c r="M112" s="32" t="n"/>
       <c r="N112" s="32" t="n"/>
@@ -9751,11 +9339,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K113" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K113" s="32" t="n"/>
       <c r="L113" s="32" t="n"/>
       <c r="M113" s="32" t="n"/>
       <c r="N113" s="32" t="n"/>
@@ -9807,11 +9391,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K114" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K114" s="32" t="n"/>
       <c r="L114" s="32" t="n"/>
       <c r="M114" s="32" t="n"/>
       <c r="N114" s="32" t="n"/>
@@ -9863,11 +9443,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K115" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K115" s="32" t="n"/>
       <c r="L115" s="32" t="n"/>
       <c r="M115" s="32" t="n"/>
       <c r="N115" s="32" t="n"/>
@@ -9923,11 +9499,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K116" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K116" s="32" t="n"/>
       <c r="L116" s="32" t="n"/>
       <c r="M116" s="32" t="inlineStr">
         <is>
@@ -10015,11 +9587,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K117" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K117" s="32" t="n"/>
       <c r="L117" s="32" t="n"/>
       <c r="M117" s="32" t="inlineStr">
         <is>
@@ -10107,11 +9675,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K118" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K118" s="32" t="n"/>
       <c r="L118" s="32" t="n"/>
       <c r="M118" s="32" t="inlineStr">
         <is>
@@ -10199,11 +9763,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K119" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K119" s="32" t="n"/>
       <c r="L119" s="32" t="n"/>
       <c r="M119" s="32" t="inlineStr">
         <is>
@@ -10291,11 +9851,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K120" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K120" s="32" t="n"/>
       <c r="L120" s="32" t="n"/>
       <c r="M120" s="32" t="inlineStr">
         <is>
@@ -10383,11 +9939,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K121" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K121" s="32" t="n"/>
       <c r="L121" s="32" t="n"/>
       <c r="M121" s="32" t="inlineStr">
         <is>
@@ -10475,11 +10027,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K122" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K122" s="32" t="n"/>
       <c r="L122" s="32" t="n"/>
       <c r="M122" s="32" t="inlineStr">
         <is>
@@ -10567,11 +10115,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K123" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K123" s="32" t="n"/>
       <c r="L123" s="32" t="n"/>
       <c r="M123" s="32" t="inlineStr">
         <is>
@@ -10659,11 +10203,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K124" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K124" s="32" t="n"/>
       <c r="L124" s="32" t="n"/>
       <c r="M124" s="32" t="inlineStr">
         <is>
@@ -10751,11 +10291,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K125" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K125" s="32" t="n"/>
       <c r="L125" s="32" t="n"/>
       <c r="M125" s="32" t="inlineStr">
         <is>
@@ -10843,11 +10379,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K126" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K126" s="32" t="n"/>
       <c r="L126" s="32" t="n"/>
       <c r="M126" s="32" t="inlineStr">
         <is>
@@ -10935,11 +10467,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K127" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K127" s="32" t="n"/>
       <c r="L127" s="32" t="n"/>
       <c r="M127" s="32" t="inlineStr">
         <is>
@@ -11027,11 +10555,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K128" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K128" s="32" t="n"/>
       <c r="L128" s="32" t="n"/>
       <c r="M128" s="32" t="inlineStr">
         <is>
@@ -11119,11 +10643,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K129" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K129" s="32" t="n"/>
       <c r="L129" s="32" t="n"/>
       <c r="M129" s="32" t="inlineStr">
         <is>
@@ -11211,11 +10731,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K130" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K130" s="32" t="n"/>
       <c r="L130" s="32" t="n"/>
       <c r="M130" s="32" t="inlineStr">
         <is>
@@ -11299,11 +10815,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K131" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K131" s="32" t="n"/>
       <c r="L131" s="32" t="n"/>
       <c r="M131" s="32" t="n"/>
       <c r="N131" s="32" t="n"/>
@@ -11355,11 +10867,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K132" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K132" s="32" t="n"/>
       <c r="L132" s="32" t="n"/>
       <c r="M132" s="32" t="n"/>
       <c r="N132" s="32" t="n"/>
@@ -11411,11 +10919,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K133" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K133" s="32" t="n"/>
       <c r="L133" s="32" t="n"/>
       <c r="M133" s="32" t="n"/>
       <c r="N133" s="32" t="n"/>
@@ -11467,11 +10971,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K134" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K134" s="32" t="n"/>
       <c r="L134" s="32" t="n"/>
       <c r="M134" s="32" t="n"/>
       <c r="N134" s="32" t="n"/>
@@ -11523,11 +11023,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K135" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K135" s="32" t="n"/>
       <c r="L135" s="32" t="n"/>
       <c r="M135" s="32" t="n"/>
       <c r="N135" s="32" t="n"/>
@@ -11579,11 +11075,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K136" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K136" s="32" t="n"/>
       <c r="L136" s="32" t="n"/>
       <c r="M136" s="32" t="n"/>
       <c r="N136" s="32" t="n"/>
@@ -11635,11 +11127,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K137" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K137" s="32" t="n"/>
       <c r="L137" s="32" t="n"/>
       <c r="M137" s="32" t="n"/>
       <c r="N137" s="32" t="n"/>
@@ -11691,11 +11179,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K138" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K138" s="32" t="n"/>
       <c r="L138" s="32" t="n"/>
       <c r="M138" s="32" t="n"/>
       <c r="N138" s="32" t="n"/>
@@ -11747,11 +11231,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K139" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K139" s="32" t="n"/>
       <c r="L139" s="32" t="n"/>
       <c r="M139" s="32" t="n"/>
       <c r="N139" s="32" t="n"/>
@@ -11803,11 +11283,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K140" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K140" s="32" t="n"/>
       <c r="L140" s="32" t="n"/>
       <c r="M140" s="32" t="n"/>
       <c r="N140" s="32" t="n"/>
@@ -11859,11 +11335,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K141" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K141" s="32" t="n"/>
       <c r="L141" s="32" t="n"/>
       <c r="M141" s="32" t="n"/>
       <c r="N141" s="32" t="n"/>
@@ -11915,11 +11387,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K142" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K142" s="32" t="n"/>
       <c r="L142" s="32" t="n"/>
       <c r="M142" s="32" t="n"/>
       <c r="N142" s="32" t="n"/>
@@ -11971,11 +11439,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K143" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K143" s="32" t="n"/>
       <c r="L143" s="32" t="n"/>
       <c r="M143" s="32" t="n"/>
       <c r="N143" s="32" t="n"/>
@@ -12027,11 +11491,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K144" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K144" s="32" t="n"/>
       <c r="L144" s="32" t="n"/>
       <c r="M144" s="32" t="n"/>
       <c r="N144" s="32" t="n"/>
@@ -12083,11 +11543,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K145" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K145" s="32" t="n"/>
       <c r="L145" s="32" t="n"/>
       <c r="M145" s="32" t="n"/>
       <c r="N145" s="32" t="n"/>
@@ -12261,11 +11717,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K148" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K148" s="32" t="n"/>
       <c r="L148" s="32" t="n"/>
       <c r="M148" s="32" t="n"/>
       <c r="N148" s="32" t="n"/>
@@ -12318,11 +11770,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K149" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K149" s="32" t="n"/>
       <c r="L149" s="32" t="n"/>
       <c r="M149" s="32" t="n"/>
       <c r="N149" s="32" t="n"/>
@@ -12375,11 +11823,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K150" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K150" s="32" t="n"/>
       <c r="L150" s="32" t="n"/>
       <c r="M150" s="32" t="n"/>
       <c r="N150" s="32" t="n"/>
@@ -12434,11 +11878,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K151" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K151" s="32" t="n"/>
       <c r="L151" s="32" t="n"/>
       <c r="M151" s="32" t="n"/>
       <c r="N151" s="32" t="n"/>
@@ -12493,11 +11933,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K152" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K152" s="32" t="n"/>
       <c r="L152" s="32" t="n"/>
       <c r="M152" s="32" t="n"/>
       <c r="N152" s="32" t="n"/>
@@ -12549,11 +11985,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K153" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K153" s="32" t="n"/>
       <c r="L153" s="32" t="n"/>
       <c r="M153" s="32" t="n"/>
       <c r="N153" s="32" t="n"/>
@@ -12609,11 +12041,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K154" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K154" s="32" t="n"/>
       <c r="L154" s="32" t="n"/>
       <c r="M154" s="32" t="n"/>
       <c r="N154" s="32" t="n"/>
@@ -12665,11 +12093,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K155" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K155" s="32" t="n"/>
       <c r="L155" s="32" t="n"/>
       <c r="M155" s="32" t="n"/>
       <c r="N155" s="32" t="n"/>
@@ -12721,11 +12145,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K156" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K156" s="32" t="n"/>
       <c r="L156" s="32" t="n"/>
       <c r="M156" s="32" t="n"/>
       <c r="N156" s="32" t="n"/>
@@ -12777,11 +12197,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K157" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K157" s="32" t="n"/>
       <c r="L157" s="32" t="n"/>
       <c r="M157" s="32" t="n"/>
       <c r="N157" s="32" t="n"/>
@@ -12833,11 +12249,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K158" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K158" s="32" t="n"/>
       <c r="L158" s="32" t="n"/>
       <c r="M158" s="32" t="n"/>
       <c r="N158" s="32" t="n"/>
@@ -12889,11 +12301,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K159" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K159" s="32" t="n"/>
       <c r="L159" s="32" t="n"/>
       <c r="M159" s="32" t="n"/>
       <c r="N159" s="32" t="n"/>
@@ -12945,11 +12353,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K160" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K160" s="32" t="n"/>
       <c r="L160" s="32" t="n"/>
       <c r="M160" s="32" t="n"/>
       <c r="N160" s="32" t="n"/>
@@ -13001,11 +12405,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K161" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K161" s="32" t="n"/>
       <c r="L161" s="32" t="n"/>
       <c r="M161" s="32" t="n"/>
       <c r="N161" s="32" t="n"/>
@@ -13057,11 +12457,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K162" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K162" s="32" t="n"/>
       <c r="L162" s="32" t="n"/>
       <c r="M162" s="32" t="n"/>
       <c r="N162" s="32" t="n"/>
@@ -13113,11 +12509,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K163" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K163" s="32" t="n"/>
       <c r="L163" s="32" t="n"/>
       <c r="M163" s="32" t="n"/>
       <c r="N163" s="32" t="n"/>
@@ -13313,11 +12705,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K166" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K166" s="32" t="n"/>
       <c r="L166" s="32" t="n"/>
       <c r="M166" s="32" t="n"/>
       <c r="N166" s="32" t="n"/>
@@ -13369,11 +12757,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K167" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K167" s="32" t="n"/>
       <c r="L167" s="32" t="n"/>
       <c r="M167" s="32" t="n"/>
       <c r="N167" s="32" t="n"/>
@@ -13498,11 +12882,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K169" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K169" s="32" t="n"/>
       <c r="L169" s="32" t="n"/>
       <c r="M169" s="32" t="n"/>
       <c r="N169" s="32" t="n"/>
@@ -13554,11 +12934,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K170" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K170" s="32" t="n"/>
       <c r="L170" s="32" t="n"/>
       <c r="M170" s="32" t="n"/>
       <c r="N170" s="32" t="n"/>
@@ -13610,11 +12986,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K171" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K171" s="32" t="n"/>
       <c r="L171" s="32" t="n"/>
       <c r="M171" s="32" t="n"/>
       <c r="N171" s="32" t="n"/>
@@ -13666,11 +13038,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K172" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K172" s="32" t="n"/>
       <c r="L172" s="32" t="n"/>
       <c r="M172" s="32" t="n"/>
       <c r="N172" s="32" t="n"/>
@@ -13722,11 +13090,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K173" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K173" s="32" t="n"/>
       <c r="L173" s="32" t="n"/>
       <c r="M173" s="32" t="n"/>
       <c r="N173" s="32" t="n"/>
@@ -13778,11 +13142,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K174" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K174" s="32" t="n"/>
       <c r="L174" s="32" t="n"/>
       <c r="M174" s="32" t="n"/>
       <c r="N174" s="32" t="n"/>
@@ -13834,11 +13194,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K175" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K175" s="32" t="n"/>
       <c r="L175" s="32" t="n"/>
       <c r="M175" s="32" t="n"/>
       <c r="N175" s="32" t="n"/>
@@ -13894,11 +13250,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K176" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K176" s="32" t="n"/>
       <c r="L176" s="29" t="n"/>
       <c r="M176" s="32" t="inlineStr">
         <is>
@@ -13986,11 +13338,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K177" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K177" s="32" t="n"/>
       <c r="L177" s="29" t="n"/>
       <c r="M177" s="32" t="inlineStr">
         <is>
@@ -14074,11 +13422,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K178" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K178" s="32" t="n"/>
       <c r="L178" s="29" t="n"/>
       <c r="M178" s="32" t="n"/>
       <c r="N178" s="32" t="n"/>
@@ -14130,11 +13474,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K179" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K179" s="32" t="n"/>
       <c r="L179" s="29" t="n"/>
       <c r="M179" s="32" t="n"/>
       <c r="N179" s="32" t="n"/>
@@ -14186,11 +13526,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K180" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K180" s="32" t="n"/>
       <c r="L180" s="29" t="n"/>
       <c r="M180" s="32" t="n"/>
       <c r="N180" s="32" t="n"/>
@@ -14246,11 +13582,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K181" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K181" s="32" t="n"/>
       <c r="L181" s="29" t="n"/>
       <c r="M181" s="32" t="inlineStr">
         <is>
@@ -14334,11 +13666,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K182" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K182" s="32" t="n"/>
       <c r="L182" s="29" t="n"/>
       <c r="M182" s="32" t="n"/>
       <c r="N182" s="32" t="n"/>
@@ -14394,11 +13722,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K183" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K183" s="32" t="n"/>
       <c r="L183" s="29" t="n"/>
       <c r="M183" s="32" t="inlineStr">
         <is>
@@ -14482,11 +13806,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K184" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K184" s="32" t="n"/>
       <c r="L184" s="29" t="n"/>
       <c r="M184" s="32" t="n"/>
       <c r="N184" s="32" t="n"/>
@@ -14538,11 +13858,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K185" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K185" s="32" t="n"/>
       <c r="L185" s="29" t="n"/>
       <c r="M185" s="32" t="n"/>
       <c r="N185" s="32" t="n"/>
@@ -14742,11 +14058,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K188" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K188" s="32" t="n"/>
       <c r="L188" s="32" t="n"/>
       <c r="M188" s="32" t="inlineStr">
         <is>
@@ -14834,11 +14146,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K189" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K189" s="32" t="n"/>
       <c r="L189" s="32" t="n"/>
       <c r="M189" s="32" t="inlineStr">
         <is>
@@ -14926,11 +14234,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="K190" s="32" t="inlineStr">
-        <is>
-          <t>L'applicativo effettua controlli preventivi sul dato inserito</t>
-        </is>
-      </c>
+      <c r="K190" s="32" t="n"/>
       <c r="L190" s="32" t="n"/>
       <c r="M190" s="32" t="inlineStr">
         <is>
@@ -15006,20 +14310,32 @@
 </t>
         </is>
       </c>
-      <c r="F191" s="31" t="n"/>
-      <c r="G191" s="31" t="n"/>
-      <c r="H191" s="31" t="n"/>
-      <c r="I191" s="36" t="n"/>
+      <c r="F191" s="31" t="inlineStr">
+        <is>
+          <t>25/03/2026</t>
+        </is>
+      </c>
+      <c r="G191" s="31" t="inlineStr">
+        <is>
+          <t>346c86394d9e19688c98e1eac3507b73</t>
+        </is>
+      </c>
+      <c r="H191" s="31" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.2081e93bc59b43e49e3aeae958e60c84dccb7d9ecdcb4e330174098f046ce5f1.617e1f2a25^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
+      <c r="I191" s="36" t="inlineStr">
+        <is>
+          <t>LAB_VALIDATION.pdf</t>
+        </is>
+      </c>
       <c r="J191" s="32" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="K191" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K191" s="32" t="n"/>
       <c r="L191" s="32" t="n"/>
       <c r="M191" s="32" t="n"/>
       <c r="N191" s="32" t="n"/>
@@ -15072,11 +14388,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K192" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K192" s="32" t="n"/>
       <c r="L192" s="32" t="n"/>
       <c r="M192" s="32" t="n"/>
       <c r="N192" s="32" t="n"/>
@@ -15128,11 +14440,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K193" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K193" s="32" t="n"/>
       <c r="L193" s="32" t="n"/>
       <c r="M193" s="32" t="n"/>
       <c r="N193" s="32" t="n"/>
@@ -15184,11 +14492,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K194" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K194" s="32" t="n"/>
       <c r="L194" s="32" t="n"/>
       <c r="M194" s="32" t="n"/>
       <c r="N194" s="32" t="n"/>
@@ -15240,11 +14544,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K195" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K195" s="32" t="n"/>
       <c r="L195" s="32" t="n"/>
       <c r="M195" s="32" t="n"/>
       <c r="N195" s="32" t="n"/>
@@ -15296,11 +14596,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K196" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K196" s="32" t="n"/>
       <c r="L196" s="32" t="n"/>
       <c r="M196" s="32" t="n"/>
       <c r="N196" s="32" t="n"/>
@@ -15352,11 +14648,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K197" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K197" s="32" t="n"/>
       <c r="L197" s="32" t="n"/>
       <c r="M197" s="32" t="n"/>
       <c r="N197" s="32" t="n"/>
@@ -15408,11 +14700,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K198" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K198" s="32" t="n"/>
       <c r="L198" s="32" t="n"/>
       <c r="M198" s="32" t="n"/>
       <c r="N198" s="32" t="n"/>
@@ -15464,11 +14752,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K199" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K199" s="32" t="n"/>
       <c r="L199" s="32" t="n"/>
       <c r="M199" s="32" t="n"/>
       <c r="N199" s="32" t="n"/>
@@ -15520,11 +14804,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K200" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K200" s="32" t="n"/>
       <c r="L200" s="32" t="n"/>
       <c r="M200" s="32" t="n"/>
       <c r="N200" s="32" t="n"/>
@@ -15576,11 +14856,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K201" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K201" s="32" t="n"/>
       <c r="L201" s="32" t="n"/>
       <c r="M201" s="32" t="n"/>
       <c r="N201" s="32" t="n"/>
@@ -15632,11 +14908,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K202" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K202" s="32" t="n"/>
       <c r="L202" s="32" t="n"/>
       <c r="M202" s="32" t="n"/>
       <c r="N202" s="32" t="n"/>
@@ -15688,11 +14960,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K203" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K203" s="32" t="n"/>
       <c r="L203" s="32" t="n"/>
       <c r="M203" s="32" t="n"/>
       <c r="N203" s="32" t="n"/>
@@ -15747,11 +15015,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K204" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K204" s="32" t="n"/>
       <c r="L204" s="32" t="n"/>
       <c r="M204" s="32" t="n"/>
       <c r="N204" s="32" t="n"/>
@@ -15803,11 +15067,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K205" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K205" s="32" t="n"/>
       <c r="L205" s="32" t="n"/>
       <c r="M205" s="32" t="n"/>
       <c r="N205" s="32" t="n"/>
@@ -15863,11 +15123,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K206" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K206" s="32" t="n"/>
       <c r="L206" s="32" t="n"/>
       <c r="M206" s="32" t="n"/>
       <c r="N206" s="32" t="n"/>
@@ -15919,11 +15175,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K207" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K207" s="32" t="n"/>
       <c r="L207" s="32" t="n"/>
       <c r="M207" s="32" t="n"/>
       <c r="N207" s="32" t="n"/>
@@ -15975,11 +15227,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K208" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K208" s="32" t="n"/>
       <c r="L208" s="32" t="n"/>
       <c r="M208" s="32" t="n"/>
       <c r="N208" s="32" t="n"/>
@@ -16031,11 +15279,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K209" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K209" s="32" t="n"/>
       <c r="L209" s="32" t="n"/>
       <c r="M209" s="32" t="n"/>
       <c r="N209" s="32" t="n"/>
@@ -16087,11 +15331,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K210" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K210" s="32" t="n"/>
       <c r="L210" s="32" t="n"/>
       <c r="M210" s="32" t="n"/>
       <c r="N210" s="32" t="n"/>
@@ -16143,11 +15383,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K211" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K211" s="32" t="n"/>
       <c r="L211" s="32" t="n"/>
       <c r="M211" s="32" t="n"/>
       <c r="N211" s="32" t="n"/>
@@ -16199,11 +15435,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K212" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K212" s="32" t="n"/>
       <c r="L212" s="32" t="n"/>
       <c r="M212" s="32" t="n"/>
       <c r="N212" s="32" t="n"/>
@@ -16255,11 +15487,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K213" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K213" s="32" t="n"/>
       <c r="L213" s="32" t="n"/>
       <c r="M213" s="32" t="n"/>
       <c r="N213" s="32" t="n"/>
@@ -16311,11 +15539,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K214" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K214" s="32" t="n"/>
       <c r="L214" s="32" t="n"/>
       <c r="M214" s="32" t="n"/>
       <c r="N214" s="32" t="n"/>
@@ -16367,11 +15591,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K215" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K215" s="32" t="n"/>
       <c r="L215" s="32" t="n"/>
       <c r="M215" s="32" t="n"/>
       <c r="N215" s="32" t="n"/>
@@ -16423,11 +15643,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K216" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K216" s="32" t="n"/>
       <c r="L216" s="32" t="n"/>
       <c r="M216" s="32" t="n"/>
       <c r="N216" s="32" t="n"/>
@@ -16479,11 +15695,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K217" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K217" s="32" t="n"/>
       <c r="L217" s="32" t="n"/>
       <c r="M217" s="32" t="n"/>
       <c r="N217" s="32" t="n"/>
@@ -16535,11 +15747,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K218" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K218" s="32" t="n"/>
       <c r="L218" s="32" t="n"/>
       <c r="M218" s="32" t="n"/>
       <c r="N218" s="32" t="n"/>
@@ -16594,11 +15802,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K219" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K219" s="32" t="n"/>
       <c r="L219" s="32" t="n"/>
       <c r="M219" s="32" t="n"/>
       <c r="N219" s="32" t="n"/>
@@ -16650,11 +15854,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K220" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K220" s="32" t="n"/>
       <c r="L220" s="32" t="n"/>
       <c r="M220" s="32" t="n"/>
       <c r="N220" s="32" t="n"/>
@@ -16710,11 +15910,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K221" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K221" s="32" t="n"/>
       <c r="L221" s="32" t="n"/>
       <c r="M221" s="32" t="n"/>
       <c r="N221" s="32" t="n"/>
@@ -16766,11 +15962,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K222" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K222" s="32" t="n"/>
       <c r="L222" s="32" t="n"/>
       <c r="M222" s="32" t="n"/>
       <c r="N222" s="32" t="n"/>
@@ -16822,11 +16014,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K223" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K223" s="32" t="n"/>
       <c r="L223" s="32" t="n"/>
       <c r="M223" s="32" t="n"/>
       <c r="N223" s="32" t="n"/>
@@ -16878,11 +16066,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K224" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K224" s="32" t="n"/>
       <c r="L224" s="32" t="n"/>
       <c r="M224" s="32" t="n"/>
       <c r="N224" s="32" t="n"/>
@@ -16934,11 +16118,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K225" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K225" s="32" t="n"/>
       <c r="L225" s="32" t="n"/>
       <c r="M225" s="32" t="n"/>
       <c r="N225" s="32" t="n"/>
@@ -16990,11 +16170,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K226" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K226" s="32" t="n"/>
       <c r="L226" s="32" t="n"/>
       <c r="M226" s="32" t="n"/>
       <c r="N226" s="32" t="n"/>
@@ -17046,11 +16222,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K227" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K227" s="32" t="n"/>
       <c r="L227" s="32" t="n"/>
       <c r="M227" s="32" t="n"/>
       <c r="N227" s="32" t="n"/>
@@ -17102,11 +16274,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K228" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K228" s="32" t="n"/>
       <c r="L228" s="32" t="n"/>
       <c r="M228" s="32" t="n"/>
       <c r="N228" s="32" t="n"/>
@@ -17158,11 +16326,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K229" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K229" s="32" t="n"/>
       <c r="L229" s="32" t="n"/>
       <c r="M229" s="32" t="n"/>
       <c r="N229" s="32" t="n"/>
@@ -17214,11 +16378,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K230" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K230" s="32" t="n"/>
       <c r="L230" s="32" t="n"/>
       <c r="M230" s="32" t="n"/>
       <c r="N230" s="32" t="n"/>
@@ -17270,11 +16430,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K231" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K231" s="32" t="n"/>
       <c r="L231" s="32" t="n"/>
       <c r="M231" s="32" t="n"/>
       <c r="N231" s="32" t="n"/>
@@ -17326,11 +16482,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K232" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K232" s="32" t="n"/>
       <c r="L232" s="32" t="n"/>
       <c r="M232" s="32" t="n"/>
       <c r="N232" s="32" t="n"/>
@@ -17382,11 +16534,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K233" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K233" s="32" t="n"/>
       <c r="L233" s="32" t="n"/>
       <c r="M233" s="32" t="n"/>
       <c r="N233" s="32" t="n"/>
@@ -17441,11 +16589,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K234" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K234" s="32" t="n"/>
       <c r="L234" s="32" t="n"/>
       <c r="M234" s="32" t="n"/>
       <c r="N234" s="32" t="n"/>
@@ -17497,11 +16641,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K235" s="32" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K235" s="32" t="n"/>
       <c r="L235" s="32" t="n"/>
       <c r="M235" s="32" t="n"/>
       <c r="N235" s="32" t="n"/>
@@ -17557,11 +16697,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K236" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K236" s="66" t="n"/>
       <c r="L236" s="66" t="n"/>
       <c r="M236" s="66" t="n"/>
       <c r="N236" s="66" t="n"/>
@@ -17613,11 +16749,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K237" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K237" s="66" t="n"/>
       <c r="L237" s="66" t="n"/>
       <c r="M237" s="66" t="n"/>
       <c r="N237" s="66" t="n"/>
@@ -17669,11 +16801,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K238" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K238" s="66" t="n"/>
       <c r="L238" s="66" t="n"/>
       <c r="M238" s="66" t="n"/>
       <c r="N238" s="66" t="n"/>
@@ -17725,11 +16853,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K239" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K239" s="66" t="n"/>
       <c r="L239" s="66" t="n"/>
       <c r="M239" s="66" t="n"/>
       <c r="N239" s="66" t="n"/>
@@ -17781,11 +16905,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K240" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K240" s="66" t="n"/>
       <c r="L240" s="66" t="n"/>
       <c r="M240" s="66" t="n"/>
       <c r="N240" s="66" t="n"/>
@@ -17837,11 +16957,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K241" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K241" s="66" t="n"/>
       <c r="L241" s="66" t="n"/>
       <c r="M241" s="66" t="n"/>
       <c r="N241" s="66" t="n"/>
@@ -17893,11 +17009,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K242" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K242" s="66" t="n"/>
       <c r="L242" s="66" t="n"/>
       <c r="M242" s="66" t="n"/>
       <c r="N242" s="66" t="n"/>
@@ -17949,11 +17061,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K243" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K243" s="66" t="n"/>
       <c r="L243" s="66" t="n"/>
       <c r="M243" s="66" t="n"/>
       <c r="N243" s="66" t="n"/>
@@ -18008,11 +17116,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K244" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K244" s="66" t="n"/>
       <c r="L244" s="66" t="n"/>
       <c r="M244" s="66" t="n"/>
       <c r="N244" s="66" t="n"/>
@@ -18064,11 +17168,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K245" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K245" s="66" t="n"/>
       <c r="L245" s="66" t="n"/>
       <c r="M245" s="66" t="n"/>
       <c r="N245" s="66" t="n"/>
@@ -18124,11 +17224,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K246" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K246" s="66" t="n"/>
       <c r="L246" s="66" t="n"/>
       <c r="M246" s="66" t="n"/>
       <c r="N246" s="66" t="n"/>
@@ -18180,11 +17276,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K247" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K247" s="66" t="n"/>
       <c r="L247" s="66" t="n"/>
       <c r="M247" s="66" t="n"/>
       <c r="N247" s="66" t="n"/>
@@ -18236,11 +17328,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K248" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K248" s="66" t="n"/>
       <c r="L248" s="66" t="n"/>
       <c r="M248" s="66" t="n"/>
       <c r="N248" s="66" t="n"/>
@@ -18292,11 +17380,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K249" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K249" s="66" t="n"/>
       <c r="L249" s="66" t="n"/>
       <c r="M249" s="66" t="n"/>
       <c r="N249" s="66" t="n"/>
@@ -18348,11 +17432,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K250" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K250" s="66" t="n"/>
       <c r="L250" s="66" t="n"/>
       <c r="M250" s="66" t="n"/>
       <c r="N250" s="66" t="n"/>
@@ -18404,11 +17484,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K251" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K251" s="66" t="n"/>
       <c r="L251" s="66" t="n"/>
       <c r="M251" s="66" t="n"/>
       <c r="N251" s="66" t="n"/>
@@ -18460,11 +17536,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K252" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K252" s="66" t="n"/>
       <c r="L252" s="66" t="n"/>
       <c r="M252" s="66" t="n"/>
       <c r="N252" s="66" t="n"/>
@@ -18516,11 +17588,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K253" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K253" s="66" t="n"/>
       <c r="L253" s="66" t="n"/>
       <c r="M253" s="66" t="n"/>
       <c r="N253" s="66" t="n"/>
@@ -18572,11 +17640,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K254" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K254" s="66" t="n"/>
       <c r="L254" s="66" t="n"/>
       <c r="M254" s="66" t="n"/>
       <c r="N254" s="66" t="n"/>
@@ -18628,11 +17692,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K255" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K255" s="66" t="n"/>
       <c r="L255" s="66" t="n"/>
       <c r="M255" s="66" t="n"/>
       <c r="N255" s="66" t="n"/>
@@ -18684,11 +17744,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K256" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K256" s="66" t="n"/>
       <c r="L256" s="66" t="n"/>
       <c r="M256" s="66" t="n"/>
       <c r="N256" s="66" t="n"/>
@@ -18740,11 +17796,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K257" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K257" s="66" t="n"/>
       <c r="L257" s="66" t="n"/>
       <c r="M257" s="66" t="n"/>
       <c r="N257" s="66" t="n"/>
@@ -18796,11 +17848,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K258" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K258" s="66" t="n"/>
       <c r="L258" s="66" t="n"/>
       <c r="M258" s="66" t="n"/>
       <c r="N258" s="66" t="n"/>
@@ -18852,11 +17900,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K259" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K259" s="66" t="n"/>
       <c r="L259" s="66" t="n"/>
       <c r="M259" s="66" t="n"/>
       <c r="N259" s="66" t="n"/>
@@ -18908,11 +17952,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K260" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K260" s="66" t="n"/>
       <c r="L260" s="66" t="n"/>
       <c r="M260" s="66" t="n"/>
       <c r="N260" s="66" t="n"/>
@@ -18964,11 +18004,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K261" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K261" s="66" t="n"/>
       <c r="L261" s="66" t="n"/>
       <c r="M261" s="66" t="n"/>
       <c r="N261" s="66" t="n"/>
@@ -19020,11 +18056,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K262" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K262" s="66" t="n"/>
       <c r="L262" s="66" t="n"/>
       <c r="M262" s="66" t="n"/>
       <c r="N262" s="66" t="n"/>
@@ -19076,11 +18108,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K263" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K263" s="66" t="n"/>
       <c r="L263" s="66" t="n"/>
       <c r="M263" s="66" t="n"/>
       <c r="N263" s="66" t="n"/>
@@ -19135,11 +18163,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K264" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K264" s="66" t="n"/>
       <c r="L264" s="66" t="n"/>
       <c r="M264" s="66" t="n"/>
       <c r="N264" s="66" t="n"/>
@@ -19191,11 +18215,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K265" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K265" s="66" t="n"/>
       <c r="L265" s="66" t="n"/>
       <c r="M265" s="66" t="n"/>
       <c r="N265" s="66" t="n"/>
@@ -19251,11 +18271,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K266" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K266" s="66" t="n"/>
       <c r="L266" s="66" t="n"/>
       <c r="M266" s="66" t="n"/>
       <c r="N266" s="66" t="n"/>
@@ -19307,11 +18323,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K267" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K267" s="66" t="n"/>
       <c r="L267" s="66" t="n"/>
       <c r="M267" s="66" t="n"/>
       <c r="N267" s="66" t="n"/>
@@ -19363,11 +18375,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K268" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K268" s="66" t="n"/>
       <c r="L268" s="66" t="n"/>
       <c r="M268" s="66" t="n"/>
       <c r="N268" s="66" t="n"/>
@@ -19419,11 +18427,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K269" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K269" s="66" t="n"/>
       <c r="L269" s="66" t="n"/>
       <c r="M269" s="66" t="n"/>
       <c r="N269" s="66" t="n"/>
@@ -19475,11 +18479,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K270" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K270" s="66" t="n"/>
       <c r="L270" s="66" t="n"/>
       <c r="M270" s="66" t="n"/>
       <c r="N270" s="66" t="n"/>
@@ -19531,11 +18531,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K271" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K271" s="66" t="n"/>
       <c r="L271" s="66" t="n"/>
       <c r="M271" s="66" t="n"/>
       <c r="N271" s="66" t="n"/>
@@ -19587,11 +18583,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K272" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K272" s="66" t="n"/>
       <c r="L272" s="66" t="n"/>
       <c r="M272" s="66" t="n"/>
       <c r="N272" s="66" t="n"/>
@@ -19643,11 +18635,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K273" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K273" s="66" t="n"/>
       <c r="L273" s="66" t="n"/>
       <c r="M273" s="66" t="n"/>
       <c r="N273" s="66" t="n"/>
@@ -19699,11 +18687,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K274" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K274" s="66" t="n"/>
       <c r="L274" s="66" t="n"/>
       <c r="M274" s="66" t="n"/>
       <c r="N274" s="66" t="n"/>
@@ -19755,11 +18739,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K275" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K275" s="66" t="n"/>
       <c r="L275" s="66" t="n"/>
       <c r="M275" s="66" t="n"/>
       <c r="N275" s="66" t="n"/>
@@ -19811,11 +18791,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K276" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K276" s="66" t="n"/>
       <c r="L276" s="66" t="n"/>
       <c r="M276" s="66" t="n"/>
       <c r="N276" s="66" t="n"/>
@@ -19867,11 +18843,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K277" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K277" s="66" t="n"/>
       <c r="L277" s="66" t="n"/>
       <c r="M277" s="66" t="n"/>
       <c r="N277" s="66" t="n"/>
@@ -19923,11 +18895,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K278" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K278" s="66" t="n"/>
       <c r="L278" s="66" t="n"/>
       <c r="M278" s="66" t="n"/>
       <c r="N278" s="66" t="n"/>
@@ -19979,11 +18947,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K279" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K279" s="66" t="n"/>
       <c r="L279" s="66" t="n"/>
       <c r="M279" s="66" t="n"/>
       <c r="N279" s="66" t="n"/>
@@ -20035,11 +18999,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K280" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K280" s="66" t="n"/>
       <c r="L280" s="66" t="n"/>
       <c r="M280" s="66" t="n"/>
       <c r="N280" s="66" t="n"/>
@@ -20091,11 +19051,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K281" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K281" s="66" t="n"/>
       <c r="L281" s="66" t="n"/>
       <c r="M281" s="66" t="n"/>
       <c r="N281" s="66" t="n"/>
@@ -20147,11 +19103,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K282" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K282" s="66" t="n"/>
       <c r="L282" s="66" t="n"/>
       <c r="M282" s="66" t="n"/>
       <c r="N282" s="66" t="n"/>
@@ -20203,11 +19155,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K283" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K283" s="66" t="n"/>
       <c r="L283" s="66" t="n"/>
       <c r="M283" s="66" t="n"/>
       <c r="N283" s="66" t="n"/>
@@ -20262,11 +19210,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K284" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K284" s="66" t="n"/>
       <c r="L284" s="66" t="n"/>
       <c r="M284" s="66" t="n"/>
       <c r="N284" s="66" t="n"/>
@@ -20318,11 +19262,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K285" s="66" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
+      <c r="K285" s="66" t="n"/>
       <c r="L285" s="66" t="n"/>
       <c r="M285" s="66" t="n"/>
       <c r="N285" s="66" t="n"/>
@@ -21397,6 +20337,26 @@
       <c r="W375" s="7" t="n"/>
     </row>
     <row r="376" ht="14.25" customHeight="1" s="50">
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>25/03/2026</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>346c86394d9e19688c98e1eac3507b73</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.2081e93bc59b43e49e3aeae958e60c84dccb7d9ecdcb4e330174098f046ce5f1.617e1f2a25^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>LAB_VALIDATION.pdf</t>
+        </is>
+      </c>
       <c r="W376" s="7" t="n"/>
     </row>
     <row r="377" ht="14.25" customHeight="1" s="50">

</xml_diff>

<commit_message>
Fix report-checklist v2: correct column mapping (J=Applicabilita, L=Razionale), fill all SI rows
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#CENTROPOLISPECIALISTICOGIOVANNIPAOLOIXX/GPI_HEALTH_SYSTEM/FSE_SENDER/V.1.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#CENTROPOLISPECIALISTICOGIOVANNIPAOLOIXX/GPI_HEALTH_SYSTEM/FSE_SENDER/V.1.0/report-checklist.xlsx
@@ -2862,7 +2862,11 @@
         </is>
       </c>
       <c r="K12" s="32" t="n"/>
-      <c r="L12" s="32" t="n"/>
+      <c r="L12" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M12" s="32" t="n"/>
       <c r="N12" s="32" t="n"/>
       <c r="O12" s="32" t="n"/>
@@ -2917,7 +2921,11 @@
         </is>
       </c>
       <c r="K13" s="32" t="n"/>
-      <c r="L13" s="32" t="n"/>
+      <c r="L13" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M13" s="32" t="n"/>
       <c r="N13" s="32" t="n"/>
       <c r="O13" s="32" t="n"/>
@@ -3154,7 +3162,11 @@
         </is>
       </c>
       <c r="K16" s="32" t="n"/>
-      <c r="L16" s="32" t="n"/>
+      <c r="L16" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M16" s="32" t="n"/>
       <c r="N16" s="32" t="n"/>
       <c r="O16" s="32" t="n"/>
@@ -3209,7 +3221,11 @@
         </is>
       </c>
       <c r="K17" s="32" t="n"/>
-      <c r="L17" s="32" t="n"/>
+      <c r="L17" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M17" s="32" t="n"/>
       <c r="N17" s="32" t="n"/>
       <c r="O17" s="32" t="n"/>
@@ -3264,7 +3280,11 @@
         </is>
       </c>
       <c r="K18" s="32" t="n"/>
-      <c r="L18" s="32" t="n"/>
+      <c r="L18" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M18" s="32" t="n"/>
       <c r="N18" s="32" t="n"/>
       <c r="O18" s="32" t="n"/>
@@ -3410,7 +3430,11 @@
         </is>
       </c>
       <c r="K20" s="32" t="n"/>
-      <c r="L20" s="32" t="n"/>
+      <c r="L20" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M20" s="32" t="n"/>
       <c r="N20" s="32" t="n"/>
       <c r="O20" s="32" t="n"/>
@@ -3465,7 +3489,11 @@
         </is>
       </c>
       <c r="K21" s="32" t="n"/>
-      <c r="L21" s="32" t="n"/>
+      <c r="L21" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M21" s="32" t="n"/>
       <c r="N21" s="32" t="n"/>
       <c r="O21" s="32" t="n"/>
@@ -3702,7 +3730,11 @@
         </is>
       </c>
       <c r="K24" s="32" t="n"/>
-      <c r="L24" s="32" t="n"/>
+      <c r="L24" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M24" s="32" t="n"/>
       <c r="N24" s="32" t="n"/>
       <c r="O24" s="32" t="n"/>
@@ -3757,7 +3789,11 @@
         </is>
       </c>
       <c r="K25" s="32" t="n"/>
-      <c r="L25" s="32" t="n"/>
+      <c r="L25" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M25" s="32" t="n"/>
       <c r="N25" s="32" t="n"/>
       <c r="O25" s="32" t="n"/>
@@ -3812,7 +3848,11 @@
         </is>
       </c>
       <c r="K26" s="32" t="n"/>
-      <c r="L26" s="32" t="n"/>
+      <c r="L26" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M26" s="32" t="n"/>
       <c r="N26" s="32" t="n"/>
       <c r="O26" s="32" t="n"/>
@@ -3956,7 +3996,11 @@
         </is>
       </c>
       <c r="K28" s="32" t="n"/>
-      <c r="L28" s="32" t="n"/>
+      <c r="L28" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M28" s="32" t="n"/>
       <c r="N28" s="32" t="n"/>
       <c r="O28" s="32" t="n"/>
@@ -4012,7 +4056,11 @@
         </is>
       </c>
       <c r="K29" s="32" t="n"/>
-      <c r="L29" s="32" t="n"/>
+      <c r="L29" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M29" s="32" t="n"/>
       <c r="N29" s="32" t="n"/>
       <c r="O29" s="32" t="n"/>
@@ -4252,7 +4300,11 @@
         </is>
       </c>
       <c r="K32" s="32" t="n"/>
-      <c r="L32" s="32" t="n"/>
+      <c r="L32" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M32" s="32" t="n"/>
       <c r="N32" s="32" t="n"/>
       <c r="O32" s="32" t="n"/>
@@ -4308,7 +4360,11 @@
         </is>
       </c>
       <c r="K33" s="32" t="n"/>
-      <c r="L33" s="32" t="n"/>
+      <c r="L33" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M33" s="32" t="n"/>
       <c r="N33" s="32" t="n"/>
       <c r="O33" s="32" t="n"/>
@@ -4364,7 +4420,11 @@
         </is>
       </c>
       <c r="K34" s="32" t="n"/>
-      <c r="L34" s="32" t="n"/>
+      <c r="L34" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M34" s="32" t="n"/>
       <c r="N34" s="32" t="n"/>
       <c r="O34" s="32" t="n"/>
@@ -5124,7 +5184,11 @@
         </is>
       </c>
       <c r="K43" s="32" t="n"/>
-      <c r="L43" s="32" t="n"/>
+      <c r="L43" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M43" s="32" t="n"/>
       <c r="N43" s="32" t="n"/>
       <c r="O43" s="32" t="n"/>
@@ -5176,7 +5240,11 @@
         </is>
       </c>
       <c r="K44" s="32" t="n"/>
-      <c r="L44" s="32" t="n"/>
+      <c r="L44" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M44" s="32" t="n"/>
       <c r="N44" s="32" t="n"/>
       <c r="O44" s="32" t="n"/>
@@ -5228,7 +5296,11 @@
         </is>
       </c>
       <c r="K45" s="32" t="n"/>
-      <c r="L45" s="32" t="n"/>
+      <c r="L45" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M45" s="32" t="n"/>
       <c r="N45" s="32" t="n"/>
       <c r="O45" s="32" t="n"/>
@@ -5280,7 +5352,11 @@
         </is>
       </c>
       <c r="K46" s="32" t="n"/>
-      <c r="L46" s="32" t="n"/>
+      <c r="L46" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M46" s="32" t="n"/>
       <c r="N46" s="32" t="n"/>
       <c r="O46" s="32" t="n"/>
@@ -5332,7 +5408,11 @@
         </is>
       </c>
       <c r="K47" s="32" t="n"/>
-      <c r="L47" s="32" t="n"/>
+      <c r="L47" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M47" s="32" t="n"/>
       <c r="N47" s="32" t="n"/>
       <c r="O47" s="32" t="n"/>
@@ -5384,7 +5464,11 @@
         </is>
       </c>
       <c r="K48" s="32" t="n"/>
-      <c r="L48" s="32" t="n"/>
+      <c r="L48" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M48" s="32" t="n"/>
       <c r="N48" s="32" t="n"/>
       <c r="O48" s="32" t="n"/>
@@ -5436,7 +5520,11 @@
         </is>
       </c>
       <c r="K49" s="32" t="n"/>
-      <c r="L49" s="32" t="n"/>
+      <c r="L49" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M49" s="32" t="n"/>
       <c r="N49" s="32" t="n"/>
       <c r="O49" s="32" t="n"/>
@@ -5488,7 +5576,11 @@
         </is>
       </c>
       <c r="K50" s="32" t="n"/>
-      <c r="L50" s="32" t="n"/>
+      <c r="L50" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M50" s="32" t="n"/>
       <c r="N50" s="32" t="n"/>
       <c r="O50" s="32" t="n"/>
@@ -5540,7 +5632,11 @@
         </is>
       </c>
       <c r="K51" s="32" t="n"/>
-      <c r="L51" s="32" t="n"/>
+      <c r="L51" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M51" s="32" t="n"/>
       <c r="N51" s="32" t="n"/>
       <c r="O51" s="32" t="n"/>
@@ -5592,7 +5688,11 @@
         </is>
       </c>
       <c r="K52" s="32" t="n"/>
-      <c r="L52" s="32" t="n"/>
+      <c r="L52" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M52" s="32" t="n"/>
       <c r="N52" s="32" t="n"/>
       <c r="O52" s="32" t="n"/>
@@ -7052,7 +7152,11 @@
         </is>
       </c>
       <c r="K69" s="32" t="n"/>
-      <c r="L69" s="32" t="n"/>
+      <c r="L69" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M69" s="32" t="n"/>
       <c r="N69" s="32" t="n"/>
       <c r="O69" s="32" t="n"/>
@@ -7104,7 +7208,11 @@
         </is>
       </c>
       <c r="K70" s="32" t="n"/>
-      <c r="L70" s="32" t="n"/>
+      <c r="L70" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M70" s="32" t="n"/>
       <c r="N70" s="32" t="n"/>
       <c r="O70" s="32" t="n"/>
@@ -7156,7 +7264,11 @@
         </is>
       </c>
       <c r="K71" s="32" t="n"/>
-      <c r="L71" s="32" t="n"/>
+      <c r="L71" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M71" s="32" t="n"/>
       <c r="N71" s="32" t="n"/>
       <c r="O71" s="32" t="n"/>
@@ -7208,7 +7320,11 @@
         </is>
       </c>
       <c r="K72" s="32" t="n"/>
-      <c r="L72" s="32" t="n"/>
+      <c r="L72" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M72" s="32" t="n"/>
       <c r="N72" s="32" t="n"/>
       <c r="O72" s="32" t="n"/>
@@ -7260,7 +7376,11 @@
         </is>
       </c>
       <c r="K73" s="32" t="n"/>
-      <c r="L73" s="32" t="n"/>
+      <c r="L73" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M73" s="32" t="n"/>
       <c r="N73" s="32" t="n"/>
       <c r="O73" s="32" t="n"/>
@@ -7312,7 +7432,11 @@
         </is>
       </c>
       <c r="K74" s="32" t="n"/>
-      <c r="L74" s="32" t="n"/>
+      <c r="L74" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M74" s="32" t="n"/>
       <c r="N74" s="32" t="n"/>
       <c r="O74" s="32" t="n"/>
@@ -7364,7 +7488,11 @@
         </is>
       </c>
       <c r="K75" s="32" t="n"/>
-      <c r="L75" s="32" t="n"/>
+      <c r="L75" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M75" s="32" t="n"/>
       <c r="N75" s="32" t="n"/>
       <c r="O75" s="32" t="n"/>
@@ -7416,7 +7544,11 @@
         </is>
       </c>
       <c r="K76" s="32" t="n"/>
-      <c r="L76" s="32" t="n"/>
+      <c r="L76" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M76" s="32" t="n"/>
       <c r="N76" s="32" t="n"/>
       <c r="O76" s="32" t="n"/>
@@ -7468,7 +7600,11 @@
         </is>
       </c>
       <c r="K77" s="32" t="n"/>
-      <c r="L77" s="32" t="n"/>
+      <c r="L77" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M77" s="32" t="n"/>
       <c r="N77" s="32" t="n"/>
       <c r="O77" s="32" t="n"/>
@@ -7520,7 +7656,11 @@
         </is>
       </c>
       <c r="K78" s="32" t="n"/>
-      <c r="L78" s="32" t="n"/>
+      <c r="L78" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M78" s="32" t="n"/>
       <c r="N78" s="32" t="n"/>
       <c r="O78" s="32" t="n"/>
@@ -7572,7 +7712,11 @@
         </is>
       </c>
       <c r="K79" s="32" t="n"/>
-      <c r="L79" s="32" t="n"/>
+      <c r="L79" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M79" s="32" t="n"/>
       <c r="N79" s="32" t="n"/>
       <c r="O79" s="32" t="n"/>
@@ -7624,7 +7768,11 @@
         </is>
       </c>
       <c r="K80" s="32" t="n"/>
-      <c r="L80" s="32" t="n"/>
+      <c r="L80" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M80" s="32" t="n"/>
       <c r="N80" s="32" t="n"/>
       <c r="O80" s="32" t="n"/>
@@ -7676,7 +7824,11 @@
         </is>
       </c>
       <c r="K81" s="32" t="n"/>
-      <c r="L81" s="32" t="n"/>
+      <c r="L81" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M81" s="32" t="n"/>
       <c r="N81" s="32" t="n"/>
       <c r="O81" s="32" t="n"/>
@@ -7728,7 +7880,11 @@
         </is>
       </c>
       <c r="K82" s="32" t="n"/>
-      <c r="L82" s="32" t="n"/>
+      <c r="L82" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M82" s="32" t="n"/>
       <c r="N82" s="32" t="n"/>
       <c r="O82" s="32" t="n"/>
@@ -7780,7 +7936,11 @@
         </is>
       </c>
       <c r="K83" s="32" t="n"/>
-      <c r="L83" s="32" t="n"/>
+      <c r="L83" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M83" s="32" t="n"/>
       <c r="N83" s="32" t="n"/>
       <c r="O83" s="32" t="n"/>
@@ -7832,7 +7992,11 @@
         </is>
       </c>
       <c r="K84" s="32" t="n"/>
-      <c r="L84" s="32" t="n"/>
+      <c r="L84" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M84" s="32" t="n"/>
       <c r="N84" s="32" t="n"/>
       <c r="O84" s="32" t="n"/>
@@ -7884,7 +8048,11 @@
         </is>
       </c>
       <c r="K85" s="32" t="n"/>
-      <c r="L85" s="32" t="n"/>
+      <c r="L85" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M85" s="32" t="n"/>
       <c r="N85" s="32" t="n"/>
       <c r="O85" s="32" t="n"/>
@@ -7936,7 +8104,11 @@
         </is>
       </c>
       <c r="K86" s="32" t="n"/>
-      <c r="L86" s="32" t="n"/>
+      <c r="L86" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M86" s="32" t="n"/>
       <c r="N86" s="32" t="n"/>
       <c r="O86" s="32" t="n"/>
@@ -7988,7 +8160,11 @@
         </is>
       </c>
       <c r="K87" s="32" t="n"/>
-      <c r="L87" s="32" t="n"/>
+      <c r="L87" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M87" s="32" t="n"/>
       <c r="N87" s="32" t="n"/>
       <c r="O87" s="32" t="n"/>
@@ -8040,7 +8216,11 @@
         </is>
       </c>
       <c r="K88" s="32" t="n"/>
-      <c r="L88" s="32" t="n"/>
+      <c r="L88" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M88" s="32" t="n"/>
       <c r="N88" s="32" t="n"/>
       <c r="O88" s="32" t="n"/>
@@ -8092,7 +8272,11 @@
         </is>
       </c>
       <c r="K89" s="32" t="n"/>
-      <c r="L89" s="32" t="n"/>
+      <c r="L89" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M89" s="32" t="n"/>
       <c r="N89" s="32" t="n"/>
       <c r="O89" s="32" t="n"/>
@@ -8144,7 +8328,11 @@
         </is>
       </c>
       <c r="K90" s="32" t="n"/>
-      <c r="L90" s="32" t="n"/>
+      <c r="L90" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M90" s="32" t="n"/>
       <c r="N90" s="32" t="n"/>
       <c r="O90" s="32" t="n"/>
@@ -8196,7 +8384,11 @@
         </is>
       </c>
       <c r="K91" s="32" t="n"/>
-      <c r="L91" s="32" t="n"/>
+      <c r="L91" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M91" s="32" t="n"/>
       <c r="N91" s="32" t="n"/>
       <c r="O91" s="32" t="n"/>
@@ -8248,7 +8440,11 @@
         </is>
       </c>
       <c r="K92" s="32" t="n"/>
-      <c r="L92" s="32" t="n"/>
+      <c r="L92" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M92" s="32" t="n"/>
       <c r="N92" s="32" t="n"/>
       <c r="O92" s="32" t="n"/>
@@ -8300,7 +8496,11 @@
         </is>
       </c>
       <c r="K93" s="32" t="n"/>
-      <c r="L93" s="32" t="n"/>
+      <c r="L93" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M93" s="32" t="n"/>
       <c r="N93" s="32" t="n"/>
       <c r="O93" s="32" t="n"/>
@@ -8352,7 +8552,11 @@
         </is>
       </c>
       <c r="K94" s="32" t="n"/>
-      <c r="L94" s="32" t="n"/>
+      <c r="L94" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M94" s="32" t="n"/>
       <c r="N94" s="32" t="n"/>
       <c r="O94" s="32" t="n"/>
@@ -8404,7 +8608,11 @@
         </is>
       </c>
       <c r="K95" s="32" t="n"/>
-      <c r="L95" s="32" t="n"/>
+      <c r="L95" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M95" s="32" t="n"/>
       <c r="N95" s="32" t="n"/>
       <c r="O95" s="32" t="n"/>
@@ -8456,7 +8664,11 @@
         </is>
       </c>
       <c r="K96" s="32" t="n"/>
-      <c r="L96" s="32" t="n"/>
+      <c r="L96" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M96" s="32" t="n"/>
       <c r="N96" s="32" t="n"/>
       <c r="O96" s="32" t="n"/>
@@ -8508,7 +8720,11 @@
         </is>
       </c>
       <c r="K97" s="32" t="n"/>
-      <c r="L97" s="32" t="n"/>
+      <c r="L97" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M97" s="32" t="n"/>
       <c r="N97" s="32" t="n"/>
       <c r="O97" s="32" t="n"/>
@@ -8560,7 +8776,11 @@
         </is>
       </c>
       <c r="K98" s="32" t="n"/>
-      <c r="L98" s="32" t="n"/>
+      <c r="L98" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M98" s="32" t="n"/>
       <c r="N98" s="32" t="n"/>
       <c r="O98" s="32" t="n"/>
@@ -8612,7 +8832,11 @@
         </is>
       </c>
       <c r="K99" s="32" t="n"/>
-      <c r="L99" s="32" t="n"/>
+      <c r="L99" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M99" s="32" t="n"/>
       <c r="N99" s="32" t="n"/>
       <c r="O99" s="32" t="n"/>
@@ -8664,7 +8888,11 @@
         </is>
       </c>
       <c r="K100" s="32" t="n"/>
-      <c r="L100" s="32" t="n"/>
+      <c r="L100" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M100" s="32" t="n"/>
       <c r="N100" s="32" t="n"/>
       <c r="O100" s="32" t="n"/>
@@ -8716,7 +8944,11 @@
         </is>
       </c>
       <c r="K101" s="32" t="n"/>
-      <c r="L101" s="32" t="n"/>
+      <c r="L101" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M101" s="32" t="n"/>
       <c r="N101" s="32" t="n"/>
       <c r="O101" s="32" t="n"/>
@@ -8768,7 +9000,11 @@
         </is>
       </c>
       <c r="K102" s="32" t="n"/>
-      <c r="L102" s="32" t="n"/>
+      <c r="L102" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M102" s="32" t="n"/>
       <c r="N102" s="32" t="n"/>
       <c r="O102" s="32" t="n"/>
@@ -8820,7 +9056,11 @@
         </is>
       </c>
       <c r="K103" s="32" t="n"/>
-      <c r="L103" s="32" t="n"/>
+      <c r="L103" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M103" s="32" t="n"/>
       <c r="N103" s="32" t="n"/>
       <c r="O103" s="32" t="n"/>
@@ -8872,7 +9112,11 @@
         </is>
       </c>
       <c r="K104" s="32" t="n"/>
-      <c r="L104" s="32" t="n"/>
+      <c r="L104" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M104" s="32" t="n"/>
       <c r="N104" s="32" t="n"/>
       <c r="O104" s="32" t="n"/>
@@ -8924,7 +9168,11 @@
         </is>
       </c>
       <c r="K105" s="32" t="n"/>
-      <c r="L105" s="32" t="n"/>
+      <c r="L105" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M105" s="32" t="n"/>
       <c r="N105" s="32" t="n"/>
       <c r="O105" s="32" t="n"/>
@@ -8976,7 +9224,11 @@
         </is>
       </c>
       <c r="K106" s="32" t="n"/>
-      <c r="L106" s="32" t="n"/>
+      <c r="L106" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M106" s="32" t="n"/>
       <c r="N106" s="32" t="n"/>
       <c r="O106" s="32" t="n"/>
@@ -9028,7 +9280,11 @@
         </is>
       </c>
       <c r="K107" s="32" t="n"/>
-      <c r="L107" s="32" t="n"/>
+      <c r="L107" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M107" s="32" t="n"/>
       <c r="N107" s="32" t="n"/>
       <c r="O107" s="32" t="n"/>
@@ -9080,7 +9336,11 @@
         </is>
       </c>
       <c r="K108" s="32" t="n"/>
-      <c r="L108" s="32" t="n"/>
+      <c r="L108" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M108" s="32" t="n"/>
       <c r="N108" s="32" t="n"/>
       <c r="O108" s="32" t="n"/>
@@ -9132,7 +9392,11 @@
         </is>
       </c>
       <c r="K109" s="32" t="n"/>
-      <c r="L109" s="32" t="n"/>
+      <c r="L109" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M109" s="32" t="n"/>
       <c r="N109" s="32" t="n"/>
       <c r="O109" s="32" t="n"/>
@@ -9184,7 +9448,11 @@
         </is>
       </c>
       <c r="K110" s="32" t="n"/>
-      <c r="L110" s="32" t="n"/>
+      <c r="L110" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M110" s="32" t="n"/>
       <c r="N110" s="32" t="n"/>
       <c r="O110" s="32" t="n"/>
@@ -9236,7 +9504,11 @@
         </is>
       </c>
       <c r="K111" s="32" t="n"/>
-      <c r="L111" s="32" t="n"/>
+      <c r="L111" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M111" s="32" t="n"/>
       <c r="N111" s="32" t="n"/>
       <c r="O111" s="32" t="n"/>
@@ -9288,7 +9560,11 @@
         </is>
       </c>
       <c r="K112" s="32" t="n"/>
-      <c r="L112" s="32" t="n"/>
+      <c r="L112" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M112" s="32" t="n"/>
       <c r="N112" s="32" t="n"/>
       <c r="O112" s="32" t="n"/>
@@ -9340,7 +9616,11 @@
         </is>
       </c>
       <c r="K113" s="32" t="n"/>
-      <c r="L113" s="32" t="n"/>
+      <c r="L113" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M113" s="32" t="n"/>
       <c r="N113" s="32" t="n"/>
       <c r="O113" s="32" t="n"/>
@@ -9392,7 +9672,11 @@
         </is>
       </c>
       <c r="K114" s="32" t="n"/>
-      <c r="L114" s="32" t="n"/>
+      <c r="L114" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M114" s="32" t="n"/>
       <c r="N114" s="32" t="n"/>
       <c r="O114" s="32" t="n"/>
@@ -9444,7 +9728,11 @@
         </is>
       </c>
       <c r="K115" s="32" t="n"/>
-      <c r="L115" s="32" t="n"/>
+      <c r="L115" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M115" s="32" t="n"/>
       <c r="N115" s="32" t="n"/>
       <c r="O115" s="32" t="n"/>
@@ -10816,7 +11104,11 @@
         </is>
       </c>
       <c r="K131" s="32" t="n"/>
-      <c r="L131" s="32" t="n"/>
+      <c r="L131" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M131" s="32" t="n"/>
       <c r="N131" s="32" t="n"/>
       <c r="O131" s="32" t="n"/>
@@ -10868,7 +11160,11 @@
         </is>
       </c>
       <c r="K132" s="32" t="n"/>
-      <c r="L132" s="32" t="n"/>
+      <c r="L132" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M132" s="32" t="n"/>
       <c r="N132" s="32" t="n"/>
       <c r="O132" s="32" t="n"/>
@@ -10920,7 +11216,11 @@
         </is>
       </c>
       <c r="K133" s="32" t="n"/>
-      <c r="L133" s="32" t="n"/>
+      <c r="L133" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M133" s="32" t="n"/>
       <c r="N133" s="32" t="n"/>
       <c r="O133" s="32" t="n"/>
@@ -10972,7 +11272,11 @@
         </is>
       </c>
       <c r="K134" s="32" t="n"/>
-      <c r="L134" s="32" t="n"/>
+      <c r="L134" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M134" s="32" t="n"/>
       <c r="N134" s="32" t="n"/>
       <c r="O134" s="32" t="n"/>
@@ -11024,7 +11328,11 @@
         </is>
       </c>
       <c r="K135" s="32" t="n"/>
-      <c r="L135" s="32" t="n"/>
+      <c r="L135" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M135" s="32" t="n"/>
       <c r="N135" s="32" t="n"/>
       <c r="O135" s="32" t="n"/>
@@ -11076,7 +11384,11 @@
         </is>
       </c>
       <c r="K136" s="32" t="n"/>
-      <c r="L136" s="32" t="n"/>
+      <c r="L136" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M136" s="32" t="n"/>
       <c r="N136" s="32" t="n"/>
       <c r="O136" s="32" t="n"/>
@@ -11128,7 +11440,11 @@
         </is>
       </c>
       <c r="K137" s="32" t="n"/>
-      <c r="L137" s="32" t="n"/>
+      <c r="L137" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M137" s="32" t="n"/>
       <c r="N137" s="32" t="n"/>
       <c r="O137" s="32" t="n"/>
@@ -11180,7 +11496,11 @@
         </is>
       </c>
       <c r="K138" s="32" t="n"/>
-      <c r="L138" s="32" t="n"/>
+      <c r="L138" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M138" s="32" t="n"/>
       <c r="N138" s="32" t="n"/>
       <c r="O138" s="32" t="n"/>
@@ -11232,7 +11552,11 @@
         </is>
       </c>
       <c r="K139" s="32" t="n"/>
-      <c r="L139" s="32" t="n"/>
+      <c r="L139" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M139" s="32" t="n"/>
       <c r="N139" s="32" t="n"/>
       <c r="O139" s="32" t="n"/>
@@ -11284,7 +11608,11 @@
         </is>
       </c>
       <c r="K140" s="32" t="n"/>
-      <c r="L140" s="32" t="n"/>
+      <c r="L140" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M140" s="32" t="n"/>
       <c r="N140" s="32" t="n"/>
       <c r="O140" s="32" t="n"/>
@@ -11336,7 +11664,11 @@
         </is>
       </c>
       <c r="K141" s="32" t="n"/>
-      <c r="L141" s="32" t="n"/>
+      <c r="L141" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M141" s="32" t="n"/>
       <c r="N141" s="32" t="n"/>
       <c r="O141" s="32" t="n"/>
@@ -11388,7 +11720,11 @@
         </is>
       </c>
       <c r="K142" s="32" t="n"/>
-      <c r="L142" s="32" t="n"/>
+      <c r="L142" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M142" s="32" t="n"/>
       <c r="N142" s="32" t="n"/>
       <c r="O142" s="32" t="n"/>
@@ -11440,7 +11776,11 @@
         </is>
       </c>
       <c r="K143" s="32" t="n"/>
-      <c r="L143" s="32" t="n"/>
+      <c r="L143" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M143" s="32" t="n"/>
       <c r="N143" s="32" t="n"/>
       <c r="O143" s="32" t="n"/>
@@ -11492,7 +11832,11 @@
         </is>
       </c>
       <c r="K144" s="32" t="n"/>
-      <c r="L144" s="32" t="n"/>
+      <c r="L144" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M144" s="32" t="n"/>
       <c r="N144" s="32" t="n"/>
       <c r="O144" s="32" t="n"/>
@@ -11544,7 +11888,11 @@
         </is>
       </c>
       <c r="K145" s="32" t="n"/>
-      <c r="L145" s="32" t="n"/>
+      <c r="L145" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M145" s="32" t="n"/>
       <c r="N145" s="32" t="n"/>
       <c r="O145" s="32" t="n"/>
@@ -11592,9 +11940,21 @@
           <t>25/03/2026</t>
         </is>
       </c>
-      <c r="G146" s="31" t="n"/>
-      <c r="H146" s="31" t="n"/>
-      <c r="I146" s="36" t="n"/>
+      <c r="G146" s="31" t="inlineStr">
+        <is>
+          <t>2026-03-26T08:16:15</t>
+        </is>
+      </c>
+      <c r="H146" s="31" t="inlineStr">
+        <is>
+          <t>ff55db762ded2539affd730de18bd8c1</t>
+        </is>
+      </c>
+      <c r="I146" s="36" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.8b4e07e56d5aa565f9a8de121321d2d8eb791aefc994d88859d9672a4b396b04.66e074ff48^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J146" s="32" t="inlineStr">
         <is>
           <t>SI</t>
@@ -11653,9 +12013,21 @@
           <t>25/03/2026</t>
         </is>
       </c>
-      <c r="G147" s="31" t="n"/>
-      <c r="H147" s="31" t="n"/>
-      <c r="I147" s="36" t="n"/>
+      <c r="G147" s="31" t="inlineStr">
+        <is>
+          <t>2026-03-26T08:16:12</t>
+        </is>
+      </c>
+      <c r="H147" s="31" t="inlineStr">
+        <is>
+          <t>e7b184d9004b721d45058522970f3cb8</t>
+        </is>
+      </c>
+      <c r="I147" s="36" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.c7cfc54dcfac0c48c09bb8cfef8f6d91bce2ddc0f8c56e438d3312b3358a249c.8538eae2a6^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J147" s="32" t="inlineStr">
         <is>
           <t>SI</t>
@@ -11718,7 +12090,11 @@
         </is>
       </c>
       <c r="K148" s="32" t="n"/>
-      <c r="L148" s="32" t="n"/>
+      <c r="L148" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M148" s="32" t="n"/>
       <c r="N148" s="32" t="n"/>
       <c r="O148" s="32" t="n"/>
@@ -11771,7 +12147,11 @@
         </is>
       </c>
       <c r="K149" s="32" t="n"/>
-      <c r="L149" s="32" t="n"/>
+      <c r="L149" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M149" s="32" t="n"/>
       <c r="N149" s="32" t="n"/>
       <c r="O149" s="32" t="n"/>
@@ -11824,7 +12204,11 @@
         </is>
       </c>
       <c r="K150" s="32" t="n"/>
-      <c r="L150" s="32" t="n"/>
+      <c r="L150" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M150" s="32" t="n"/>
       <c r="N150" s="32" t="n"/>
       <c r="O150" s="32" t="n"/>
@@ -11879,7 +12263,11 @@
         </is>
       </c>
       <c r="K151" s="32" t="n"/>
-      <c r="L151" s="32" t="n"/>
+      <c r="L151" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M151" s="32" t="n"/>
       <c r="N151" s="32" t="n"/>
       <c r="O151" s="32" t="n"/>
@@ -11934,7 +12322,11 @@
         </is>
       </c>
       <c r="K152" s="32" t="n"/>
-      <c r="L152" s="32" t="n"/>
+      <c r="L152" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M152" s="32" t="n"/>
       <c r="N152" s="32" t="n"/>
       <c r="O152" s="32" t="n"/>
@@ -11986,7 +12378,11 @@
         </is>
       </c>
       <c r="K153" s="32" t="n"/>
-      <c r="L153" s="32" t="n"/>
+      <c r="L153" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M153" s="32" t="n"/>
       <c r="N153" s="32" t="n"/>
       <c r="O153" s="32" t="n"/>
@@ -12042,7 +12438,11 @@
         </is>
       </c>
       <c r="K154" s="32" t="n"/>
-      <c r="L154" s="32" t="n"/>
+      <c r="L154" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M154" s="32" t="n"/>
       <c r="N154" s="32" t="n"/>
       <c r="O154" s="32" t="n"/>
@@ -12094,7 +12494,11 @@
         </is>
       </c>
       <c r="K155" s="32" t="n"/>
-      <c r="L155" s="32" t="n"/>
+      <c r="L155" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M155" s="32" t="n"/>
       <c r="N155" s="32" t="n"/>
       <c r="O155" s="32" t="n"/>
@@ -12146,7 +12550,11 @@
         </is>
       </c>
       <c r="K156" s="32" t="n"/>
-      <c r="L156" s="32" t="n"/>
+      <c r="L156" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M156" s="32" t="n"/>
       <c r="N156" s="32" t="n"/>
       <c r="O156" s="32" t="n"/>
@@ -12198,7 +12606,11 @@
         </is>
       </c>
       <c r="K157" s="32" t="n"/>
-      <c r="L157" s="32" t="n"/>
+      <c r="L157" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M157" s="32" t="n"/>
       <c r="N157" s="32" t="n"/>
       <c r="O157" s="32" t="n"/>
@@ -12250,7 +12662,11 @@
         </is>
       </c>
       <c r="K158" s="32" t="n"/>
-      <c r="L158" s="32" t="n"/>
+      <c r="L158" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M158" s="32" t="n"/>
       <c r="N158" s="32" t="n"/>
       <c r="O158" s="32" t="n"/>
@@ -12302,7 +12718,11 @@
         </is>
       </c>
       <c r="K159" s="32" t="n"/>
-      <c r="L159" s="32" t="n"/>
+      <c r="L159" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M159" s="32" t="n"/>
       <c r="N159" s="32" t="n"/>
       <c r="O159" s="32" t="n"/>
@@ -12354,7 +12774,11 @@
         </is>
       </c>
       <c r="K160" s="32" t="n"/>
-      <c r="L160" s="32" t="n"/>
+      <c r="L160" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M160" s="32" t="n"/>
       <c r="N160" s="32" t="n"/>
       <c r="O160" s="32" t="n"/>
@@ -12406,7 +12830,11 @@
         </is>
       </c>
       <c r="K161" s="32" t="n"/>
-      <c r="L161" s="32" t="n"/>
+      <c r="L161" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M161" s="32" t="n"/>
       <c r="N161" s="32" t="n"/>
       <c r="O161" s="32" t="n"/>
@@ -12458,7 +12886,11 @@
         </is>
       </c>
       <c r="K162" s="32" t="n"/>
-      <c r="L162" s="32" t="n"/>
+      <c r="L162" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M162" s="32" t="n"/>
       <c r="N162" s="32" t="n"/>
       <c r="O162" s="32" t="n"/>
@@ -12510,7 +12942,11 @@
         </is>
       </c>
       <c r="K163" s="32" t="n"/>
-      <c r="L163" s="32" t="n"/>
+      <c r="L163" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M163" s="32" t="n"/>
       <c r="N163" s="32" t="n"/>
       <c r="O163" s="32" t="n"/>
@@ -12706,7 +13142,11 @@
         </is>
       </c>
       <c r="K166" s="32" t="n"/>
-      <c r="L166" s="32" t="n"/>
+      <c r="L166" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M166" s="32" t="n"/>
       <c r="N166" s="32" t="n"/>
       <c r="O166" s="32" t="n"/>
@@ -12758,7 +13198,11 @@
         </is>
       </c>
       <c r="K167" s="32" t="n"/>
-      <c r="L167" s="32" t="n"/>
+      <c r="L167" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M167" s="32" t="n"/>
       <c r="N167" s="32" t="n"/>
       <c r="O167" s="32" t="n"/>
@@ -12883,7 +13327,11 @@
         </is>
       </c>
       <c r="K169" s="32" t="n"/>
-      <c r="L169" s="32" t="n"/>
+      <c r="L169" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M169" s="32" t="n"/>
       <c r="N169" s="32" t="n"/>
       <c r="O169" s="32" t="n"/>
@@ -12935,7 +13383,11 @@
         </is>
       </c>
       <c r="K170" s="32" t="n"/>
-      <c r="L170" s="32" t="n"/>
+      <c r="L170" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M170" s="32" t="n"/>
       <c r="N170" s="32" t="n"/>
       <c r="O170" s="32" t="n"/>
@@ -12987,7 +13439,11 @@
         </is>
       </c>
       <c r="K171" s="32" t="n"/>
-      <c r="L171" s="32" t="n"/>
+      <c r="L171" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M171" s="32" t="n"/>
       <c r="N171" s="32" t="n"/>
       <c r="O171" s="32" t="n"/>
@@ -13039,7 +13495,11 @@
         </is>
       </c>
       <c r="K172" s="32" t="n"/>
-      <c r="L172" s="32" t="n"/>
+      <c r="L172" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M172" s="32" t="n"/>
       <c r="N172" s="32" t="n"/>
       <c r="O172" s="32" t="n"/>
@@ -13091,7 +13551,11 @@
         </is>
       </c>
       <c r="K173" s="32" t="n"/>
-      <c r="L173" s="32" t="n"/>
+      <c r="L173" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M173" s="32" t="n"/>
       <c r="N173" s="32" t="n"/>
       <c r="O173" s="32" t="n"/>
@@ -13143,7 +13607,11 @@
         </is>
       </c>
       <c r="K174" s="32" t="n"/>
-      <c r="L174" s="32" t="n"/>
+      <c r="L174" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M174" s="32" t="n"/>
       <c r="N174" s="32" t="n"/>
       <c r="O174" s="32" t="n"/>
@@ -13195,7 +13663,11 @@
         </is>
       </c>
       <c r="K175" s="32" t="n"/>
-      <c r="L175" s="32" t="n"/>
+      <c r="L175" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M175" s="32" t="n"/>
       <c r="N175" s="32" t="n"/>
       <c r="O175" s="32" t="n"/>
@@ -13423,7 +13895,11 @@
         </is>
       </c>
       <c r="K178" s="32" t="n"/>
-      <c r="L178" s="29" t="n"/>
+      <c r="L178" s="29" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M178" s="32" t="n"/>
       <c r="N178" s="32" t="n"/>
       <c r="O178" s="29" t="n"/>
@@ -13475,7 +13951,11 @@
         </is>
       </c>
       <c r="K179" s="32" t="n"/>
-      <c r="L179" s="29" t="n"/>
+      <c r="L179" s="29" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M179" s="32" t="n"/>
       <c r="N179" s="32" t="n"/>
       <c r="O179" s="29" t="n"/>
@@ -13527,7 +14007,11 @@
         </is>
       </c>
       <c r="K180" s="32" t="n"/>
-      <c r="L180" s="29" t="n"/>
+      <c r="L180" s="29" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M180" s="32" t="n"/>
       <c r="N180" s="32" t="n"/>
       <c r="O180" s="29" t="n"/>
@@ -13667,7 +14151,11 @@
         </is>
       </c>
       <c r="K182" s="32" t="n"/>
-      <c r="L182" s="29" t="n"/>
+      <c r="L182" s="29" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M182" s="32" t="n"/>
       <c r="N182" s="32" t="n"/>
       <c r="O182" s="29" t="n"/>
@@ -13807,7 +14295,11 @@
         </is>
       </c>
       <c r="K184" s="32" t="n"/>
-      <c r="L184" s="29" t="n"/>
+      <c r="L184" s="29" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M184" s="32" t="n"/>
       <c r="N184" s="32" t="n"/>
       <c r="O184" s="29" t="n"/>
@@ -13859,7 +14351,11 @@
         </is>
       </c>
       <c r="K185" s="32" t="n"/>
-      <c r="L185" s="29" t="n"/>
+      <c r="L185" s="29" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M185" s="32" t="n"/>
       <c r="N185" s="32" t="n"/>
       <c r="O185" s="29" t="n"/>
@@ -14336,7 +14832,11 @@
         </is>
       </c>
       <c r="K191" s="32" t="n"/>
-      <c r="L191" s="32" t="n"/>
+      <c r="L191" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M191" s="32" t="n"/>
       <c r="N191" s="32" t="n"/>
       <c r="O191" s="32" t="n"/>
@@ -14389,7 +14889,11 @@
         </is>
       </c>
       <c r="K192" s="32" t="n"/>
-      <c r="L192" s="32" t="n"/>
+      <c r="L192" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M192" s="32" t="n"/>
       <c r="N192" s="32" t="n"/>
       <c r="O192" s="32" t="n"/>
@@ -14441,7 +14945,11 @@
         </is>
       </c>
       <c r="K193" s="32" t="n"/>
-      <c r="L193" s="32" t="n"/>
+      <c r="L193" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M193" s="32" t="n"/>
       <c r="N193" s="32" t="n"/>
       <c r="O193" s="32" t="n"/>
@@ -14493,7 +15001,11 @@
         </is>
       </c>
       <c r="K194" s="32" t="n"/>
-      <c r="L194" s="32" t="n"/>
+      <c r="L194" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M194" s="32" t="n"/>
       <c r="N194" s="32" t="n"/>
       <c r="O194" s="32" t="n"/>
@@ -14545,7 +15057,11 @@
         </is>
       </c>
       <c r="K195" s="32" t="n"/>
-      <c r="L195" s="32" t="n"/>
+      <c r="L195" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M195" s="32" t="n"/>
       <c r="N195" s="32" t="n"/>
       <c r="O195" s="32" t="n"/>
@@ -14597,7 +15113,11 @@
         </is>
       </c>
       <c r="K196" s="32" t="n"/>
-      <c r="L196" s="32" t="n"/>
+      <c r="L196" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M196" s="32" t="n"/>
       <c r="N196" s="32" t="n"/>
       <c r="O196" s="32" t="n"/>
@@ -14649,7 +15169,11 @@
         </is>
       </c>
       <c r="K197" s="32" t="n"/>
-      <c r="L197" s="32" t="n"/>
+      <c r="L197" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M197" s="32" t="n"/>
       <c r="N197" s="32" t="n"/>
       <c r="O197" s="32" t="n"/>
@@ -14701,7 +15225,11 @@
         </is>
       </c>
       <c r="K198" s="32" t="n"/>
-      <c r="L198" s="32" t="n"/>
+      <c r="L198" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M198" s="32" t="n"/>
       <c r="N198" s="32" t="n"/>
       <c r="O198" s="32" t="n"/>
@@ -14753,7 +15281,11 @@
         </is>
       </c>
       <c r="K199" s="32" t="n"/>
-      <c r="L199" s="32" t="n"/>
+      <c r="L199" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M199" s="32" t="n"/>
       <c r="N199" s="32" t="n"/>
       <c r="O199" s="32" t="n"/>
@@ -14805,7 +15337,11 @@
         </is>
       </c>
       <c r="K200" s="32" t="n"/>
-      <c r="L200" s="32" t="n"/>
+      <c r="L200" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M200" s="32" t="n"/>
       <c r="N200" s="32" t="n"/>
       <c r="O200" s="32" t="n"/>
@@ -14857,7 +15393,11 @@
         </is>
       </c>
       <c r="K201" s="32" t="n"/>
-      <c r="L201" s="32" t="n"/>
+      <c r="L201" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M201" s="32" t="n"/>
       <c r="N201" s="32" t="n"/>
       <c r="O201" s="32" t="n"/>
@@ -14909,7 +15449,11 @@
         </is>
       </c>
       <c r="K202" s="32" t="n"/>
-      <c r="L202" s="32" t="n"/>
+      <c r="L202" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M202" s="32" t="n"/>
       <c r="N202" s="32" t="n"/>
       <c r="O202" s="32" t="n"/>
@@ -14961,7 +15505,11 @@
         </is>
       </c>
       <c r="K203" s="32" t="n"/>
-      <c r="L203" s="32" t="n"/>
+      <c r="L203" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M203" s="32" t="n"/>
       <c r="N203" s="32" t="n"/>
       <c r="O203" s="32" t="n"/>
@@ -15016,7 +15564,11 @@
         </is>
       </c>
       <c r="K204" s="32" t="n"/>
-      <c r="L204" s="32" t="n"/>
+      <c r="L204" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M204" s="32" t="n"/>
       <c r="N204" s="32" t="n"/>
       <c r="O204" s="32" t="n"/>
@@ -15068,7 +15620,11 @@
         </is>
       </c>
       <c r="K205" s="32" t="n"/>
-      <c r="L205" s="32" t="n"/>
+      <c r="L205" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M205" s="32" t="n"/>
       <c r="N205" s="32" t="n"/>
       <c r="O205" s="32" t="n"/>
@@ -15124,7 +15680,11 @@
         </is>
       </c>
       <c r="K206" s="32" t="n"/>
-      <c r="L206" s="32" t="n"/>
+      <c r="L206" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M206" s="32" t="n"/>
       <c r="N206" s="32" t="n"/>
       <c r="O206" s="32" t="n"/>
@@ -15176,7 +15736,11 @@
         </is>
       </c>
       <c r="K207" s="32" t="n"/>
-      <c r="L207" s="32" t="n"/>
+      <c r="L207" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M207" s="32" t="n"/>
       <c r="N207" s="32" t="n"/>
       <c r="O207" s="32" t="n"/>
@@ -15228,7 +15792,11 @@
         </is>
       </c>
       <c r="K208" s="32" t="n"/>
-      <c r="L208" s="32" t="n"/>
+      <c r="L208" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M208" s="32" t="n"/>
       <c r="N208" s="32" t="n"/>
       <c r="O208" s="32" t="n"/>
@@ -15280,7 +15848,11 @@
         </is>
       </c>
       <c r="K209" s="32" t="n"/>
-      <c r="L209" s="32" t="n"/>
+      <c r="L209" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M209" s="32" t="n"/>
       <c r="N209" s="32" t="n"/>
       <c r="O209" s="32" t="n"/>
@@ -15332,7 +15904,11 @@
         </is>
       </c>
       <c r="K210" s="32" t="n"/>
-      <c r="L210" s="32" t="n"/>
+      <c r="L210" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M210" s="32" t="n"/>
       <c r="N210" s="32" t="n"/>
       <c r="O210" s="32" t="n"/>
@@ -15384,7 +15960,11 @@
         </is>
       </c>
       <c r="K211" s="32" t="n"/>
-      <c r="L211" s="32" t="n"/>
+      <c r="L211" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M211" s="32" t="n"/>
       <c r="N211" s="32" t="n"/>
       <c r="O211" s="32" t="n"/>
@@ -15436,7 +16016,11 @@
         </is>
       </c>
       <c r="K212" s="32" t="n"/>
-      <c r="L212" s="32" t="n"/>
+      <c r="L212" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M212" s="32" t="n"/>
       <c r="N212" s="32" t="n"/>
       <c r="O212" s="32" t="n"/>
@@ -15488,7 +16072,11 @@
         </is>
       </c>
       <c r="K213" s="32" t="n"/>
-      <c r="L213" s="32" t="n"/>
+      <c r="L213" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M213" s="32" t="n"/>
       <c r="N213" s="32" t="n"/>
       <c r="O213" s="32" t="n"/>
@@ -15540,7 +16128,11 @@
         </is>
       </c>
       <c r="K214" s="32" t="n"/>
-      <c r="L214" s="32" t="n"/>
+      <c r="L214" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M214" s="32" t="n"/>
       <c r="N214" s="32" t="n"/>
       <c r="O214" s="32" t="n"/>
@@ -15592,7 +16184,11 @@
         </is>
       </c>
       <c r="K215" s="32" t="n"/>
-      <c r="L215" s="32" t="n"/>
+      <c r="L215" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M215" s="32" t="n"/>
       <c r="N215" s="32" t="n"/>
       <c r="O215" s="32" t="n"/>
@@ -15644,7 +16240,11 @@
         </is>
       </c>
       <c r="K216" s="32" t="n"/>
-      <c r="L216" s="32" t="n"/>
+      <c r="L216" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M216" s="32" t="n"/>
       <c r="N216" s="32" t="n"/>
       <c r="O216" s="32" t="n"/>
@@ -15696,7 +16296,11 @@
         </is>
       </c>
       <c r="K217" s="32" t="n"/>
-      <c r="L217" s="32" t="n"/>
+      <c r="L217" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M217" s="32" t="n"/>
       <c r="N217" s="32" t="n"/>
       <c r="O217" s="32" t="n"/>
@@ -15748,7 +16352,11 @@
         </is>
       </c>
       <c r="K218" s="32" t="n"/>
-      <c r="L218" s="32" t="n"/>
+      <c r="L218" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M218" s="32" t="n"/>
       <c r="N218" s="32" t="n"/>
       <c r="O218" s="32" t="n"/>
@@ -15803,7 +16411,11 @@
         </is>
       </c>
       <c r="K219" s="32" t="n"/>
-      <c r="L219" s="32" t="n"/>
+      <c r="L219" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M219" s="32" t="n"/>
       <c r="N219" s="32" t="n"/>
       <c r="O219" s="32" t="n"/>
@@ -15855,7 +16467,11 @@
         </is>
       </c>
       <c r="K220" s="32" t="n"/>
-      <c r="L220" s="32" t="n"/>
+      <c r="L220" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M220" s="32" t="n"/>
       <c r="N220" s="32" t="n"/>
       <c r="O220" s="32" t="n"/>
@@ -15911,7 +16527,11 @@
         </is>
       </c>
       <c r="K221" s="32" t="n"/>
-      <c r="L221" s="32" t="n"/>
+      <c r="L221" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M221" s="32" t="n"/>
       <c r="N221" s="32" t="n"/>
       <c r="O221" s="32" t="n"/>
@@ -15963,7 +16583,11 @@
         </is>
       </c>
       <c r="K222" s="32" t="n"/>
-      <c r="L222" s="32" t="n"/>
+      <c r="L222" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M222" s="32" t="n"/>
       <c r="N222" s="32" t="n"/>
       <c r="O222" s="32" t="n"/>
@@ -16015,7 +16639,11 @@
         </is>
       </c>
       <c r="K223" s="32" t="n"/>
-      <c r="L223" s="32" t="n"/>
+      <c r="L223" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M223" s="32" t="n"/>
       <c r="N223" s="32" t="n"/>
       <c r="O223" s="32" t="n"/>
@@ -16067,7 +16695,11 @@
         </is>
       </c>
       <c r="K224" s="32" t="n"/>
-      <c r="L224" s="32" t="n"/>
+      <c r="L224" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M224" s="32" t="n"/>
       <c r="N224" s="32" t="n"/>
       <c r="O224" s="32" t="n"/>
@@ -16119,7 +16751,11 @@
         </is>
       </c>
       <c r="K225" s="32" t="n"/>
-      <c r="L225" s="32" t="n"/>
+      <c r="L225" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M225" s="32" t="n"/>
       <c r="N225" s="32" t="n"/>
       <c r="O225" s="32" t="n"/>
@@ -16171,7 +16807,11 @@
         </is>
       </c>
       <c r="K226" s="32" t="n"/>
-      <c r="L226" s="32" t="n"/>
+      <c r="L226" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M226" s="32" t="n"/>
       <c r="N226" s="32" t="n"/>
       <c r="O226" s="32" t="n"/>
@@ -16223,7 +16863,11 @@
         </is>
       </c>
       <c r="K227" s="32" t="n"/>
-      <c r="L227" s="32" t="n"/>
+      <c r="L227" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M227" s="32" t="n"/>
       <c r="N227" s="32" t="n"/>
       <c r="O227" s="32" t="n"/>
@@ -16275,7 +16919,11 @@
         </is>
       </c>
       <c r="K228" s="32" t="n"/>
-      <c r="L228" s="32" t="n"/>
+      <c r="L228" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M228" s="32" t="n"/>
       <c r="N228" s="32" t="n"/>
       <c r="O228" s="32" t="n"/>
@@ -16327,7 +16975,11 @@
         </is>
       </c>
       <c r="K229" s="32" t="n"/>
-      <c r="L229" s="32" t="n"/>
+      <c r="L229" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M229" s="32" t="n"/>
       <c r="N229" s="32" t="n"/>
       <c r="O229" s="32" t="n"/>
@@ -16379,7 +17031,11 @@
         </is>
       </c>
       <c r="K230" s="32" t="n"/>
-      <c r="L230" s="32" t="n"/>
+      <c r="L230" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M230" s="32" t="n"/>
       <c r="N230" s="32" t="n"/>
       <c r="O230" s="32" t="n"/>
@@ -16431,7 +17087,11 @@
         </is>
       </c>
       <c r="K231" s="32" t="n"/>
-      <c r="L231" s="32" t="n"/>
+      <c r="L231" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M231" s="32" t="n"/>
       <c r="N231" s="32" t="n"/>
       <c r="O231" s="32" t="n"/>
@@ -16483,7 +17143,11 @@
         </is>
       </c>
       <c r="K232" s="32" t="n"/>
-      <c r="L232" s="32" t="n"/>
+      <c r="L232" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M232" s="32" t="n"/>
       <c r="N232" s="32" t="n"/>
       <c r="O232" s="32" t="n"/>
@@ -16535,7 +17199,11 @@
         </is>
       </c>
       <c r="K233" s="32" t="n"/>
-      <c r="L233" s="32" t="n"/>
+      <c r="L233" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M233" s="32" t="n"/>
       <c r="N233" s="32" t="n"/>
       <c r="O233" s="32" t="n"/>
@@ -16590,7 +17258,11 @@
         </is>
       </c>
       <c r="K234" s="32" t="n"/>
-      <c r="L234" s="32" t="n"/>
+      <c r="L234" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M234" s="32" t="n"/>
       <c r="N234" s="32" t="n"/>
       <c r="O234" s="32" t="n"/>
@@ -16642,7 +17314,11 @@
         </is>
       </c>
       <c r="K235" s="32" t="n"/>
-      <c r="L235" s="32" t="n"/>
+      <c r="L235" s="32" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M235" s="32" t="n"/>
       <c r="N235" s="32" t="n"/>
       <c r="O235" s="32" t="n"/>
@@ -16698,7 +17374,11 @@
         </is>
       </c>
       <c r="K236" s="66" t="n"/>
-      <c r="L236" s="66" t="n"/>
+      <c r="L236" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M236" s="66" t="n"/>
       <c r="N236" s="66" t="n"/>
       <c r="O236" s="66" t="n"/>
@@ -16750,7 +17430,11 @@
         </is>
       </c>
       <c r="K237" s="66" t="n"/>
-      <c r="L237" s="66" t="n"/>
+      <c r="L237" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M237" s="66" t="n"/>
       <c r="N237" s="66" t="n"/>
       <c r="O237" s="66" t="n"/>
@@ -16802,7 +17486,11 @@
         </is>
       </c>
       <c r="K238" s="66" t="n"/>
-      <c r="L238" s="66" t="n"/>
+      <c r="L238" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M238" s="66" t="n"/>
       <c r="N238" s="66" t="n"/>
       <c r="O238" s="66" t="n"/>
@@ -16854,7 +17542,11 @@
         </is>
       </c>
       <c r="K239" s="66" t="n"/>
-      <c r="L239" s="66" t="n"/>
+      <c r="L239" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M239" s="66" t="n"/>
       <c r="N239" s="66" t="n"/>
       <c r="O239" s="66" t="n"/>
@@ -16906,7 +17598,11 @@
         </is>
       </c>
       <c r="K240" s="66" t="n"/>
-      <c r="L240" s="66" t="n"/>
+      <c r="L240" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M240" s="66" t="n"/>
       <c r="N240" s="66" t="n"/>
       <c r="O240" s="66" t="n"/>
@@ -16958,7 +17654,11 @@
         </is>
       </c>
       <c r="K241" s="66" t="n"/>
-      <c r="L241" s="66" t="n"/>
+      <c r="L241" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M241" s="66" t="n"/>
       <c r="N241" s="66" t="n"/>
       <c r="O241" s="66" t="n"/>
@@ -17010,7 +17710,11 @@
         </is>
       </c>
       <c r="K242" s="66" t="n"/>
-      <c r="L242" s="66" t="n"/>
+      <c r="L242" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M242" s="66" t="n"/>
       <c r="N242" s="66" t="n"/>
       <c r="O242" s="66" t="n"/>
@@ -17062,7 +17766,11 @@
         </is>
       </c>
       <c r="K243" s="66" t="n"/>
-      <c r="L243" s="66" t="n"/>
+      <c r="L243" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M243" s="66" t="n"/>
       <c r="N243" s="66" t="n"/>
       <c r="O243" s="66" t="n"/>
@@ -17117,7 +17825,11 @@
         </is>
       </c>
       <c r="K244" s="66" t="n"/>
-      <c r="L244" s="66" t="n"/>
+      <c r="L244" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M244" s="66" t="n"/>
       <c r="N244" s="66" t="n"/>
       <c r="O244" s="66" t="n"/>
@@ -17169,7 +17881,11 @@
         </is>
       </c>
       <c r="K245" s="66" t="n"/>
-      <c r="L245" s="66" t="n"/>
+      <c r="L245" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M245" s="66" t="n"/>
       <c r="N245" s="66" t="n"/>
       <c r="O245" s="66" t="n"/>
@@ -17225,7 +17941,11 @@
         </is>
       </c>
       <c r="K246" s="66" t="n"/>
-      <c r="L246" s="66" t="n"/>
+      <c r="L246" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M246" s="66" t="n"/>
       <c r="N246" s="66" t="n"/>
       <c r="O246" s="66" t="n"/>
@@ -17277,7 +17997,11 @@
         </is>
       </c>
       <c r="K247" s="66" t="n"/>
-      <c r="L247" s="66" t="n"/>
+      <c r="L247" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M247" s="66" t="n"/>
       <c r="N247" s="66" t="n"/>
       <c r="O247" s="66" t="n"/>
@@ -17329,7 +18053,11 @@
         </is>
       </c>
       <c r="K248" s="66" t="n"/>
-      <c r="L248" s="66" t="n"/>
+      <c r="L248" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M248" s="66" t="n"/>
       <c r="N248" s="66" t="n"/>
       <c r="O248" s="66" t="n"/>
@@ -17381,7 +18109,11 @@
         </is>
       </c>
       <c r="K249" s="66" t="n"/>
-      <c r="L249" s="66" t="n"/>
+      <c r="L249" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M249" s="66" t="n"/>
       <c r="N249" s="66" t="n"/>
       <c r="O249" s="66" t="n"/>
@@ -17433,7 +18165,11 @@
         </is>
       </c>
       <c r="K250" s="66" t="n"/>
-      <c r="L250" s="66" t="n"/>
+      <c r="L250" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M250" s="66" t="n"/>
       <c r="N250" s="66" t="n"/>
       <c r="O250" s="66" t="n"/>
@@ -17485,7 +18221,11 @@
         </is>
       </c>
       <c r="K251" s="66" t="n"/>
-      <c r="L251" s="66" t="n"/>
+      <c r="L251" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M251" s="66" t="n"/>
       <c r="N251" s="66" t="n"/>
       <c r="O251" s="66" t="n"/>
@@ -17537,7 +18277,11 @@
         </is>
       </c>
       <c r="K252" s="66" t="n"/>
-      <c r="L252" s="66" t="n"/>
+      <c r="L252" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M252" s="66" t="n"/>
       <c r="N252" s="66" t="n"/>
       <c r="O252" s="66" t="n"/>
@@ -17589,7 +18333,11 @@
         </is>
       </c>
       <c r="K253" s="66" t="n"/>
-      <c r="L253" s="66" t="n"/>
+      <c r="L253" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M253" s="66" t="n"/>
       <c r="N253" s="66" t="n"/>
       <c r="O253" s="66" t="n"/>
@@ -17641,7 +18389,11 @@
         </is>
       </c>
       <c r="K254" s="66" t="n"/>
-      <c r="L254" s="66" t="n"/>
+      <c r="L254" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M254" s="66" t="n"/>
       <c r="N254" s="66" t="n"/>
       <c r="O254" s="66" t="n"/>
@@ -17693,7 +18445,11 @@
         </is>
       </c>
       <c r="K255" s="66" t="n"/>
-      <c r="L255" s="66" t="n"/>
+      <c r="L255" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M255" s="66" t="n"/>
       <c r="N255" s="66" t="n"/>
       <c r="O255" s="66" t="n"/>
@@ -17745,7 +18501,11 @@
         </is>
       </c>
       <c r="K256" s="66" t="n"/>
-      <c r="L256" s="66" t="n"/>
+      <c r="L256" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M256" s="66" t="n"/>
       <c r="N256" s="66" t="n"/>
       <c r="O256" s="66" t="n"/>
@@ -17797,7 +18557,11 @@
         </is>
       </c>
       <c r="K257" s="66" t="n"/>
-      <c r="L257" s="66" t="n"/>
+      <c r="L257" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M257" s="66" t="n"/>
       <c r="N257" s="66" t="n"/>
       <c r="O257" s="66" t="n"/>
@@ -17849,7 +18613,11 @@
         </is>
       </c>
       <c r="K258" s="66" t="n"/>
-      <c r="L258" s="66" t="n"/>
+      <c r="L258" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M258" s="66" t="n"/>
       <c r="N258" s="66" t="n"/>
       <c r="O258" s="66" t="n"/>
@@ -17901,7 +18669,11 @@
         </is>
       </c>
       <c r="K259" s="66" t="n"/>
-      <c r="L259" s="66" t="n"/>
+      <c r="L259" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M259" s="66" t="n"/>
       <c r="N259" s="66" t="n"/>
       <c r="O259" s="66" t="n"/>
@@ -17953,7 +18725,11 @@
         </is>
       </c>
       <c r="K260" s="66" t="n"/>
-      <c r="L260" s="66" t="n"/>
+      <c r="L260" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M260" s="66" t="n"/>
       <c r="N260" s="66" t="n"/>
       <c r="O260" s="66" t="n"/>
@@ -18005,7 +18781,11 @@
         </is>
       </c>
       <c r="K261" s="66" t="n"/>
-      <c r="L261" s="66" t="n"/>
+      <c r="L261" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M261" s="66" t="n"/>
       <c r="N261" s="66" t="n"/>
       <c r="O261" s="66" t="n"/>
@@ -18057,7 +18837,11 @@
         </is>
       </c>
       <c r="K262" s="66" t="n"/>
-      <c r="L262" s="66" t="n"/>
+      <c r="L262" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M262" s="66" t="n"/>
       <c r="N262" s="66" t="n"/>
       <c r="O262" s="66" t="n"/>
@@ -18109,7 +18893,11 @@
         </is>
       </c>
       <c r="K263" s="66" t="n"/>
-      <c r="L263" s="66" t="n"/>
+      <c r="L263" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M263" s="66" t="n"/>
       <c r="N263" s="66" t="n"/>
       <c r="O263" s="66" t="n"/>
@@ -18164,7 +18952,11 @@
         </is>
       </c>
       <c r="K264" s="66" t="n"/>
-      <c r="L264" s="66" t="n"/>
+      <c r="L264" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M264" s="66" t="n"/>
       <c r="N264" s="66" t="n"/>
       <c r="O264" s="66" t="n"/>
@@ -18216,7 +19008,11 @@
         </is>
       </c>
       <c r="K265" s="66" t="n"/>
-      <c r="L265" s="66" t="n"/>
+      <c r="L265" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M265" s="66" t="n"/>
       <c r="N265" s="66" t="n"/>
       <c r="O265" s="66" t="n"/>
@@ -18272,7 +19068,11 @@
         </is>
       </c>
       <c r="K266" s="66" t="n"/>
-      <c r="L266" s="66" t="n"/>
+      <c r="L266" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M266" s="66" t="n"/>
       <c r="N266" s="66" t="n"/>
       <c r="O266" s="66" t="n"/>
@@ -18324,7 +19124,11 @@
         </is>
       </c>
       <c r="K267" s="66" t="n"/>
-      <c r="L267" s="66" t="n"/>
+      <c r="L267" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M267" s="66" t="n"/>
       <c r="N267" s="66" t="n"/>
       <c r="O267" s="66" t="n"/>
@@ -18376,7 +19180,11 @@
         </is>
       </c>
       <c r="K268" s="66" t="n"/>
-      <c r="L268" s="66" t="n"/>
+      <c r="L268" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M268" s="66" t="n"/>
       <c r="N268" s="66" t="n"/>
       <c r="O268" s="66" t="n"/>
@@ -18428,7 +19236,11 @@
         </is>
       </c>
       <c r="K269" s="66" t="n"/>
-      <c r="L269" s="66" t="n"/>
+      <c r="L269" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M269" s="66" t="n"/>
       <c r="N269" s="66" t="n"/>
       <c r="O269" s="66" t="n"/>
@@ -18480,7 +19292,11 @@
         </is>
       </c>
       <c r="K270" s="66" t="n"/>
-      <c r="L270" s="66" t="n"/>
+      <c r="L270" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M270" s="66" t="n"/>
       <c r="N270" s="66" t="n"/>
       <c r="O270" s="66" t="n"/>
@@ -18532,7 +19348,11 @@
         </is>
       </c>
       <c r="K271" s="66" t="n"/>
-      <c r="L271" s="66" t="n"/>
+      <c r="L271" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M271" s="66" t="n"/>
       <c r="N271" s="66" t="n"/>
       <c r="O271" s="66" t="n"/>
@@ -18584,7 +19404,11 @@
         </is>
       </c>
       <c r="K272" s="66" t="n"/>
-      <c r="L272" s="66" t="n"/>
+      <c r="L272" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M272" s="66" t="n"/>
       <c r="N272" s="66" t="n"/>
       <c r="O272" s="66" t="n"/>
@@ -18636,7 +19460,11 @@
         </is>
       </c>
       <c r="K273" s="66" t="n"/>
-      <c r="L273" s="66" t="n"/>
+      <c r="L273" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M273" s="66" t="n"/>
       <c r="N273" s="66" t="n"/>
       <c r="O273" s="66" t="n"/>
@@ -18688,7 +19516,11 @@
         </is>
       </c>
       <c r="K274" s="66" t="n"/>
-      <c r="L274" s="66" t="n"/>
+      <c r="L274" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M274" s="66" t="n"/>
       <c r="N274" s="66" t="n"/>
       <c r="O274" s="66" t="n"/>
@@ -18740,7 +19572,11 @@
         </is>
       </c>
       <c r="K275" s="66" t="n"/>
-      <c r="L275" s="66" t="n"/>
+      <c r="L275" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M275" s="66" t="n"/>
       <c r="N275" s="66" t="n"/>
       <c r="O275" s="66" t="n"/>
@@ -18792,7 +19628,11 @@
         </is>
       </c>
       <c r="K276" s="66" t="n"/>
-      <c r="L276" s="66" t="n"/>
+      <c r="L276" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M276" s="66" t="n"/>
       <c r="N276" s="66" t="n"/>
       <c r="O276" s="66" t="n"/>
@@ -18844,7 +19684,11 @@
         </is>
       </c>
       <c r="K277" s="66" t="n"/>
-      <c r="L277" s="66" t="n"/>
+      <c r="L277" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M277" s="66" t="n"/>
       <c r="N277" s="66" t="n"/>
       <c r="O277" s="66" t="n"/>
@@ -18896,7 +19740,11 @@
         </is>
       </c>
       <c r="K278" s="66" t="n"/>
-      <c r="L278" s="66" t="n"/>
+      <c r="L278" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M278" s="66" t="n"/>
       <c r="N278" s="66" t="n"/>
       <c r="O278" s="66" t="n"/>
@@ -18948,7 +19796,11 @@
         </is>
       </c>
       <c r="K279" s="66" t="n"/>
-      <c r="L279" s="66" t="n"/>
+      <c r="L279" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M279" s="66" t="n"/>
       <c r="N279" s="66" t="n"/>
       <c r="O279" s="66" t="n"/>
@@ -19000,7 +19852,11 @@
         </is>
       </c>
       <c r="K280" s="66" t="n"/>
-      <c r="L280" s="66" t="n"/>
+      <c r="L280" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M280" s="66" t="n"/>
       <c r="N280" s="66" t="n"/>
       <c r="O280" s="66" t="n"/>
@@ -19052,7 +19908,11 @@
         </is>
       </c>
       <c r="K281" s="66" t="n"/>
-      <c r="L281" s="66" t="n"/>
+      <c r="L281" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M281" s="66" t="n"/>
       <c r="N281" s="66" t="n"/>
       <c r="O281" s="66" t="n"/>
@@ -19104,7 +19964,11 @@
         </is>
       </c>
       <c r="K282" s="66" t="n"/>
-      <c r="L282" s="66" t="n"/>
+      <c r="L282" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M282" s="66" t="n"/>
       <c r="N282" s="66" t="n"/>
       <c r="O282" s="66" t="n"/>
@@ -19156,7 +20020,11 @@
         </is>
       </c>
       <c r="K283" s="66" t="n"/>
-      <c r="L283" s="66" t="n"/>
+      <c r="L283" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M283" s="66" t="n"/>
       <c r="N283" s="66" t="n"/>
       <c r="O283" s="66" t="n"/>
@@ -19211,7 +20079,11 @@
         </is>
       </c>
       <c r="K284" s="66" t="n"/>
-      <c r="L284" s="66" t="n"/>
+      <c r="L284" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M284" s="66" t="n"/>
       <c r="N284" s="66" t="n"/>
       <c r="O284" s="66" t="n"/>
@@ -19263,7 +20135,11 @@
         </is>
       </c>
       <c r="K285" s="66" t="n"/>
-      <c r="L285" s="66" t="n"/>
+      <c r="L285" s="66" t="inlineStr">
+        <is>
+          <t>Tipologia documentale non gestita dall'applicativo nella versione corrente</t>
+        </is>
+      </c>
       <c r="M285" s="66" t="n"/>
       <c r="N285" s="66" t="n"/>
       <c r="O285" s="66" t="n"/>

</xml_diff>

<commit_message>
REBUILD report-checklist.xlsx from scratch: SI=all fields, NO=only J+K
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#CENTROPOLISPECIALISTICOGIOVANNIPAOLOIXX/GPI_HEALTH_SYSTEM/FSE_SENDER/V.1.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#CENTROPOLISPECIALISTICOGIOVANNIPAOLOIXX/GPI_HEALTH_SYSTEM/FSE_SENDER/V.1.0/report-checklist.xlsx
@@ -2697,7 +2697,7 @@
       </c>
       <c r="G10" s="30" t="inlineStr">
         <is>
-          <t>2026-03-26T08:16:15</t>
+          <t>2026-03-26T08:16:15Z</t>
         </is>
       </c>
       <c r="H10" s="30" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="S11" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T11" s="32" t="inlineStr">
@@ -3073,7 +3073,7 @@
       </c>
       <c r="S14" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T14" s="32" t="inlineStr">
@@ -3176,7 +3176,7 @@
       </c>
       <c r="S15" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T15" s="32" t="inlineStr">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="S19" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T19" s="32" t="inlineStr">
@@ -3677,7 +3677,7 @@
       </c>
       <c r="S22" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T22" s="32" t="inlineStr">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="S23" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T23" s="32" t="inlineStr">
@@ -4057,7 +4057,7 @@
       </c>
       <c r="S27" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T27" s="32" t="inlineStr">
@@ -4102,26 +4102,10 @@
 "ERRORE BLOCCANTE (SI/NO)", "ERRORE VISIBILE A UTENTE (SI/NO)", "MESSAGGIO DI ERRORE", "GESTITO IN BACKOFFICE (SI/NO)", " PRESENTE CODA DI RETRY AUTOMATICA PER L'INVIO DEL DOCUMENTO AL FSE SERVIZIO DI VALIDAZIONE DEL GATEWAY A SEGUITO DELLA RISOLUZIONE DELL'ERRORE (SI/NO)",  "INVIO MANUALE DEL DOCUMENTO AL FSE A SEGUITO DELLA RISOLUZIONE DELL'ERRORE (SI/NO)", "GESTIONE ERRORE".</t>
         </is>
       </c>
-      <c r="F28" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G28" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:15</t>
-        </is>
-      </c>
-      <c r="H28" s="31" t="inlineStr">
-        <is>
-          <t>ff55db762ded2539affd730de18bd8c1</t>
-        </is>
-      </c>
-      <c r="I28" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.8b4e07e56d5aa565f9a8de121321d2d8eb791aefc994d88859d9672a4b396b04.66e074ff48^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F28" s="31" t="n"/>
+      <c r="G28" s="31" t="n"/>
+      <c r="H28" s="31" t="n"/>
+      <c r="I28" s="36" t="n"/>
       <c r="J28" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -4133,46 +4117,14 @@
         </is>
       </c>
       <c r="L28" s="32" t="n"/>
-      <c r="M28" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N28" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O28" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P28" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q28" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R28" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S28" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T28" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M28" s="32" t="n"/>
+      <c r="N28" s="32" t="n"/>
+      <c r="O28" s="32" t="n"/>
+      <c r="P28" s="32" t="n"/>
+      <c r="Q28" s="32" t="n"/>
+      <c r="R28" s="32" t="n"/>
+      <c r="S28" s="32" t="n"/>
+      <c r="T28" s="32" t="n"/>
       <c r="U28" s="33" t="inlineStr">
         <is>
           <t>SI</t>
@@ -4329,7 +4281,7 @@
       </c>
       <c r="S30" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T30" s="32" t="inlineStr">
@@ -4381,17 +4333,17 @@
       </c>
       <c r="G31" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:17:47</t>
+          <t>2026-03-26T08:16:49Z</t>
         </is>
       </c>
       <c r="H31" s="31" t="inlineStr">
         <is>
-          <t>346c86394d9e19688c98e1eac3507b73</t>
+          <t>acaaee0bef9df190c95a8e1922b13422</t>
         </is>
       </c>
       <c r="I31" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.2081e93bc59b43e49e3aeae958e60c84dccb7d9ecdcb4e330174098f046ce5f1.617e1f2a25^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.803c6bbaf321647710ce6fe3fe1c2d532c81a9bca2ce4bf6a38b58bfd7f39a94.591366733d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J31" s="32" t="inlineStr">
@@ -4433,7 +4385,7 @@
       </c>
       <c r="S31" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T31" s="32" t="inlineStr">
@@ -4478,26 +4430,10 @@
 "ERRORE BLOCCANTE (SI/NO)", "ERRORE VISIBILE A UTENTE (SI/NO)", "MESSAGGIO DI ERRORE", "GESTITO IN BACKOFFICE (SI/NO)", " PRESENTE CODA DI RETRY AUTOMATICA PER L'INVIO DEL DOCUMENTO AL FSE SERVIZIO DI VALIDAZIONE DEL GATEWAY A SEGUITO DELLA RISOLUZIONE DELL'ERRORE (SI/NO)",  "INVIO MANUALE DEL DOCUMENTO AL FSE A SEGUITO DELLA RISOLUZIONE DELL'ERRORE (SI/NO)", "GESTIONE ERRORE".</t>
         </is>
       </c>
-      <c r="F32" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G32" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:52</t>
-        </is>
-      </c>
-      <c r="H32" s="31" t="inlineStr">
-        <is>
-          <t>a0cb1ce26dd8782352e5f05ddef141a2</t>
-        </is>
-      </c>
-      <c r="I32" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.b9a0ee4080bbd8e3616f9fe9ac6ae4e7be45391a9498d7b89ee4c3483892a723.da957b601c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F32" s="31" t="n"/>
+      <c r="G32" s="31" t="n"/>
+      <c r="H32" s="31" t="n"/>
+      <c r="I32" s="36" t="n"/>
       <c r="J32" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -4509,46 +4445,14 @@
         </is>
       </c>
       <c r="L32" s="32" t="n"/>
-      <c r="M32" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N32" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O32" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P32" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q32" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R32" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S32" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T32" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M32" s="32" t="n"/>
+      <c r="N32" s="32" t="n"/>
+      <c r="O32" s="32" t="n"/>
+      <c r="P32" s="32" t="n"/>
+      <c r="Q32" s="32" t="n"/>
+      <c r="R32" s="32" t="n"/>
+      <c r="S32" s="32" t="n"/>
+      <c r="T32" s="32" t="n"/>
       <c r="U32" s="33" t="inlineStr">
         <is>
           <t>SI</t>
@@ -4765,7 +4669,7 @@
       </c>
       <c r="S35" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T35" s="32" t="inlineStr">
@@ -4813,17 +4717,17 @@
       </c>
       <c r="G36" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:16:12</t>
+          <t>2026-03-26T08:16:01Z</t>
         </is>
       </c>
       <c r="H36" s="31" t="inlineStr">
         <is>
-          <t>e7b184d9004b721d45058522970f3cb8</t>
+          <t>ca18186dadcd003ef0c803bb91f4c326</t>
         </is>
       </c>
       <c r="I36" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.c7cfc54dcfac0c48c09bb8cfef8f6d91bce2ddc0f8c56e438d3312b3358a249c.8538eae2a6^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.f94e51ce9a72f7518ddba2a331e883662f8907b2e4f2643bff4649fc6c9bf7ed.0bb6fe99bd^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J36" s="32" t="inlineStr">
@@ -4865,7 +4769,7 @@
       </c>
       <c r="S36" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T36" s="32" t="inlineStr">
@@ -4965,7 +4869,7 @@
       </c>
       <c r="S37" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T37" s="32" t="inlineStr">
@@ -5065,7 +4969,7 @@
       </c>
       <c r="S38" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T38" s="32" t="inlineStr">
@@ -5113,17 +5017,17 @@
       </c>
       <c r="G39" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:17:46</t>
+          <t>2026-03-26T08:15:54Z</t>
         </is>
       </c>
       <c r="H39" s="31" t="inlineStr">
         <is>
-          <t>2004061566587dcf572a534701ee0c4f</t>
+          <t>83be47000336cf4ba1b3d8240a0badf6</t>
         </is>
       </c>
       <c r="I39" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.7e4bd7df0b7fcc4937fd1dc164c43f55889e4f64f91ecac8c9cdfdae45fa3124.e84aabc8d7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.4f60e06ab03c9f311d0ec24434ea697c0f9df2782d332783d62b32bb2bd349b8.1400a76f92^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J39" s="32" t="inlineStr">
@@ -5165,7 +5069,7 @@
       </c>
       <c r="S39" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T39" s="32" t="inlineStr">
@@ -5213,17 +5117,17 @@
       </c>
       <c r="G40" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:16:51</t>
+          <t>2026-03-26T08:15:52Z</t>
         </is>
       </c>
       <c r="H40" s="31" t="inlineStr">
         <is>
-          <t>db39cac5c8c5804640e75bea38bc7b37</t>
+          <t>cc88836949681b485e0a0c38292085a7</t>
         </is>
       </c>
       <c r="I40" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.fc1f4ad5ea95e6f48b902f5fe383ae99a3da61a65f0dc53830b78929479ddd3d.3786d8ab7b^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.9a4f23bce9d012d6fe3a5706b36a6f89ff750a338b0d9b7edb9637bef6322231.186ff9eabc^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J40" s="32" t="inlineStr">
@@ -5265,7 +5169,7 @@
       </c>
       <c r="S40" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T40" s="32" t="inlineStr">
@@ -5365,7 +5269,7 @@
       </c>
       <c r="S41" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T41" s="32" t="inlineStr">
@@ -5465,7 +5369,7 @@
       </c>
       <c r="S42" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T42" s="32" t="inlineStr">
@@ -6073,17 +5977,17 @@
       </c>
       <c r="G53" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:16:09</t>
+          <t>2026-03-26T08:17:43Z</t>
         </is>
       </c>
       <c r="H53" s="31" t="inlineStr">
         <is>
-          <t>50a2d5255994760191912f3e5db901b8</t>
+          <t>77463446540f43c6179cc98cf7f0b851</t>
         </is>
       </c>
       <c r="I53" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.01e6e0d273b0aa21e7077088a79700b63f4d4f56bfc125549fb332b77f1f5ac6.5592d64822^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.2f6508dfdd49f71b50664009a32ce80f6a0ce57561a1bea5f7b8480d6d60ceed.ce1b23c9d3^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J53" s="32" t="inlineStr">
@@ -6125,7 +6029,7 @@
       </c>
       <c r="S53" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T53" s="32" t="inlineStr">
@@ -6225,7 +6129,7 @@
       </c>
       <c r="S54" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T54" s="32" t="inlineStr">
@@ -6273,17 +6177,17 @@
       </c>
       <c r="G55" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:16:05</t>
+          <t>2026-03-26T08:17:40Z</t>
         </is>
       </c>
       <c r="H55" s="31" t="inlineStr">
         <is>
-          <t>39bf5a23f89affe2c2caf41ee117af53</t>
+          <t>e390e20d4a4f215bdafcf2c05b9d7086</t>
         </is>
       </c>
       <c r="I55" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.c1d6cf78d1042e56a6418170d49febb3ea72c59e997f9e70e184e877b391aade.508fd7c970^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.11c39bdc287d6498094ef3994468020daeb19d6411e283977d3ba4762f9d76e0.61605fdded^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J55" s="32" t="inlineStr">
@@ -6325,7 +6229,7 @@
       </c>
       <c r="S55" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T55" s="32" t="inlineStr">
@@ -6373,17 +6277,17 @@
       </c>
       <c r="G56" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:16:03</t>
+          <t>2026-03-26T08:17:38Z</t>
         </is>
       </c>
       <c r="H56" s="31" t="inlineStr">
         <is>
-          <t>4f81a52a074de362116fe5b83bd88d1c</t>
+          <t>4ac4b40c10866efb5f4a7c029a9513b7</t>
         </is>
       </c>
       <c r="I56" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.1d1e8bfe895a15711fddad4b7bd2dcaa7a03f0afcd46bcb80715cab089b72de1.4e1ce9c542^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.1fba18e124d4d2a456f0e44e8c8e5d2ec9d8079f22b91464c7f6591fd5947240.5396d18ce7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J56" s="32" t="inlineStr">
@@ -6425,7 +6329,7 @@
       </c>
       <c r="S56" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T56" s="32" t="inlineStr">
@@ -6473,17 +6377,17 @@
       </c>
       <c r="G57" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:16:15</t>
+          <t>2026-03-26T08:17:37Z</t>
         </is>
       </c>
       <c r="H57" s="31" t="inlineStr">
         <is>
-          <t>ff55db762ded2539affd730de18bd8c1</t>
+          <t>c950f2759ad837e425a39a928c24642f</t>
         </is>
       </c>
       <c r="I57" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.8b4e07e56d5aa565f9a8de121321d2d8eb791aefc994d88859d9672a4b396b04.66e074ff48^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.5fd589e19be7e51245b7ace3fcfa501077a8c5d5d1c5b104b8ddd55f36997418.0ef63f0f37^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J57" s="32" t="inlineStr">
@@ -6525,7 +6429,7 @@
       </c>
       <c r="S57" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T57" s="32" t="inlineStr">
@@ -6625,7 +6529,7 @@
       </c>
       <c r="S58" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T58" s="32" t="inlineStr">
@@ -6673,17 +6577,17 @@
       </c>
       <c r="G59" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:16:12</t>
+          <t>2026-03-26T08:17:34Z</t>
         </is>
       </c>
       <c r="H59" s="31" t="inlineStr">
         <is>
-          <t>e7b184d9004b721d45058522970f3cb8</t>
+          <t>095a62f9f67312f5b0e024ebf5abef81</t>
         </is>
       </c>
       <c r="I59" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.c7cfc54dcfac0c48c09bb8cfef8f6d91bce2ddc0f8c56e438d3312b3358a249c.8538eae2a6^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.d318d84c6020ae66a7d87cbb6ef857855c927ce63049b7f0ddf4077115dc1109.b51bf468f8^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J59" s="32" t="inlineStr">
@@ -6725,7 +6629,7 @@
       </c>
       <c r="S59" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T59" s="32" t="inlineStr">
@@ -6773,17 +6677,17 @@
       </c>
       <c r="G60" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:16:09</t>
+          <t>2026-03-26T08:17:47Z</t>
         </is>
       </c>
       <c r="H60" s="31" t="inlineStr">
         <is>
-          <t>50a2d5255994760191912f3e5db901b8</t>
+          <t>346c86394d9e19688c98e1eac3507b73</t>
         </is>
       </c>
       <c r="I60" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.01e6e0d273b0aa21e7077088a79700b63f4d4f56bfc125549fb332b77f1f5ac6.5592d64822^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.2081e93bc59b43e49e3aeae958e60c84dccb7d9ecdcb4e330174098f046ce5f1.617e1f2a25^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J60" s="32" t="inlineStr">
@@ -6825,7 +6729,7 @@
       </c>
       <c r="S60" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T60" s="32" t="inlineStr">
@@ -6873,17 +6777,17 @@
       </c>
       <c r="G61" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:16:05</t>
+          <t>2026-03-26T08:17:46Z</t>
         </is>
       </c>
       <c r="H61" s="31" t="inlineStr">
         <is>
-          <t>39bf5a23f89affe2c2caf41ee117af53</t>
+          <t>2004061566587dcf572a534701ee0c4f</t>
         </is>
       </c>
       <c r="I61" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.c1d6cf78d1042e56a6418170d49febb3ea72c59e997f9e70e184e877b391aade.508fd7c970^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.7e4bd7df0b7fcc4937fd1dc164c43f55889e4f64f91ecac8c9cdfdae45fa3124.e84aabc8d7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J61" s="32" t="inlineStr">
@@ -6925,7 +6829,7 @@
       </c>
       <c r="S61" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T61" s="32" t="inlineStr">
@@ -6973,17 +6877,17 @@
       </c>
       <c r="G62" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:16:03</t>
+          <t>2026-03-26T08:17:44Z</t>
         </is>
       </c>
       <c r="H62" s="31" t="inlineStr">
         <is>
-          <t>4f81a52a074de362116fe5b83bd88d1c</t>
+          <t>1934186e7e728b4f72aa8b556f9e9efd</t>
         </is>
       </c>
       <c r="I62" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.1d1e8bfe895a15711fddad4b7bd2dcaa7a03f0afcd46bcb80715cab089b72de1.4e1ce9c542^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.0fde0276e8077f4bef24425cac8abdeb6c34b904cde51bb985f1aa2ac04ca359.90a459ae96^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J62" s="32" t="inlineStr">
@@ -7025,7 +6929,7 @@
       </c>
       <c r="S62" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T62" s="32" t="inlineStr">
@@ -7125,7 +7029,7 @@
       </c>
       <c r="S63" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T63" s="32" t="inlineStr">
@@ -7225,7 +7129,7 @@
       </c>
       <c r="S64" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T64" s="32" t="inlineStr">
@@ -7325,7 +7229,7 @@
       </c>
       <c r="S65" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T65" s="32" t="inlineStr">
@@ -7425,7 +7329,7 @@
       </c>
       <c r="S66" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T66" s="32" t="inlineStr">
@@ -7525,7 +7429,7 @@
       </c>
       <c r="S67" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T67" s="32" t="inlineStr">
@@ -7625,7 +7529,7 @@
       </c>
       <c r="S68" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T68" s="32" t="inlineStr">
@@ -8058,26 +7962,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 14" riportata nei documenti "casi di test CERT_VACC" e "CDA2_Certificato Vaccinale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F76" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G76" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:17:44</t>
-        </is>
-      </c>
-      <c r="H76" s="31" t="inlineStr">
-        <is>
-          <t>1934186e7e728b4f72aa8b556f9e9efd</t>
-        </is>
-      </c>
-      <c r="I76" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.0fde0276e8077f4bef24425cac8abdeb6c34b904cde51bb985f1aa2ac04ca359.90a459ae96^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F76" s="31" t="n"/>
+      <c r="G76" s="31" t="n"/>
+      <c r="H76" s="31" t="n"/>
+      <c r="I76" s="36" t="n"/>
       <c r="J76" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -8089,46 +7977,14 @@
         </is>
       </c>
       <c r="L76" s="32" t="n"/>
-      <c r="M76" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N76" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O76" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P76" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q76" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R76" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S76" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T76" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M76" s="32" t="n"/>
+      <c r="N76" s="32" t="n"/>
+      <c r="O76" s="32" t="n"/>
+      <c r="P76" s="32" t="n"/>
+      <c r="Q76" s="32" t="n"/>
+      <c r="R76" s="32" t="n"/>
+      <c r="S76" s="32" t="n"/>
+      <c r="T76" s="32" t="n"/>
       <c r="U76" s="33" t="n"/>
       <c r="V76" s="34" t="n"/>
       <c r="W76" s="32" t="inlineStr">
@@ -8218,26 +8074,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 16" riportata nei documenti "casi di test CERT_VACC" e "CDA2_Certificato Vaccinale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F78" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G78" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:17:43</t>
-        </is>
-      </c>
-      <c r="H78" s="31" t="inlineStr">
-        <is>
-          <t>77463446540f43c6179cc98cf7f0b851</t>
-        </is>
-      </c>
-      <c r="I78" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.2f6508dfdd49f71b50664009a32ce80f6a0ce57561a1bea5f7b8480d6d60ceed.ce1b23c9d3^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F78" s="31" t="n"/>
+      <c r="G78" s="31" t="n"/>
+      <c r="H78" s="31" t="n"/>
+      <c r="I78" s="36" t="n"/>
       <c r="J78" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -8249,46 +8089,14 @@
         </is>
       </c>
       <c r="L78" s="32" t="n"/>
-      <c r="M78" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N78" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O78" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P78" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q78" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R78" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S78" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T78" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M78" s="32" t="n"/>
+      <c r="N78" s="32" t="n"/>
+      <c r="O78" s="32" t="n"/>
+      <c r="P78" s="32" t="n"/>
+      <c r="Q78" s="32" t="n"/>
+      <c r="R78" s="32" t="n"/>
+      <c r="S78" s="32" t="n"/>
+      <c r="T78" s="32" t="n"/>
       <c r="U78" s="33" t="n"/>
       <c r="V78" s="34" t="n"/>
       <c r="W78" s="32" t="inlineStr">
@@ -8322,26 +8130,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 17" riportata nei documenti "casi di test CERT_VACC" e "CDA2_Certificato Vaccinale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F79" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G79" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:17:41</t>
-        </is>
-      </c>
-      <c r="H79" s="31" t="inlineStr">
-        <is>
-          <t>1e4947ef5f60b248f6cc587048c9f450</t>
-        </is>
-      </c>
-      <c r="I79" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.63396cbcbe3dfc78b5ad3904be91376e9f2d6731cb0763a0b5fd41cefd2a03f4.39eb44eb8d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F79" s="31" t="n"/>
+      <c r="G79" s="31" t="n"/>
+      <c r="H79" s="31" t="n"/>
+      <c r="I79" s="36" t="n"/>
       <c r="J79" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -8353,46 +8145,14 @@
         </is>
       </c>
       <c r="L79" s="32" t="n"/>
-      <c r="M79" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N79" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O79" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P79" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q79" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R79" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S79" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T79" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M79" s="32" t="n"/>
+      <c r="N79" s="32" t="n"/>
+      <c r="O79" s="32" t="n"/>
+      <c r="P79" s="32" t="n"/>
+      <c r="Q79" s="32" t="n"/>
+      <c r="R79" s="32" t="n"/>
+      <c r="S79" s="32" t="n"/>
+      <c r="T79" s="32" t="n"/>
       <c r="U79" s="33" t="n"/>
       <c r="V79" s="34" t="n"/>
       <c r="W79" s="32" t="inlineStr">
@@ -8426,26 +8186,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 6" riportata nei documenti "casi di test SING_VACC" e "CDA2_Scheda_Singola Vaccinazione_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F80" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G80" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:17:47</t>
-        </is>
-      </c>
-      <c r="H80" s="31" t="inlineStr">
-        <is>
-          <t>346c86394d9e19688c98e1eac3507b73</t>
-        </is>
-      </c>
-      <c r="I80" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.2081e93bc59b43e49e3aeae958e60c84dccb7d9ecdcb4e330174098f046ce5f1.617e1f2a25^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F80" s="31" t="n"/>
+      <c r="G80" s="31" t="n"/>
+      <c r="H80" s="31" t="n"/>
+      <c r="I80" s="36" t="n"/>
       <c r="J80" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -8457,46 +8201,14 @@
         </is>
       </c>
       <c r="L80" s="32" t="n"/>
-      <c r="M80" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N80" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O80" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P80" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q80" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R80" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S80" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T80" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M80" s="32" t="n"/>
+      <c r="N80" s="32" t="n"/>
+      <c r="O80" s="32" t="n"/>
+      <c r="P80" s="32" t="n"/>
+      <c r="Q80" s="32" t="n"/>
+      <c r="R80" s="32" t="n"/>
+      <c r="S80" s="32" t="n"/>
+      <c r="T80" s="32" t="n"/>
       <c r="U80" s="33" t="n"/>
       <c r="V80" s="34" t="n"/>
       <c r="W80" s="32" t="inlineStr">
@@ -8530,26 +8242,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 8" riportata nei documenti "casi di test SING_VACC" e "CDA2_Scheda_Singola Vaccinazione_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F81" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G81" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:17:46</t>
-        </is>
-      </c>
-      <c r="H81" s="31" t="inlineStr">
-        <is>
-          <t>2004061566587dcf572a534701ee0c4f</t>
-        </is>
-      </c>
-      <c r="I81" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.7e4bd7df0b7fcc4937fd1dc164c43f55889e4f64f91ecac8c9cdfdae45fa3124.e84aabc8d7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F81" s="31" t="n"/>
+      <c r="G81" s="31" t="n"/>
+      <c r="H81" s="31" t="n"/>
+      <c r="I81" s="36" t="n"/>
       <c r="J81" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -8561,46 +8257,14 @@
         </is>
       </c>
       <c r="L81" s="32" t="n"/>
-      <c r="M81" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N81" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O81" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P81" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q81" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R81" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S81" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T81" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M81" s="32" t="n"/>
+      <c r="N81" s="32" t="n"/>
+      <c r="O81" s="32" t="n"/>
+      <c r="P81" s="32" t="n"/>
+      <c r="Q81" s="32" t="n"/>
+      <c r="R81" s="32" t="n"/>
+      <c r="S81" s="32" t="n"/>
+      <c r="T81" s="32" t="n"/>
       <c r="U81" s="33" t="n"/>
       <c r="V81" s="34" t="n"/>
       <c r="W81" s="32" t="inlineStr">
@@ -8690,26 +8354,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 10" riportata nei documenti "casi di test SING_VACC" e "CDA2_Scheda_Singola Vaccinazione_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F83" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G83" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:17:44</t>
-        </is>
-      </c>
-      <c r="H83" s="31" t="inlineStr">
-        <is>
-          <t>1934186e7e728b4f72aa8b556f9e9efd</t>
-        </is>
-      </c>
-      <c r="I83" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.0fde0276e8077f4bef24425cac8abdeb6c34b904cde51bb985f1aa2ac04ca359.90a459ae96^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F83" s="31" t="n"/>
+      <c r="G83" s="31" t="n"/>
+      <c r="H83" s="31" t="n"/>
+      <c r="I83" s="36" t="n"/>
       <c r="J83" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -8721,46 +8369,14 @@
         </is>
       </c>
       <c r="L83" s="32" t="n"/>
-      <c r="M83" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N83" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O83" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P83" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q83" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R83" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S83" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T83" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M83" s="32" t="n"/>
+      <c r="N83" s="32" t="n"/>
+      <c r="O83" s="32" t="n"/>
+      <c r="P83" s="32" t="n"/>
+      <c r="Q83" s="32" t="n"/>
+      <c r="R83" s="32" t="n"/>
+      <c r="S83" s="32" t="n"/>
+      <c r="T83" s="32" t="n"/>
       <c r="U83" s="33" t="n"/>
       <c r="V83" s="34" t="n"/>
       <c r="W83" s="32" t="inlineStr">
@@ -8794,26 +8410,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 11" riportata nei documenti "casi di test SING_VACC" e "CDA2_Scheda_Singola Vaccinazione_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F84" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G84" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:17:43</t>
-        </is>
-      </c>
-      <c r="H84" s="31" t="inlineStr">
-        <is>
-          <t>77463446540f43c6179cc98cf7f0b851</t>
-        </is>
-      </c>
-      <c r="I84" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.2f6508dfdd49f71b50664009a32ce80f6a0ce57561a1bea5f7b8480d6d60ceed.ce1b23c9d3^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F84" s="31" t="n"/>
+      <c r="G84" s="31" t="n"/>
+      <c r="H84" s="31" t="n"/>
+      <c r="I84" s="36" t="n"/>
       <c r="J84" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -8825,46 +8425,14 @@
         </is>
       </c>
       <c r="L84" s="32" t="n"/>
-      <c r="M84" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N84" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O84" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P84" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q84" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R84" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S84" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T84" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M84" s="32" t="n"/>
+      <c r="N84" s="32" t="n"/>
+      <c r="O84" s="32" t="n"/>
+      <c r="P84" s="32" t="n"/>
+      <c r="Q84" s="32" t="n"/>
+      <c r="R84" s="32" t="n"/>
+      <c r="S84" s="32" t="n"/>
+      <c r="T84" s="32" t="n"/>
       <c r="U84" s="33" t="n"/>
       <c r="V84" s="34" t="n"/>
       <c r="W84" s="32" t="inlineStr">
@@ -8898,26 +8466,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 12" riportata nei documenti "casi di test SING_VACC" e "CDA2_Scheda_Singola Vaccinazione_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F85" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G85" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:17:41</t>
-        </is>
-      </c>
-      <c r="H85" s="31" t="inlineStr">
-        <is>
-          <t>1e4947ef5f60b248f6cc587048c9f450</t>
-        </is>
-      </c>
-      <c r="I85" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.63396cbcbe3dfc78b5ad3904be91376e9f2d6731cb0763a0b5fd41cefd2a03f4.39eb44eb8d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F85" s="31" t="n"/>
+      <c r="G85" s="31" t="n"/>
+      <c r="H85" s="31" t="n"/>
+      <c r="I85" s="36" t="n"/>
       <c r="J85" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -8929,46 +8481,14 @@
         </is>
       </c>
       <c r="L85" s="32" t="n"/>
-      <c r="M85" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N85" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O85" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P85" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q85" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R85" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S85" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T85" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M85" s="32" t="n"/>
+      <c r="N85" s="32" t="n"/>
+      <c r="O85" s="32" t="n"/>
+      <c r="P85" s="32" t="n"/>
+      <c r="Q85" s="32" t="n"/>
+      <c r="R85" s="32" t="n"/>
+      <c r="S85" s="32" t="n"/>
+      <c r="T85" s="32" t="n"/>
       <c r="U85" s="33" t="n"/>
       <c r="V85" s="34" t="n"/>
       <c r="W85" s="32" t="inlineStr">
@@ -9002,26 +8522,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 13" riportata nei documenti "casi di test SING_VACC" e "CDA2_Scheda_Singola Vaccinazione_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F86" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G86" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:17:47</t>
-        </is>
-      </c>
-      <c r="H86" s="31" t="inlineStr">
-        <is>
-          <t>346c86394d9e19688c98e1eac3507b73</t>
-        </is>
-      </c>
-      <c r="I86" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.2081e93bc59b43e49e3aeae958e60c84dccb7d9ecdcb4e330174098f046ce5f1.617e1f2a25^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F86" s="31" t="n"/>
+      <c r="G86" s="31" t="n"/>
+      <c r="H86" s="31" t="n"/>
+      <c r="I86" s="36" t="n"/>
       <c r="J86" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -9033,46 +8537,14 @@
         </is>
       </c>
       <c r="L86" s="32" t="n"/>
-      <c r="M86" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N86" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O86" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P86" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q86" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R86" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S86" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T86" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M86" s="32" t="n"/>
+      <c r="N86" s="32" t="n"/>
+      <c r="O86" s="32" t="n"/>
+      <c r="P86" s="32" t="n"/>
+      <c r="Q86" s="32" t="n"/>
+      <c r="R86" s="32" t="n"/>
+      <c r="S86" s="32" t="n"/>
+      <c r="T86" s="32" t="n"/>
       <c r="U86" s="33" t="n"/>
       <c r="V86" s="34" t="n"/>
       <c r="W86" s="32" t="inlineStr">
@@ -9106,26 +8578,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 14" riportata nei documenti "casi di test SING_VACC" e "CDA2_Scheda_Singola Vaccinazione_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F87" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G87" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:17:46</t>
-        </is>
-      </c>
-      <c r="H87" s="31" t="inlineStr">
-        <is>
-          <t>2004061566587dcf572a534701ee0c4f</t>
-        </is>
-      </c>
-      <c r="I87" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.7e4bd7df0b7fcc4937fd1dc164c43f55889e4f64f91ecac8c9cdfdae45fa3124.e84aabc8d7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F87" s="31" t="n"/>
+      <c r="G87" s="31" t="n"/>
+      <c r="H87" s="31" t="n"/>
+      <c r="I87" s="36" t="n"/>
       <c r="J87" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -9137,46 +8593,14 @@
         </is>
       </c>
       <c r="L87" s="32" t="n"/>
-      <c r="M87" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N87" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O87" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P87" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q87" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R87" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S87" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T87" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M87" s="32" t="n"/>
+      <c r="N87" s="32" t="n"/>
+      <c r="O87" s="32" t="n"/>
+      <c r="P87" s="32" t="n"/>
+      <c r="Q87" s="32" t="n"/>
+      <c r="R87" s="32" t="n"/>
+      <c r="S87" s="32" t="n"/>
+      <c r="T87" s="32" t="n"/>
       <c r="U87" s="33" t="n"/>
       <c r="V87" s="34" t="n"/>
       <c r="W87" s="32" t="inlineStr">
@@ -9210,26 +8634,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 15" riportata nei documenti "casi di test SING_VACC" e "CDA2_Scheda_Singola Vaccinazione_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F88" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G88" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:17:44</t>
-        </is>
-      </c>
-      <c r="H88" s="31" t="inlineStr">
-        <is>
-          <t>1934186e7e728b4f72aa8b556f9e9efd</t>
-        </is>
-      </c>
-      <c r="I88" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.0fde0276e8077f4bef24425cac8abdeb6c34b904cde51bb985f1aa2ac04ca359.90a459ae96^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F88" s="31" t="n"/>
+      <c r="G88" s="31" t="n"/>
+      <c r="H88" s="31" t="n"/>
+      <c r="I88" s="36" t="n"/>
       <c r="J88" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -9241,46 +8649,14 @@
         </is>
       </c>
       <c r="L88" s="32" t="n"/>
-      <c r="M88" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N88" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O88" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P88" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q88" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R88" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S88" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T88" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M88" s="32" t="n"/>
+      <c r="N88" s="32" t="n"/>
+      <c r="O88" s="32" t="n"/>
+      <c r="P88" s="32" t="n"/>
+      <c r="Q88" s="32" t="n"/>
+      <c r="R88" s="32" t="n"/>
+      <c r="S88" s="32" t="n"/>
+      <c r="T88" s="32" t="n"/>
       <c r="U88" s="33" t="n"/>
       <c r="V88" s="34" t="n"/>
       <c r="W88" s="32" t="inlineStr">
@@ -9314,26 +8690,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 16" riportata nei documenti "casi di test SING_VACC" e "CDA2_Scheda_Singola Vaccinazione_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F89" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G89" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:17:43</t>
-        </is>
-      </c>
-      <c r="H89" s="31" t="inlineStr">
-        <is>
-          <t>77463446540f43c6179cc98cf7f0b851</t>
-        </is>
-      </c>
-      <c r="I89" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.2f6508dfdd49f71b50664009a32ce80f6a0ce57561a1bea5f7b8480d6d60ceed.ce1b23c9d3^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F89" s="31" t="n"/>
+      <c r="G89" s="31" t="n"/>
+      <c r="H89" s="31" t="n"/>
+      <c r="I89" s="36" t="n"/>
       <c r="J89" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -9345,46 +8705,14 @@
         </is>
       </c>
       <c r="L89" s="32" t="n"/>
-      <c r="M89" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N89" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O89" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P89" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q89" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R89" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S89" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T89" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M89" s="32" t="n"/>
+      <c r="N89" s="32" t="n"/>
+      <c r="O89" s="32" t="n"/>
+      <c r="P89" s="32" t="n"/>
+      <c r="Q89" s="32" t="n"/>
+      <c r="R89" s="32" t="n"/>
+      <c r="S89" s="32" t="n"/>
+      <c r="T89" s="32" t="n"/>
       <c r="U89" s="33" t="n"/>
       <c r="V89" s="34" t="n"/>
       <c r="W89" s="32" t="inlineStr">
@@ -9418,26 +8746,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 17" riportata nei documenti "casi di test SING_VACC" e "CDA2_Scheda_Singola Vaccinazione_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F90" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G90" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:17:41</t>
-        </is>
-      </c>
-      <c r="H90" s="31" t="inlineStr">
-        <is>
-          <t>1e4947ef5f60b248f6cc587048c9f450</t>
-        </is>
-      </c>
-      <c r="I90" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.63396cbcbe3dfc78b5ad3904be91376e9f2d6731cb0763a0b5fd41cefd2a03f4.39eb44eb8d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F90" s="31" t="n"/>
+      <c r="G90" s="31" t="n"/>
+      <c r="H90" s="31" t="n"/>
+      <c r="I90" s="36" t="n"/>
       <c r="J90" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -9449,46 +8761,14 @@
         </is>
       </c>
       <c r="L90" s="32" t="n"/>
-      <c r="M90" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N90" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O90" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P90" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q90" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R90" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S90" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T90" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M90" s="32" t="n"/>
+      <c r="N90" s="32" t="n"/>
+      <c r="O90" s="32" t="n"/>
+      <c r="P90" s="32" t="n"/>
+      <c r="Q90" s="32" t="n"/>
+      <c r="R90" s="32" t="n"/>
+      <c r="S90" s="32" t="n"/>
+      <c r="T90" s="32" t="n"/>
       <c r="U90" s="33" t="n"/>
       <c r="V90" s="34" t="n"/>
       <c r="W90" s="32" t="inlineStr">
@@ -9522,26 +8802,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 18" riportata nei documenti "casi di test SING_VACC" e "CDA2_Scheda_Singola Vaccinazione_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F91" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G91" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:17:47</t>
-        </is>
-      </c>
-      <c r="H91" s="31" t="inlineStr">
-        <is>
-          <t>346c86394d9e19688c98e1eac3507b73</t>
-        </is>
-      </c>
-      <c r="I91" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.2081e93bc59b43e49e3aeae958e60c84dccb7d9ecdcb4e330174098f046ce5f1.617e1f2a25^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F91" s="31" t="n"/>
+      <c r="G91" s="31" t="n"/>
+      <c r="H91" s="31" t="n"/>
+      <c r="I91" s="36" t="n"/>
       <c r="J91" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -9553,46 +8817,14 @@
         </is>
       </c>
       <c r="L91" s="32" t="n"/>
-      <c r="M91" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N91" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O91" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P91" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q91" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R91" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S91" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T91" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M91" s="32" t="n"/>
+      <c r="N91" s="32" t="n"/>
+      <c r="O91" s="32" t="n"/>
+      <c r="P91" s="32" t="n"/>
+      <c r="Q91" s="32" t="n"/>
+      <c r="R91" s="32" t="n"/>
+      <c r="S91" s="32" t="n"/>
+      <c r="T91" s="32" t="n"/>
       <c r="U91" s="33" t="n"/>
       <c r="V91" s="34" t="n"/>
       <c r="W91" s="32" t="inlineStr">
@@ -9626,26 +8858,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 19" riportata nei documenti "casi di test SING_VACC" e "CDA2_Scheda_Singola Vaccinazione_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F92" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G92" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:17:46</t>
-        </is>
-      </c>
-      <c r="H92" s="31" t="inlineStr">
-        <is>
-          <t>2004061566587dcf572a534701ee0c4f</t>
-        </is>
-      </c>
-      <c r="I92" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.7e4bd7df0b7fcc4937fd1dc164c43f55889e4f64f91ecac8c9cdfdae45fa3124.e84aabc8d7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F92" s="31" t="n"/>
+      <c r="G92" s="31" t="n"/>
+      <c r="H92" s="31" t="n"/>
+      <c r="I92" s="36" t="n"/>
       <c r="J92" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -9657,46 +8873,14 @@
         </is>
       </c>
       <c r="L92" s="32" t="n"/>
-      <c r="M92" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N92" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O92" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P92" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q92" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R92" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S92" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T92" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M92" s="32" t="n"/>
+      <c r="N92" s="32" t="n"/>
+      <c r="O92" s="32" t="n"/>
+      <c r="P92" s="32" t="n"/>
+      <c r="Q92" s="32" t="n"/>
+      <c r="R92" s="32" t="n"/>
+      <c r="S92" s="32" t="n"/>
+      <c r="T92" s="32" t="n"/>
       <c r="U92" s="33" t="n"/>
       <c r="V92" s="34" t="n"/>
       <c r="W92" s="32" t="inlineStr">
@@ -9730,26 +8914,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 6" riportata nei documenti "casi di test VPS" e "CDA2_Verbale_Pronto_Soccorso_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F93" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G93" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:17:44</t>
-        </is>
-      </c>
-      <c r="H93" s="31" t="inlineStr">
-        <is>
-          <t>1934186e7e728b4f72aa8b556f9e9efd</t>
-        </is>
-      </c>
-      <c r="I93" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.0fde0276e8077f4bef24425cac8abdeb6c34b904cde51bb985f1aa2ac04ca359.90a459ae96^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F93" s="31" t="n"/>
+      <c r="G93" s="31" t="n"/>
+      <c r="H93" s="31" t="n"/>
+      <c r="I93" s="36" t="n"/>
       <c r="J93" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -9761,46 +8929,14 @@
         </is>
       </c>
       <c r="L93" s="32" t="n"/>
-      <c r="M93" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N93" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O93" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P93" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q93" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R93" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S93" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T93" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M93" s="32" t="n"/>
+      <c r="N93" s="32" t="n"/>
+      <c r="O93" s="32" t="n"/>
+      <c r="P93" s="32" t="n"/>
+      <c r="Q93" s="32" t="n"/>
+      <c r="R93" s="32" t="n"/>
+      <c r="S93" s="32" t="n"/>
+      <c r="T93" s="32" t="n"/>
       <c r="U93" s="33" t="n"/>
       <c r="V93" s="34" t="n"/>
       <c r="W93" s="32" t="inlineStr">
@@ -11125,7 +10261,7 @@
       </c>
       <c r="S116" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T116" s="32" t="inlineStr">
@@ -11225,7 +10361,7 @@
       </c>
       <c r="S117" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T117" s="32" t="inlineStr">
@@ -11325,7 +10461,7 @@
       </c>
       <c r="S118" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T118" s="32" t="inlineStr">
@@ -11425,7 +10561,7 @@
       </c>
       <c r="S119" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T119" s="32" t="inlineStr">
@@ -11525,7 +10661,7 @@
       </c>
       <c r="S120" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T120" s="32" t="inlineStr">
@@ -11625,7 +10761,7 @@
       </c>
       <c r="S121" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T121" s="32" t="inlineStr">
@@ -11725,7 +10861,7 @@
       </c>
       <c r="S122" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T122" s="32" t="inlineStr">
@@ -11825,7 +10961,7 @@
       </c>
       <c r="S123" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T123" s="32" t="inlineStr">
@@ -11925,7 +11061,7 @@
       </c>
       <c r="S124" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T124" s="32" t="inlineStr">
@@ -12025,7 +11161,7 @@
       </c>
       <c r="S125" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T125" s="32" t="inlineStr">
@@ -12125,7 +11261,7 @@
       </c>
       <c r="S126" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T126" s="32" t="inlineStr">
@@ -12225,7 +11361,7 @@
       </c>
       <c r="S127" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T127" s="32" t="inlineStr">
@@ -12325,7 +11461,7 @@
       </c>
       <c r="S128" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T128" s="32" t="inlineStr">
@@ -12425,7 +11561,7 @@
       </c>
       <c r="S129" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T129" s="32" t="inlineStr">
@@ -12525,7 +11661,7 @@
       </c>
       <c r="S130" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T130" s="32" t="inlineStr">
@@ -13414,17 +12550,17 @@
       </c>
       <c r="G146" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:16:12</t>
+          <t>2026-03-26T08:16:09Z</t>
         </is>
       </c>
       <c r="H146" s="31" t="inlineStr">
         <is>
-          <t>e7b184d9004b721d45058522970f3cb8</t>
+          <t>50a2d5255994760191912f3e5db901b8</t>
         </is>
       </c>
       <c r="I146" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.c7cfc54dcfac0c48c09bb8cfef8f6d91bce2ddc0f8c56e438d3312b3358a249c.8538eae2a6^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.01e6e0d273b0aa21e7077088a79700b63f4d4f56bfc125549fb332b77f1f5ac6.5592d64822^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J146" s="32" t="inlineStr">
@@ -13515,17 +12651,17 @@
       </c>
       <c r="G147" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:16:09</t>
+          <t>2026-03-26T08:16:05Z</t>
         </is>
       </c>
       <c r="H147" s="31" t="inlineStr">
         <is>
-          <t>50a2d5255994760191912f3e5db901b8</t>
+          <t>39bf5a23f89affe2c2caf41ee117af53</t>
         </is>
       </c>
       <c r="I147" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.01e6e0d273b0aa21e7077088a79700b63f4d4f56bfc125549fb332b77f1f5ac6.5592d64822^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.c1d6cf78d1042e56a6418170d49febb3ea72c59e997f9e70e184e877b391aade.508fd7c970^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J147" s="32" t="inlineStr">
@@ -13840,26 +12976,10 @@
 Al fine di rendere non valido il token è necessario valorizzare il campo "action_id" con la stringa "TEST" (valore non ammesso).</t>
         </is>
       </c>
-      <c r="F152" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G152" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:49</t>
-        </is>
-      </c>
-      <c r="H152" s="31" t="inlineStr">
-        <is>
-          <t>acaaee0bef9df190c95a8e1922b13422</t>
-        </is>
-      </c>
-      <c r="I152" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.803c6bbaf321647710ce6fe3fe1c2d532c81a9bca2ce4bf6a38b58bfd7f39a94.591366733d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F152" s="31" t="n"/>
+      <c r="G152" s="31" t="n"/>
+      <c r="H152" s="31" t="n"/>
+      <c r="I152" s="36" t="n"/>
       <c r="J152" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -13871,46 +12991,14 @@
         </is>
       </c>
       <c r="L152" s="32" t="n"/>
-      <c r="M152" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N152" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O152" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P152" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q152" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R152" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S152" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T152" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M152" s="32" t="n"/>
+      <c r="N152" s="32" t="n"/>
+      <c r="O152" s="32" t="n"/>
+      <c r="P152" s="32" t="n"/>
+      <c r="Q152" s="32" t="n"/>
+      <c r="R152" s="32" t="n"/>
+      <c r="S152" s="32" t="n"/>
+      <c r="T152" s="32" t="n"/>
       <c r="U152" s="33" t="n"/>
       <c r="V152" s="34" t="n"/>
       <c r="W152" s="32" t="inlineStr">
@@ -14004,26 +13092,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto nella sezione "CASO DI TEST 12" riportata nei documenti "casi di test RAP" e "CDA2_Referto_di_Anatomia_Patologica_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F154" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G154" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:48</t>
-        </is>
-      </c>
-      <c r="H154" s="31" t="inlineStr">
-        <is>
-          <t>70bb39da81bcfc0fb8569598d4b66c36</t>
-        </is>
-      </c>
-      <c r="I154" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.588b5d3634416a6059a7318ba561bee1b3937a3a743aee7bdf6c94514c0aff0c.40b608332a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F154" s="31" t="n"/>
+      <c r="G154" s="31" t="n"/>
+      <c r="H154" s="31" t="n"/>
+      <c r="I154" s="36" t="n"/>
       <c r="J154" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -14035,46 +13107,14 @@
         </is>
       </c>
       <c r="L154" s="32" t="n"/>
-      <c r="M154" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N154" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O154" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P154" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q154" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R154" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S154" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T154" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M154" s="32" t="n"/>
+      <c r="N154" s="32" t="n"/>
+      <c r="O154" s="32" t="n"/>
+      <c r="P154" s="32" t="n"/>
+      <c r="Q154" s="32" t="n"/>
+      <c r="R154" s="32" t="n"/>
+      <c r="S154" s="32" t="n"/>
+      <c r="T154" s="32" t="n"/>
       <c r="U154" s="33" t="n"/>
       <c r="V154" s="34" t="n"/>
       <c r="W154" s="32" t="inlineStr">
@@ -14108,26 +13148,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto nella sezione "CASO DI TEST 13" riportata nei documenti "casi di test RAP" e "CDA2_Referto_di_Anatomia_Patologica_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F155" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G155" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:46</t>
-        </is>
-      </c>
-      <c r="H155" s="31" t="inlineStr">
-        <is>
-          <t>3dcaffaa4a45aa93bcd389ef97304f18</t>
-        </is>
-      </c>
-      <c r="I155" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.0d71ec15820089182c6cafc0b3549797232f132d9d3d2fd9aa9f4d1a0aab5829.4ce80475d4^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F155" s="31" t="n"/>
+      <c r="G155" s="31" t="n"/>
+      <c r="H155" s="31" t="n"/>
+      <c r="I155" s="36" t="n"/>
       <c r="J155" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -14139,46 +13163,14 @@
         </is>
       </c>
       <c r="L155" s="32" t="n"/>
-      <c r="M155" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N155" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O155" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P155" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q155" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R155" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S155" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T155" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M155" s="32" t="n"/>
+      <c r="N155" s="32" t="n"/>
+      <c r="O155" s="32" t="n"/>
+      <c r="P155" s="32" t="n"/>
+      <c r="Q155" s="32" t="n"/>
+      <c r="R155" s="32" t="n"/>
+      <c r="S155" s="32" t="n"/>
+      <c r="T155" s="32" t="n"/>
       <c r="U155" s="33" t="n"/>
       <c r="V155" s="34" t="n"/>
       <c r="W155" s="32" t="inlineStr">
@@ -14212,26 +13204,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto nella sezione "CASO DI TEST 14" riportata nei documenti "casi di test RAP" e "CDA2_Referto_di_Anatomia_Patologica_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F156" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G156" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:52</t>
-        </is>
-      </c>
-      <c r="H156" s="31" t="inlineStr">
-        <is>
-          <t>a0cb1ce26dd8782352e5f05ddef141a2</t>
-        </is>
-      </c>
-      <c r="I156" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.b9a0ee4080bbd8e3616f9fe9ac6ae4e7be45391a9498d7b89ee4c3483892a723.da957b601c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F156" s="31" t="n"/>
+      <c r="G156" s="31" t="n"/>
+      <c r="H156" s="31" t="n"/>
+      <c r="I156" s="36" t="n"/>
       <c r="J156" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -14243,46 +13219,14 @@
         </is>
       </c>
       <c r="L156" s="32" t="n"/>
-      <c r="M156" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N156" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O156" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P156" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q156" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R156" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S156" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T156" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M156" s="32" t="n"/>
+      <c r="N156" s="32" t="n"/>
+      <c r="O156" s="32" t="n"/>
+      <c r="P156" s="32" t="n"/>
+      <c r="Q156" s="32" t="n"/>
+      <c r="R156" s="32" t="n"/>
+      <c r="S156" s="32" t="n"/>
+      <c r="T156" s="32" t="n"/>
       <c r="U156" s="33" t="n"/>
       <c r="V156" s="34" t="n"/>
       <c r="W156" s="32" t="inlineStr">
@@ -14428,26 +13372,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto nella sezione "CASO DI TEST 18" riportata nei documenti "casi di test RAP" e "CDA2_Referto_di_Anatomia_Patologica_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F159" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G159" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:51</t>
-        </is>
-      </c>
-      <c r="H159" s="31" t="inlineStr">
-        <is>
-          <t>db39cac5c8c5804640e75bea38bc7b37</t>
-        </is>
-      </c>
-      <c r="I159" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.fc1f4ad5ea95e6f48b902f5fe383ae99a3da61a65f0dc53830b78929479ddd3d.3786d8ab7b^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F159" s="31" t="n"/>
+      <c r="G159" s="31" t="n"/>
+      <c r="H159" s="31" t="n"/>
+      <c r="I159" s="36" t="n"/>
       <c r="J159" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -14459,46 +13387,14 @@
         </is>
       </c>
       <c r="L159" s="32" t="n"/>
-      <c r="M159" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N159" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O159" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P159" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q159" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R159" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S159" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T159" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M159" s="32" t="n"/>
+      <c r="N159" s="32" t="n"/>
+      <c r="O159" s="32" t="n"/>
+      <c r="P159" s="32" t="n"/>
+      <c r="Q159" s="32" t="n"/>
+      <c r="R159" s="32" t="n"/>
+      <c r="S159" s="32" t="n"/>
+      <c r="T159" s="32" t="n"/>
       <c r="U159" s="33" t="n"/>
       <c r="V159" s="34" t="n"/>
       <c r="W159" s="32" t="inlineStr">
@@ -14532,26 +13428,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto nella sezione "CASO DI TEST 20" riportata nei documenti "casi di test RAP" e "CDA2_Referto_di_Anatomia_Patologica_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F160" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G160" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:49</t>
-        </is>
-      </c>
-      <c r="H160" s="31" t="inlineStr">
-        <is>
-          <t>acaaee0bef9df190c95a8e1922b13422</t>
-        </is>
-      </c>
-      <c r="I160" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.803c6bbaf321647710ce6fe3fe1c2d532c81a9bca2ce4bf6a38b58bfd7f39a94.591366733d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F160" s="31" t="n"/>
+      <c r="G160" s="31" t="n"/>
+      <c r="H160" s="31" t="n"/>
+      <c r="I160" s="36" t="n"/>
       <c r="J160" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -14563,46 +13443,14 @@
         </is>
       </c>
       <c r="L160" s="32" t="n"/>
-      <c r="M160" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N160" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O160" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P160" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q160" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R160" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S160" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T160" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M160" s="32" t="n"/>
+      <c r="N160" s="32" t="n"/>
+      <c r="O160" s="32" t="n"/>
+      <c r="P160" s="32" t="n"/>
+      <c r="Q160" s="32" t="n"/>
+      <c r="R160" s="32" t="n"/>
+      <c r="S160" s="32" t="n"/>
+      <c r="T160" s="32" t="n"/>
       <c r="U160" s="33" t="n"/>
       <c r="V160" s="34" t="n"/>
       <c r="W160" s="32" t="inlineStr">
@@ -14636,26 +13484,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto nella sezione "CASO DI TEST 21" riportata nei documenti "casi di test RAP" e "CDA2_Referto_di_Anatomia_Patologica_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F161" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G161" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:48</t>
-        </is>
-      </c>
-      <c r="H161" s="31" t="inlineStr">
-        <is>
-          <t>70bb39da81bcfc0fb8569598d4b66c36</t>
-        </is>
-      </c>
-      <c r="I161" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.588b5d3634416a6059a7318ba561bee1b3937a3a743aee7bdf6c94514c0aff0c.40b608332a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F161" s="31" t="n"/>
+      <c r="G161" s="31" t="n"/>
+      <c r="H161" s="31" t="n"/>
+      <c r="I161" s="36" t="n"/>
       <c r="J161" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -14667,46 +13499,14 @@
         </is>
       </c>
       <c r="L161" s="32" t="n"/>
-      <c r="M161" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N161" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O161" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P161" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q161" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R161" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S161" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T161" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M161" s="32" t="n"/>
+      <c r="N161" s="32" t="n"/>
+      <c r="O161" s="32" t="n"/>
+      <c r="P161" s="32" t="n"/>
+      <c r="Q161" s="32" t="n"/>
+      <c r="R161" s="32" t="n"/>
+      <c r="S161" s="32" t="n"/>
+      <c r="T161" s="32" t="n"/>
       <c r="U161" s="33" t="n"/>
       <c r="V161" s="34" t="n"/>
       <c r="W161" s="32" t="inlineStr">
@@ -14740,26 +13540,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto nella sezione "CASO DI TEST 22" riportata nei documenti "casi di test RAP" e "CDA2_Referto_di_Anatomia_Patologica_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F162" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G162" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:46</t>
-        </is>
-      </c>
-      <c r="H162" s="31" t="inlineStr">
-        <is>
-          <t>3dcaffaa4a45aa93bcd389ef97304f18</t>
-        </is>
-      </c>
-      <c r="I162" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.0d71ec15820089182c6cafc0b3549797232f132d9d3d2fd9aa9f4d1a0aab5829.4ce80475d4^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F162" s="31" t="n"/>
+      <c r="G162" s="31" t="n"/>
+      <c r="H162" s="31" t="n"/>
+      <c r="I162" s="36" t="n"/>
       <c r="J162" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -14771,46 +13555,14 @@
         </is>
       </c>
       <c r="L162" s="32" t="n"/>
-      <c r="M162" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N162" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O162" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P162" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q162" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R162" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S162" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T162" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M162" s="32" t="n"/>
+      <c r="N162" s="32" t="n"/>
+      <c r="O162" s="32" t="n"/>
+      <c r="P162" s="32" t="n"/>
+      <c r="Q162" s="32" t="n"/>
+      <c r="R162" s="32" t="n"/>
+      <c r="S162" s="32" t="n"/>
+      <c r="T162" s="32" t="n"/>
       <c r="U162" s="33" t="n"/>
       <c r="V162" s="34" t="n"/>
       <c r="W162" s="32" t="inlineStr">
@@ -14844,26 +13596,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto nella sezione "CASO DI TEST 23" riportata nei documenti "casi di test RAP" e "CDA2_Referto_di_Anatomia_Patologica_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F163" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G163" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:52</t>
-        </is>
-      </c>
-      <c r="H163" s="31" t="inlineStr">
-        <is>
-          <t>a0cb1ce26dd8782352e5f05ddef141a2</t>
-        </is>
-      </c>
-      <c r="I163" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.b9a0ee4080bbd8e3616f9fe9ac6ae4e7be45391a9498d7b89ee4c3483892a723.da957b601c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F163" s="31" t="n"/>
+      <c r="G163" s="31" t="n"/>
+      <c r="H163" s="31" t="n"/>
+      <c r="I163" s="36" t="n"/>
       <c r="J163" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -14875,46 +13611,14 @@
         </is>
       </c>
       <c r="L163" s="32" t="n"/>
-      <c r="M163" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N163" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O163" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P163" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q163" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R163" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S163" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T163" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M163" s="32" t="n"/>
+      <c r="N163" s="32" t="n"/>
+      <c r="O163" s="32" t="n"/>
+      <c r="P163" s="32" t="n"/>
+      <c r="Q163" s="32" t="n"/>
+      <c r="R163" s="32" t="n"/>
+      <c r="S163" s="32" t="n"/>
+      <c r="T163" s="32" t="n"/>
       <c r="U163" s="33" t="n"/>
       <c r="V163" s="34" t="n"/>
       <c r="W163" s="32" t="inlineStr">
@@ -14955,17 +13659,17 @@
       </c>
       <c r="G164" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:16:52</t>
+          <t>2026-03-26T08:16:40Z</t>
         </is>
       </c>
       <c r="H164" s="31" t="inlineStr">
         <is>
-          <t>a0cb1ce26dd8782352e5f05ddef141a2</t>
+          <t>eda1b7d83a4417b530d8239713c1dff2</t>
         </is>
       </c>
       <c r="I164" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.b9a0ee4080bbd8e3616f9fe9ac6ae4e7be45391a9498d7b89ee4c3483892a723.da957b601c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.ce5cc578064408b79e56c402985d5b14f6398836d305417da35843092e9b9d23.4b97ba9236^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J164" s="32" t="inlineStr">
@@ -14987,7 +13691,7 @@
       </c>
       <c r="O164" s="32" t="inlineStr">
         <is>
-          <t>Errore segnalato dal gateway FSE</t>
+          <t>Errore segnalato dal gateway FSE con dettaglio tecnico</t>
         </is>
       </c>
       <c r="P164" s="32" t="inlineStr">
@@ -15055,17 +13759,17 @@
       </c>
       <c r="G165" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:16:51</t>
+          <t>2026-03-26T08:16:38Z</t>
         </is>
       </c>
       <c r="H165" s="31" t="inlineStr">
         <is>
-          <t>db39cac5c8c5804640e75bea38bc7b37</t>
+          <t>7f55b877ff24de115b6d3400ea7b1cef</t>
         </is>
       </c>
       <c r="I165" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.fc1f4ad5ea95e6f48b902f5fe383ae99a3da61a65f0dc53830b78929479ddd3d.3786d8ab7b^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.c77b9e3a5e9d1aeccddc790c45f4cbd460d0f9575c211468bfef2feac83a8f1d.5cc1f692bc^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J165" s="32" t="inlineStr">
@@ -15087,7 +13791,7 @@
       </c>
       <c r="O165" s="32" t="inlineStr">
         <is>
-          <t>Errore segnalato dal gateway FSE</t>
+          <t>Errore segnalato dal gateway FSE con dettaglio tecnico</t>
         </is>
       </c>
       <c r="P165" s="32" t="inlineStr">
@@ -15148,26 +13852,10 @@
 Il Documento CDA2 Lettera Dimissione Ospedaliera dovrà essere composto in modo da risultare valido dal punto di vista sintattico, semantico, terminologico. I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso dalla sezione "CASO DI TEST 17" riportata nei documenti "casi di test LDO" e "CDA2_Lettera di Dimissione Ospedaliera_OK" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F166" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G166" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:48</t>
-        </is>
-      </c>
-      <c r="H166" s="31" t="inlineStr">
-        <is>
-          <t>70bb39da81bcfc0fb8569598d4b66c36</t>
-        </is>
-      </c>
-      <c r="I166" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.588b5d3634416a6059a7318ba561bee1b3937a3a743aee7bdf6c94514c0aff0c.40b608332a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F166" s="31" t="n"/>
+      <c r="G166" s="31" t="n"/>
+      <c r="H166" s="31" t="n"/>
+      <c r="I166" s="36" t="n"/>
       <c r="J166" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -15179,46 +13867,14 @@
         </is>
       </c>
       <c r="L166" s="32" t="n"/>
-      <c r="M166" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N166" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O166" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P166" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q166" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R166" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S166" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T166" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M166" s="32" t="n"/>
+      <c r="N166" s="32" t="n"/>
+      <c r="O166" s="32" t="n"/>
+      <c r="P166" s="32" t="n"/>
+      <c r="Q166" s="32" t="n"/>
+      <c r="R166" s="32" t="n"/>
+      <c r="S166" s="32" t="n"/>
+      <c r="T166" s="32" t="n"/>
       <c r="U166" s="33" t="n"/>
       <c r="V166" s="34" t="n"/>
       <c r="W166" s="32" t="inlineStr">
@@ -15252,26 +13908,10 @@
 Il Documento CDA2 Lettera Dimissione Ospedaliera dovrà essere composto in modo da risultare valido dal punto di vista sintattico, semantico, terminologico. I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso dalla sezione "CASO DI TEST 18" riportata nei documenti "casi di test LDO" e "CDA2_Lettera di Dimissione Ospedaliera_OK" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F167" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G167" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:46</t>
-        </is>
-      </c>
-      <c r="H167" s="31" t="inlineStr">
-        <is>
-          <t>3dcaffaa4a45aa93bcd389ef97304f18</t>
-        </is>
-      </c>
-      <c r="I167" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.0d71ec15820089182c6cafc0b3549797232f132d9d3d2fd9aa9f4d1a0aab5829.4ce80475d4^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F167" s="31" t="n"/>
+      <c r="G167" s="31" t="n"/>
+      <c r="H167" s="31" t="n"/>
+      <c r="I167" s="36" t="n"/>
       <c r="J167" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -15283,46 +13923,14 @@
         </is>
       </c>
       <c r="L167" s="32" t="n"/>
-      <c r="M167" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N167" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O167" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P167" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q167" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R167" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S167" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T167" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M167" s="32" t="n"/>
+      <c r="N167" s="32" t="n"/>
+      <c r="O167" s="32" t="n"/>
+      <c r="P167" s="32" t="n"/>
+      <c r="Q167" s="32" t="n"/>
+      <c r="R167" s="32" t="n"/>
+      <c r="S167" s="32" t="n"/>
+      <c r="T167" s="32" t="n"/>
       <c r="U167" s="33" t="n"/>
       <c r="V167" s="34" t="n"/>
       <c r="W167" s="32" t="inlineStr">
@@ -15364,17 +13972,17 @@
       </c>
       <c r="G168" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:16:05</t>
+          <t>2026-03-26T08:16:03Z</t>
         </is>
       </c>
       <c r="H168" s="31" t="inlineStr">
         <is>
-          <t>39bf5a23f89affe2c2caf41ee117af53</t>
+          <t>4f81a52a074de362116fe5b83bd88d1c</t>
         </is>
       </c>
       <c r="I168" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.c1d6cf78d1042e56a6418170d49febb3ea72c59e997f9e70e184e877b391aade.508fd7c970^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.1d1e8bfe895a15711fddad4b7bd2dcaa7a03f0afcd46bcb80715cab089b72de1.4e1ce9c542^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J168" s="32" t="inlineStr">
@@ -15396,7 +14004,7 @@
       </c>
       <c r="O168" s="32" t="inlineStr">
         <is>
-          <t>Errore segnalato dal gateway FSE</t>
+          <t>Errore segnalato dal gateway FSE con dettaglio tecnico</t>
         </is>
       </c>
       <c r="P168" s="32" t="inlineStr">
@@ -15457,26 +14065,10 @@
 Il Documento CDA2 Verbale di Pronto Soccorso dovrà essere composto in modo da risultare valido dal punto di vista sintattico, semantico, terminologico. I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso dalla sezione "CASO DI TEST 30" riportata nei documenti "casi di test VPS" e "CDA2_Verbale_Pronto_Soccorso_OK" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F169" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G169" s="31" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:51</t>
-        </is>
-      </c>
-      <c r="H169" s="31" t="inlineStr">
-        <is>
-          <t>db39cac5c8c5804640e75bea38bc7b37</t>
-        </is>
-      </c>
-      <c r="I169" s="36" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.fc1f4ad5ea95e6f48b902f5fe383ae99a3da61a65f0dc53830b78929479ddd3d.3786d8ab7b^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
+      <c r="F169" s="31" t="n"/>
+      <c r="G169" s="31" t="n"/>
+      <c r="H169" s="31" t="n"/>
+      <c r="I169" s="36" t="n"/>
       <c r="J169" s="32" t="inlineStr">
         <is>
           <t>NO</t>
@@ -15488,46 +14080,14 @@
         </is>
       </c>
       <c r="L169" s="32" t="n"/>
-      <c r="M169" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N169" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O169" s="32" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P169" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q169" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R169" s="32" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S169" s="32" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T169" s="32" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
+      <c r="M169" s="32" t="n"/>
+      <c r="N169" s="32" t="n"/>
+      <c r="O169" s="32" t="n"/>
+      <c r="P169" s="32" t="n"/>
+      <c r="Q169" s="32" t="n"/>
+      <c r="R169" s="32" t="n"/>
+      <c r="S169" s="32" t="n"/>
+      <c r="T169" s="32" t="n"/>
       <c r="U169" s="33" t="n"/>
       <c r="V169" s="34" t="n"/>
       <c r="W169" s="32" t="inlineStr">
@@ -15956,7 +14516,7 @@
       </c>
       <c r="S176" s="29" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T176" s="32" t="inlineStr">
@@ -16056,7 +14616,7 @@
       </c>
       <c r="S177" s="29" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T177" s="32" t="inlineStr">
@@ -16324,7 +14884,7 @@
       </c>
       <c r="S181" s="29" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T181" s="32" t="inlineStr">
@@ -16480,7 +15040,7 @@
       </c>
       <c r="S183" s="29" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T183" s="32" t="inlineStr">
@@ -16640,7 +15200,7 @@
       </c>
       <c r="G186" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:17:47</t>
+          <t>2026-03-26T08:17:47Z</t>
         </is>
       </c>
       <c r="H186" s="31" t="inlineStr">
@@ -16740,7 +15300,7 @@
       </c>
       <c r="G187" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T08:17:46</t>
+          <t>2026-03-26T08:17:46Z</t>
         </is>
       </c>
       <c r="H187" s="31" t="inlineStr">
@@ -16892,7 +15452,7 @@
       </c>
       <c r="S188" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T188" s="32" t="inlineStr">
@@ -16992,7 +15552,7 @@
       </c>
       <c r="S189" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T189" s="32" t="inlineStr">
@@ -17092,7 +15652,7 @@
       </c>
       <c r="S190" s="32" t="inlineStr">
         <is>
-          <t>L'errore viene loggato e mostrato all'operatore. Il documento viene messo in coda retry automatica. Reinvio manuale disponibile.</t>
+          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
         </is>
       </c>
       <c r="T190" s="32" t="inlineStr">
@@ -23780,129 +22340,9 @@
       <c r="W460" s="7" t="n"/>
     </row>
     <row r="461" ht="14.25" customHeight="1" s="50">
-      <c r="F461" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G461" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:49</t>
-        </is>
-      </c>
-      <c r="H461" t="inlineStr">
-        <is>
-          <t>acaaee0bef9df190c95a8e1922b13422</t>
-        </is>
-      </c>
-      <c r="I461" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.803c6bbaf321647710ce6fe3fe1c2d532c81a9bca2ce4bf6a38b58bfd7f39a94.591366733d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
-      <c r="M461" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N461" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O461" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P461" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q461" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R461" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S461" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T461" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
       <c r="W461" s="7" t="n"/>
     </row>
     <row r="462" ht="14.25" customHeight="1" s="50">
-      <c r="F462" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G462" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:17:43</t>
-        </is>
-      </c>
-      <c r="H462" t="inlineStr">
-        <is>
-          <t>77463446540f43c6179cc98cf7f0b851</t>
-        </is>
-      </c>
-      <c r="I462" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.2f6508dfdd49f71b50664009a32ce80f6a0ce57561a1bea5f7b8480d6d60ceed.ce1b23c9d3^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
-      <c r="M462" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N462" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O462" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P462" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q462" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R462" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S462" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T462" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
       <c r="W462" s="7" t="n"/>
     </row>
     <row r="463" ht="14.25" customHeight="1" s="50">
@@ -23915,132 +22355,12 @@
       <c r="W465" s="7" t="n"/>
     </row>
     <row r="466" ht="14.25" customHeight="1" s="50">
-      <c r="F466" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G466" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:15</t>
-        </is>
-      </c>
-      <c r="H466" t="inlineStr">
-        <is>
-          <t>ff55db762ded2539affd730de18bd8c1</t>
-        </is>
-      </c>
-      <c r="I466" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.8b4e07e56d5aa565f9a8de121321d2d8eb791aefc994d88859d9672a4b396b04.66e074ff48^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
-      <c r="M466" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N466" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O466" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P466" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q466" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R466" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S466" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T466" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
       <c r="W466" s="7" t="n"/>
     </row>
     <row r="467" ht="14.25" customHeight="1" s="50">
       <c r="W467" s="7" t="n"/>
     </row>
     <row r="468" ht="14.25" customHeight="1" s="50">
-      <c r="F468" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G468" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:48</t>
-        </is>
-      </c>
-      <c r="H468" t="inlineStr">
-        <is>
-          <t>70bb39da81bcfc0fb8569598d4b66c36</t>
-        </is>
-      </c>
-      <c r="I468" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.588b5d3634416a6059a7318ba561bee1b3937a3a743aee7bdf6c94514c0aff0c.40b608332a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
-      <c r="M468" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N468" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O468" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P468" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q468" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R468" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S468" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T468" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
       <c r="W468" s="7" t="n"/>
     </row>
     <row r="469" ht="14.25" customHeight="1" s="50">
@@ -24056,192 +22376,12 @@
       <c r="W472" s="7" t="n"/>
     </row>
     <row r="473" ht="14.25" customHeight="1" s="50">
-      <c r="F473" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G473" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:12</t>
-        </is>
-      </c>
-      <c r="H473" t="inlineStr">
-        <is>
-          <t>e7b184d9004b721d45058522970f3cb8</t>
-        </is>
-      </c>
-      <c r="I473" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.c7cfc54dcfac0c48c09bb8cfef8f6d91bce2ddc0f8c56e438d3312b3358a249c.8538eae2a6^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
-      <c r="M473" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N473" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O473" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P473" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q473" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R473" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S473" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T473" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
       <c r="W473" s="7" t="n"/>
     </row>
     <row r="474" ht="14.25" customHeight="1" s="50">
-      <c r="F474" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G474" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:17:41</t>
-        </is>
-      </c>
-      <c r="H474" t="inlineStr">
-        <is>
-          <t>1e4947ef5f60b248f6cc587048c9f450</t>
-        </is>
-      </c>
-      <c r="I474" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.63396cbcbe3dfc78b5ad3904be91376e9f2d6731cb0763a0b5fd41cefd2a03f4.39eb44eb8d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
-      <c r="M474" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N474" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O474" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P474" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q474" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R474" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S474" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T474" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
       <c r="W474" s="7" t="n"/>
     </row>
     <row r="475" ht="14.25" customHeight="1" s="50">
-      <c r="F475" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G475" t="inlineStr">
-        <is>
-          <t>2026-03-26T08:16:46</t>
-        </is>
-      </c>
-      <c r="H475" t="inlineStr">
-        <is>
-          <t>3dcaffaa4a45aa93bcd389ef97304f18</t>
-        </is>
-      </c>
-      <c r="I475" t="inlineStr">
-        <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.0d71ec15820089182c6cafc0b3549797232f132d9d3d2fd9aa9f4d1a0aab5829.4ce80475d4^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-        </is>
-      </c>
-      <c r="M475" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N475" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O475" t="inlineStr">
-        <is>
-          <t>Errore segnalato dal gateway FSE</t>
-        </is>
-      </c>
-      <c r="P475" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q475" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R475" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S475" t="inlineStr">
-        <is>
-          <t>Errore loggato e mostrato all'operatore. Documento in coda retry automatica. Reinvio manuale disponibile.</t>
-        </is>
-      </c>
-      <c r="T475" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
       <c r="W475" s="7" t="n"/>
     </row>
     <row r="476" ht="14.25" customHeight="1" s="50">

</xml_diff>

<commit_message>
Fix: vendor info in column D (not E)
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#CENTROPOLISPECIALISTICOGIOVANNIPAOLOIXX/GPI_HEALTH_SYSTEM/FSE_SENDER/V.1.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#CENTROPOLISPECIALISTICOGIOVANNIPAOLOIXX/GPI_HEALTH_SYSTEM/FSE_SENDER/V.1.0/report-checklist.xlsx
@@ -2354,8 +2354,7 @@
       </c>
       <c r="B2" s="82" t="n"/>
       <c r="C2" s="83" t="n"/>
-      <c r="D2" s="82" t="n"/>
-      <c r="E2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>GPI Health System (Centro Polispecialistico Giovanni Paolo I srl)</t>
         </is>
@@ -2391,8 +2390,7 @@
           <t>subject_application_id:</t>
         </is>
       </c>
-      <c r="D3" s="82" t="n"/>
-      <c r="E3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>FSE_SENDER</t>
         </is>
@@ -2424,12 +2422,12 @@
           <t>subject_application_vendor:</t>
         </is>
       </c>
-      <c r="D4" s="82" t="n"/>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>GPI_HEALTH_SYSTEM</t>
         </is>
       </c>
+      <c r="E4" s="4" t="n"/>
       <c r="F4" s="6" t="n"/>
       <c r="G4" s="6" t="n"/>
       <c r="H4" s="6" t="n"/>
@@ -2457,8 +2455,7 @@
           <t>subject_application_version:</t>
         </is>
       </c>
-      <c r="D5" s="82" t="n"/>
-      <c r="E5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>V.1.0</t>
         </is>
@@ -23210,14 +23207,10 @@
     <row r="753" ht="14.25" customHeight="1" s="50"/>
   </sheetData>
   <autoFilter ref="A9:W245"/>
-  <mergeCells count="7">
+  <mergeCells count="3">
     <mergeCell ref="A3:B5"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C3:D3"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C4:D4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Fix report-checklist.xlsx: vendor in merged cells C2:D2-C5:D5 without split
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#CENTROPOLISPECIALISTICOGIOVANNIPAOLOIXX/GPI_HEALTH_SYSTEM/FSE_SENDER/V.1.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#CENTROPOLISPECIALISTICOGIOVANNIPAOLOIXX/GPI_HEALTH_SYSTEM/FSE_SENDER/V.1.0/report-checklist.xlsx
@@ -2353,12 +2353,12 @@
         </is>
       </c>
       <c r="B2" s="82" t="n"/>
-      <c r="C2" s="83" t="n"/>
-      <c r="D2" t="inlineStr">
+      <c r="C2" s="83" t="inlineStr">
         <is>
           <t>GPI Health System (Centro Polispecialistico Giovanni Paolo I srl)</t>
         </is>
       </c>
+      <c r="D2" s="82" t="n"/>
       <c r="F2" s="6" t="n"/>
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="n"/>
@@ -2387,14 +2387,10 @@
       <c r="B3" s="84" t="n"/>
       <c r="C3" s="85" t="inlineStr">
         <is>
-          <t>subject_application_id:</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>FSE_SENDER</t>
-        </is>
-      </c>
+          <t>subject_application_id: FSE_SENDER</t>
+        </is>
+      </c>
+      <c r="D3" s="82" t="n"/>
       <c r="F3" s="6" t="n"/>
       <c r="G3" s="6" t="n"/>
       <c r="H3" s="6" t="n"/>
@@ -2419,14 +2415,10 @@
       <c r="B4" s="87" t="n"/>
       <c r="C4" s="85" t="inlineStr">
         <is>
-          <t>subject_application_vendor:</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>GPI_HEALTH_SYSTEM</t>
-        </is>
-      </c>
+          <t>subject_application_vendor: GPI_HEALTH_SYSTEM</t>
+        </is>
+      </c>
+      <c r="D4" s="82" t="n"/>
       <c r="E4" s="4" t="n"/>
       <c r="F4" s="6" t="n"/>
       <c r="G4" s="6" t="n"/>
@@ -2452,14 +2444,10 @@
       <c r="B5" s="89" t="n"/>
       <c r="C5" s="85" t="inlineStr">
         <is>
-          <t>subject_application_version:</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>V.1.0</t>
-        </is>
-      </c>
+          <t>subject_application_version: V.1.0</t>
+        </is>
+      </c>
+      <c r="D5" s="82" t="n"/>
       <c r="F5" s="6" t="n"/>
       <c r="G5" s="6" t="n"/>
       <c r="H5" s="6" t="n"/>
@@ -23207,10 +23195,14 @@
     <row r="753" ht="14.25" customHeight="1" s="50"/>
   </sheetData>
   <autoFilter ref="A9:W245"/>
-  <mergeCells count="3">
+  <mergeCells count="7">
     <mergeCell ref="A3:B5"/>
     <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C3:D3"/>
     <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C4:D4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>

</xml_diff>